<commit_message>
Record initial firmware validation captures
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Refcb0663cb2546ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R8b5e6a0a9ac44515"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R5da6982126b54dc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rf978c51535d049a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R5003fed6878c4fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rce30aadeaf484193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R3bac7abd658041f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R1b8b51dee80249f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rbd5ac429478c49a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R20f7a65f504d4fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R0a0d90a8fb2f4bec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,13 +18,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="203" formatCode="0.000"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -56,8 +58,14 @@
       <x:sz val="13"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF49657A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,8 +122,38 @@
         <x:fgColor rgb="FFFFF7D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="11">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -183,11 +221,25 @@
         <x:color rgb="FFD4DEE7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD5E1EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD5E1EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD5E1EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5E1EA"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="88">
+  <x:cellXfs count="113">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -386,6 +438,59 @@
     <x:xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -588,7 +693,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5cf859b1f5aa4c7e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R54e7786f63a94e0b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -918,7 +1023,7 @@
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>카테고리</x:v>
@@ -963,7 +1068,7 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
@@ -987,14 +1092,14 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>IFERROR(B7/B6,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.17647058823529413</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
       <x:c r="E10" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F10" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
@@ -1002,7 +1107,7 @@
       </x:c>
       <x:c r="G10" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1011,7 +1116,7 @@
       </x:c>
       <x:c r="E11" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
@@ -1019,7 +1124,7 @@
       </x:c>
       <x:c r="G11" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1146,7 +1251,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb02b781f64b43db"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R095819a589a043c4"/>
 </x:worksheet>
 </file>
 
@@ -1421,7 +1526,7 @@
         <x:v>Hz</x:v>
       </x:c>
       <x:c r="F11" s="56" t="n">
-        <x:v>4000</x:v>
+        <x:v>1980</x:v>
       </x:c>
       <x:c r="G11" s="55" t="str">
         <x:v>최소</x:v>
@@ -1433,7 +1538,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="J11" s="55" t="str">
-        <x:v>허용오차 별도 정의</x:v>
+        <x:v>명목 2 kSPS; 합격 기준은 1,980 Hz 이상 (±1%)</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1529,7 +1634,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="J14" s="55" t="str">
-        <x:v>평균/최대 jitter 기록</x:v>
+        <x:v>명목 100 ms; 합격 범위는 평균 95–105 ms</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2139,8 +2244,12 @@
       <x:c r="A11" s="25" t="str">
         <x:v>T-01</x:v>
       </x:c>
-      <x:c r="B11" s="58"/>
-      <x:c r="C11" s="57"/>
+      <x:c r="B11" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C11" s="57" t="str">
+        <x:v>0062af0</x:v>
+      </x:c>
       <x:c r="D11" s="25" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
@@ -2154,37 +2263,53 @@
         <x:v>Hz</x:v>
       </x:c>
       <x:c r="H11" s="59" t="n">
-        <x:v>4000</x:v>
+        <x:v>1980</x:v>
       </x:c>
       <x:c r="I11" s="59" t="str">
         <x:v>최소</x:v>
       </x:c>
-      <x:c r="J11" s="60"/>
+      <x:c r="J11" s="60" t="n">
+        <x:v>1999.882</x:v>
+      </x:c>
       <x:c r="K11" s="60"/>
       <x:c r="L11" s="60"/>
-      <x:c r="M11" s="60"/>
+      <x:c r="M11" s="60" t="n">
+        <x:v>1999.882</x:v>
+      </x:c>
       <x:c r="N11" s="60"/>
-      <x:c r="O11" s="60"/>
-      <x:c r="P11" s="57"/>
+      <x:c r="O11" s="60" t="n">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="P11" s="57" t="str">
+        <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
+      </x:c>
       <x:c r="Q11" s="25" t="str">
-        <x:f>IF(OR(H11="",I11="",J11=""),"INPUT",IF(I11="최대",IF(J11&lt;=H11,"PASS","FAIL"),IF(I11="최소",IF(J11&gt;=H11,"PASS","FAIL"),IF(I11="일치",IF(J11=H11,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:f>IF(J11&gt;=H11,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R11" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S11" s="57"/>
+        <x:v>예비 통과</x:v>
+      </x:c>
+      <x:c r="S11" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T11" s="57" t="str">
-        <x:v>허용오차 별도 정의</x:v>
-      </x:c>
-      <x:c r="U11" s="57"/>
+        <x:v>50.7 s 최종 부팅 구간; PC 시간 대비 보드 시간 1:1</x:v>
+      </x:c>
+      <x:c r="U11" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_090258_671647.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="25" t="str">
         <x:v>T-02</x:v>
       </x:c>
-      <x:c r="B12" s="58"/>
-      <x:c r="C12" s="57"/>
+      <x:c r="B12" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C12" s="57" t="str">
+        <x:v>0062af0</x:v>
+      </x:c>
       <x:c r="D12" s="25" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
@@ -2203,25 +2328,43 @@
       <x:c r="I12" s="59" t="str">
         <x:v>일치</x:v>
       </x:c>
-      <x:c r="J12" s="60"/>
-      <x:c r="K12" s="60"/>
-      <x:c r="L12" s="60"/>
-      <x:c r="M12" s="60"/>
-      <x:c r="N12" s="60"/>
-      <x:c r="O12" s="60"/>
-      <x:c r="P12" s="57"/>
+      <x:c r="J12" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K12" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L12" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O12" s="60" t="n">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="P12" s="57" t="str">
+        <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
+      </x:c>
       <x:c r="Q12" s="25" t="str">
-        <x:f>IF(OR(H12="",I12="",J12=""),"INPUT",IF(I12="최대",IF(J12&lt;=H12,"PASS","FAIL"),IF(I12="최소",IF(J12&gt;=H12,"PASS","FAIL"),IF(I12="일치",IF(J12=H12,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:f>IF(J12=0,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R12" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S12" s="57"/>
+        <x:v>예비 통과</x:v>
+      </x:c>
+      <x:c r="S12" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T12" s="57" t="str">
-        <x:v>10분 부하 시험</x:v>
-      </x:c>
-      <x:c r="U12" s="57"/>
+        <x:v>DMA/Ring/Start/SPI error/DAC lock 모두 0; 10분 시험은 별도 수행</x:v>
+      </x:c>
+      <x:c r="U12" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_090258_671647.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="25" t="str">
@@ -2271,8 +2414,12 @@
       <x:c r="A14" s="25" t="str">
         <x:v>N-01</x:v>
       </x:c>
-      <x:c r="B14" s="58"/>
-      <x:c r="C14" s="57"/>
+      <x:c r="B14" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C14" s="57" t="str">
+        <x:v>0062af0</x:v>
+      </x:c>
       <x:c r="D14" s="25" t="str">
         <x:v>통신</x:v>
       </x:c>
@@ -2291,25 +2438,43 @@
       <x:c r="I14" s="59" t="str">
         <x:v>일치</x:v>
       </x:c>
-      <x:c r="J14" s="60"/>
-      <x:c r="K14" s="60"/>
-      <x:c r="L14" s="60"/>
-      <x:c r="M14" s="60"/>
-      <x:c r="N14" s="60"/>
-      <x:c r="O14" s="60"/>
-      <x:c r="P14" s="57"/>
+      <x:c r="J14" s="60" t="n">
+        <x:v>100.002</x:v>
+      </x:c>
+      <x:c r="K14" s="60" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="L14" s="60" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="M14" s="60" t="n">
+        <x:v>100.002</x:v>
+      </x:c>
+      <x:c r="N14" s="60" t="n">
+        <x:v>0.213</x:v>
+      </x:c>
+      <x:c r="O14" s="60" t="n">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="P14" s="57" t="str">
+        <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
+      </x:c>
       <x:c r="Q14" s="25" t="str">
-        <x:f>IF(OR(H14="",I14="",J14=""),"INPUT",IF(I14="최대",IF(J14&lt;=H14,"PASS","FAIL"),IF(I14="최소",IF(J14&gt;=H14,"PASS","FAIL"),IF(I14="일치",IF(J14=H14,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:f>IF(AND(J14&gt;=95,J14&lt;=105),"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R14" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S14" s="57"/>
+        <x:v>예비 통과</x:v>
+      </x:c>
+      <x:c r="S14" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T14" s="57" t="str">
-        <x:v>평균/최대 jitter 기록</x:v>
-      </x:c>
-      <x:c r="U14" s="57"/>
+        <x:v>최종 부팅 구간 50.7 s, 10.0 Hz; 1분 이상 시험은 별도 수행</x:v>
+      </x:c>
+      <x:c r="U14" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_090258_671647.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="25" t="str">
@@ -2758,7 +2923,7 @@
         <x:v>APP_ADC_RING_CAPACITY</x:v>
       </x:c>
       <x:c r="B9" s="61" t="n">
-        <x:v>128</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="C9" s="61" t="n">
         <x:v>256</x:v>
@@ -3145,7 +3310,7 @@
         <x:v>프레임 수 ÷ 경과시간, dropped, CRC/SPI 오류</x:v>
       </x:c>
       <x:c r="F17" s="87" t="str">
-        <x:v>4,000 Hz 이상</x:v>
+        <x:v>1,980 Hz 이상 (명목 2 kSPS, ±1%)</x:v>
       </x:c>
       <x:c r="G17" s="82" t="str">
         <x:v>텔레메트리는 100 ms이므로 ADC 원시율은 별도 계측 권장</x:v>
@@ -3223,7 +3388,7 @@
         <x:v>평균 주기·최대 jitter·수신 frame 수</x:v>
       </x:c>
       <x:c r="F20" s="87" t="str">
-        <x:v>100 ms 일치</x:v>
+        <x:v>평균 95–105 ms (명목 100 ms)</x:v>
       </x:c>
       <x:c r="G20" s="82" t="str">
         <x:v>PC의 순간 부하는 비고에 기록</x:v>
@@ -3400,4 +3565,398 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="39" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="35" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="50" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="91" t="str">
+        <x:v>CSV 캡처 이력 및 분석 결과</x:v>
+      </x:c>
+      <x:c r="B1" s="91"/>
+      <x:c r="C1" s="91"/>
+      <x:c r="D1" s="91"/>
+      <x:c r="E1" s="91"/>
+      <x:c r="F1" s="91"/>
+      <x:c r="G1" s="91"/>
+      <x:c r="H1" s="91"/>
+      <x:c r="I1" s="91"/>
+      <x:c r="J1" s="91"/>
+      <x:c r="K1" s="91"/>
+      <x:c r="L1" s="91"/>
+      <x:c r="M1" s="91"/>
+      <x:c r="N1" s="91"/>
+      <x:c r="O1" s="91"/>
+      <x:c r="P1" s="91"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="94" t="str">
+        <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
+      </x:c>
+      <x:c r="B3" s="94"/>
+      <x:c r="C3" s="94"/>
+      <x:c r="D3" s="94"/>
+      <x:c r="E3" s="94"/>
+      <x:c r="F3" s="94"/>
+      <x:c r="G3" s="94"/>
+      <x:c r="H3" s="94"/>
+      <x:c r="I3" s="94"/>
+      <x:c r="J3" s="94"/>
+      <x:c r="K3" s="94"/>
+      <x:c r="L3" s="94"/>
+      <x:c r="M3" s="94"/>
+      <x:c r="N3" s="94"/>
+      <x:c r="O3" s="94"/>
+      <x:c r="P3" s="94"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="97" t="str">
+        <x:v>CSV 파일</x:v>
+      </x:c>
+      <x:c r="B5" s="97" t="str">
+        <x:v>시험 목적</x:v>
+      </x:c>
+      <x:c r="C5" s="97" t="str">
+        <x:v>FW commit</x:v>
+      </x:c>
+      <x:c r="D5" s="97" t="str">
+        <x:v>부팅 구간</x:v>
+      </x:c>
+      <x:c r="E5" s="97" t="str">
+        <x:v>프레임</x:v>
+      </x:c>
+      <x:c r="F5" s="97" t="str">
+        <x:v>PC 시간 (s)</x:v>
+      </x:c>
+      <x:c r="G5" s="97" t="str">
+        <x:v>보드 시간 (s)</x:v>
+      </x:c>
+      <x:c r="H5" s="97" t="str">
+        <x:v>시간비</x:v>
+      </x:c>
+      <x:c r="I5" s="97" t="str">
+        <x:v>ADC rate (Hz)</x:v>
+      </x:c>
+      <x:c r="J5" s="97" t="str">
+        <x:v>UDP 평균 (ms)</x:v>
+      </x:c>
+      <x:c r="K5" s="97" t="str">
+        <x:v>UDP 범위 (ms)</x:v>
+      </x:c>
+      <x:c r="L5" s="97" t="str">
+        <x:v>드랍 최대</x:v>
+      </x:c>
+      <x:c r="M5" s="97" t="str">
+        <x:v>오류</x:v>
+      </x:c>
+      <x:c r="N5" s="97" t="str">
+        <x:v>입력/조건</x:v>
+      </x:c>
+      <x:c r="O5" s="97" t="str">
+        <x:v>판정</x:v>
+      </x:c>
+      <x:c r="P5" s="97" t="str">
+        <x:v>분석 메모</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="100" t="str">
+        <x:v>cosmoke_capture_20260820_082036_681100.csv</x:v>
+      </x:c>
+      <x:c r="B6" s="100" t="str">
+        <x:v>초기 ADC 안정성 기준선</x:v>
+      </x:c>
+      <x:c r="C6" s="100" t="str">
+        <x:v>pre-c1000cd</x:v>
+      </x:c>
+      <x:c r="D6" s="100" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="100" t="n">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="F6" s="105" t="n">
+        <x:v>49.573</x:v>
+      </x:c>
+      <x:c r="G6" s="105" t="n">
+        <x:v>38.535</x:v>
+      </x:c>
+      <x:c r="H6" s="105" t="n">
+        <x:v>0.777</x:v>
+      </x:c>
+      <x:c r="I6" s="105" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="J6" s="105" t="n">
+        <x:v>135.816</x:v>
+      </x:c>
+      <x:c r="K6" s="100" t="str">
+        <x:v>101–167</x:v>
+      </x:c>
+      <x:c r="L6" s="106" t="n">
+        <x:v>214883</x:v>
+      </x:c>
+      <x:c r="M6" s="100" t="str">
+        <x:v>CRC/SPI/DAC=0</x:v>
+      </x:c>
+      <x:c r="N6" s="100" t="str">
+        <x:v>CH1, 11 V / 5 A</x:v>
+      </x:c>
+      <x:c r="O6" s="102" t="str">
+        <x:v>FAIL</x:v>
+      </x:c>
+      <x:c r="P6" s="100" t="str">
+        <x:v>DMA-busy 드랍이 완료 프레임과 거의 1:1로 증가; 개선 전 기준선</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="100" t="str">
+        <x:v>cosmoke_capture_20260820_084802_667740.csv</x:v>
+      </x:c>
+      <x:c r="B7" s="100" t="str">
+        <x:v>11 V 입력 ON/OFF 3회</x:v>
+      </x:c>
+      <x:c r="C7" s="100" t="str">
+        <x:v>c1000cd</x:v>
+      </x:c>
+      <x:c r="D7" s="100" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="100" t="n">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="F7" s="105" t="n">
+        <x:v>102.878</x:v>
+      </x:c>
+      <x:c r="G7" s="105" t="n">
+        <x:v>45.145</x:v>
+      </x:c>
+      <x:c r="H7" s="105" t="n">
+        <x:v>0.439</x:v>
+      </x:c>
+      <x:c r="I7" s="105" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J7" s="105" t="n">
+        <x:v>230.15</x:v>
+      </x:c>
+      <x:c r="K7" s="100" t="str">
+        <x:v>229–242</x:v>
+      </x:c>
+      <x:c r="L7" s="106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="100" t="str">
+        <x:v>CRC/SPI/DAC=0</x:v>
+      </x:c>
+      <x:c r="N7" s="100" t="str">
+        <x:v>CH1, 11 V / 5 A</x:v>
+      </x:c>
+      <x:c r="O7" s="103" t="str">
+        <x:v>PASS (입력 응답)</x:v>
+      </x:c>
+      <x:c r="P7" s="100" t="str">
+        <x:v>ON 안정: 약 4.92–4.94 A / 10.951 V; OFF 안정: 약 12.6 mA / -21 mV. 시간축 수정 전</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="A8" s="100" t="str">
+        <x:v>cosmoke_capture_20260820_085948_533730.csv</x:v>
+      </x:c>
+      <x:c r="B8" s="100" t="str">
+        <x:v>TIM6 우선순위 수정 검증</x:v>
+      </x:c>
+      <x:c r="C8" s="100" t="str">
+        <x:v>0062af0</x:v>
+      </x:c>
+      <x:c r="D8" s="100" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" s="100" t="n">
+        <x:v>494</x:v>
+      </x:c>
+      <x:c r="F8" s="105" t="n">
+        <x:v>74.591</x:v>
+      </x:c>
+      <x:c r="G8" s="105"/>
+      <x:c r="H8" s="105"/>
+      <x:c r="I8" s="105" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J8" s="105" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K8" s="100" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="L8" s="106" t="n">
+        <x:v>39965</x:v>
+      </x:c>
+      <x:c r="M8" s="100" t="str">
+        <x:v>초기 1회 DMA drop</x:v>
+      </x:c>
+      <x:c r="N8" s="100" t="str">
+        <x:v>Reset 반복</x:v>
+      </x:c>
+      <x:c r="O8" s="104" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="P8" s="100" t="str">
+        <x:v>첫 부팅은 기존 드랍 이력 포함. 뒤 3회 부팅은 시간 1:1 및 드랍 0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="100" t="str">
+        <x:v>cosmoke_capture_20260820_090258_671647.csv</x:v>
+      </x:c>
+      <x:c r="B9" s="100" t="str">
+        <x:v>최종 시간축·ADC·UDP 확인</x:v>
+      </x:c>
+      <x:c r="C9" s="100" t="str">
+        <x:v>0062af0</x:v>
+      </x:c>
+      <x:c r="D9" s="100" t="str">
+        <x:v>2 (최종 2번째)</x:v>
+      </x:c>
+      <x:c r="E9" s="100" t="n">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="F9" s="105" t="n">
+        <x:v>50.701</x:v>
+      </x:c>
+      <x:c r="G9" s="105" t="n">
+        <x:v>50.699</x:v>
+      </x:c>
+      <x:c r="H9" s="105" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I9" s="105" t="n">
+        <x:v>1999.882</x:v>
+      </x:c>
+      <x:c r="J9" s="105" t="n">
+        <x:v>100.002</x:v>
+      </x:c>
+      <x:c r="K9" s="100" t="str">
+        <x:v>98–102</x:v>
+      </x:c>
+      <x:c r="L9" s="106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M9" s="100" t="str">
+        <x:v>CRC/SPI/DAC=0</x:v>
+      </x:c>
+      <x:c r="N9" s="100" t="str">
+        <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
+      </x:c>
+      <x:c r="O9" s="103" t="str">
+        <x:v>PASS (예비)</x:v>
+      </x:c>
+      <x:c r="P9" s="100" t="str">
+        <x:v>50.7 s 동안 10.0 Hz, 시간축 1:1, 모든 드랍 원인 0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="108" t="str">
+        <x:v>현재 검증된 펌웨어 프로파일</x:v>
+      </x:c>
+      <x:c r="B11" s="108"/>
+      <x:c r="C11" s="108"/>
+      <x:c r="D11" s="108"/>
+      <x:c r="E11" s="108"/>
+      <x:c r="F11" s="108"/>
+      <x:c r="G11" s="108"/>
+      <x:c r="H11" s="108"/>
+      <x:c r="I11" s="108"/>
+      <x:c r="J11" s="108"/>
+      <x:c r="K11" s="108"/>
+      <x:c r="L11" s="108"/>
+      <x:c r="M11" s="108"/>
+      <x:c r="N11" s="108"/>
+      <x:c r="O11" s="108"/>
+      <x:c r="P11" s="108"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="109" t="str">
+        <x:v>설정</x:v>
+      </x:c>
+      <x:c r="B12" s="109" t="str">
+        <x:v>현재값</x:v>
+      </x:c>
+      <x:c r="C12" s="109" t="str">
+        <x:v>근거</x:v>
+      </x:c>
+      <x:c r="D12" s="109" t="str">
+        <x:v>상태</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="110" t="str">
+        <x:v>ADC sample rate</x:v>
+      </x:c>
+      <x:c r="B13" s="110" t="str">
+        <x:v>2,000 Hz</x:v>
+      </x:c>
+      <x:c r="C13" s="110" t="str">
+        <x:v>최종 CSV: 1,999.882 Hz</x:v>
+      </x:c>
+      <x:c r="D13" s="112" t="str">
+        <x:v>검증됨</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="110" t="str">
+        <x:v>SPI1 clock</x:v>
+      </x:c>
+      <x:c r="B14" s="110" t="str">
+        <x:v>5.33 MHz</x:v>
+      </x:c>
+      <x:c r="C14" s="110" t="str">
+        <x:v>ADC DMA 전송 여유 확보</x:v>
+      </x:c>
+      <x:c r="D14" s="112" t="str">
+        <x:v>검증됨</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="110" t="str">
+        <x:v>TIM6 priority</x:v>
+      </x:c>
+      <x:c r="B15" s="110" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C15" s="110" t="str">
+        <x:v>PC/보드 시간 1:1</x:v>
+      </x:c>
+      <x:c r="D15" s="112" t="str">
+        <x:v>검증됨</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:P1"/>
+    <x:mergeCell ref="A3:P3"/>
+    <x:mergeCell ref="A11:P11"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record zero-input calibration results
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rce30aadeaf484193"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R3bac7abd658041f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R1b8b51dee80249f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rbd5ac429478c49a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R20f7a65f504d4fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R0a0d90a8fb2f4bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3bb4e9d9b2c345f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R2f5082d810b343f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R6a67e313337044d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rfd699b596f8140f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R4c54b1ecbe5a4aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R6aa0f94d95eb4fae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,12 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="203" formatCode="0.000"/>
     <x:numFmt numFmtId="204" formatCode="#,##0"/>
+    <x:numFmt numFmtId="205" formatCode="0.000000"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -65,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -120,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -239,7 +270,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="113">
+  <x:cellXfs count="127">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -491,6 +522,34 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="20" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -693,7 +752,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R54e7786f63a94e0b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd79283ba94794f0b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1023,7 +1082,7 @@
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"PASS")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>카테고리</x:v>
@@ -1068,14 +1127,14 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
       <x:c r="E9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
@@ -1083,7 +1142,7 @@
       </x:c>
       <x:c r="G9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1092,7 +1151,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>IFERROR(B7/B6,0)</x:f>
-        <x:v>0.17647058823529413</x:v>
+        <x:v>0.23529411764705882</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>시간 성능</x:v>
@@ -1251,7 +1310,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R095819a589a043c4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b5dac42a23f481e"/>
 </x:worksheet>
 </file>
 
@@ -2068,16 +2127,20 @@
       <x:c r="A7" s="25" t="str">
         <x:v>A-01</x:v>
       </x:c>
-      <x:c r="B7" s="58"/>
-      <x:c r="C7" s="57"/>
+      <x:c r="B7" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C7" s="57" t="str">
+        <x:v>4b7b1d3</x:v>
+      </x:c>
       <x:c r="D7" s="25" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
       <x:c r="E7" s="25" t="str">
-        <x:v>영점 오차</x:v>
+        <x:v>CH1·CH2 영점</x:v>
       </x:c>
       <x:c r="F7" s="25" t="str">
-        <x:v>0 입력 오차</x:v>
+        <x:v>0 입력 최대 오차</x:v>
       </x:c>
       <x:c r="G7" s="25" t="str">
         <x:v>%FS</x:v>
@@ -2088,25 +2151,43 @@
       <x:c r="I7" s="59" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J7" s="60"/>
-      <x:c r="K7" s="60"/>
-      <x:c r="L7" s="60"/>
-      <x:c r="M7" s="60"/>
-      <x:c r="N7" s="60"/>
-      <x:c r="O7" s="60"/>
-      <x:c r="P7" s="57"/>
+      <x:c r="J7" s="60" t="n">
+        <x:v>0.041553</x:v>
+      </x:c>
+      <x:c r="K7" s="60" t="n">
+        <x:v>0.004694</x:v>
+      </x:c>
+      <x:c r="L7" s="60" t="n">
+        <x:v>0.041553</x:v>
+      </x:c>
+      <x:c r="M7" s="60" t="n">
+        <x:v>0.023963</x:v>
+      </x:c>
+      <x:c r="N7" s="60" t="n">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="O7" s="60" t="n">
+        <x:v>3001</x:v>
+      </x:c>
+      <x:c r="P7" s="57" t="str">
+        <x:v>0 V / 0 A; CH1+CH2; final 5 min</x:v>
+      </x:c>
       <x:c r="Q7" s="25" t="str">
         <x:f>IF(OR(H7="",I7="",J7=""),"INPUT",IF(I7="최대",IF(J7&lt;=H7,"PASS","FAIL"),IF(I7="최소",IF(J7&gt;=H7,"PASS","FAIL"),IF(I7="일치",IF(J7=H7,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R7" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S7" s="57"/>
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="S7" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T7" s="57" t="str">
-        <x:v>채널별 기록</x:v>
-      </x:c>
-      <x:c r="U7" s="57"/>
+        <x:v>CH1 I +12.466 mA, V -11.734 mV; CH2 I +11.331 mA, V +29.593 mV. OFFSET_UNITS 적용.</x:v>
+      </x:c>
+      <x:c r="U7" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_091833_148511.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="25" t="str">
@@ -3574,9 +3655,9 @@
     <x:col min="1" max="1" width="39" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
@@ -3590,92 +3671,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="91" t="str">
+      <x:c r="A1" s="113" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="91"/>
-      <x:c r="C1" s="91"/>
-      <x:c r="D1" s="91"/>
-      <x:c r="E1" s="91"/>
-      <x:c r="F1" s="91"/>
-      <x:c r="G1" s="91"/>
-      <x:c r="H1" s="91"/>
-      <x:c r="I1" s="91"/>
-      <x:c r="J1" s="91"/>
-      <x:c r="K1" s="91"/>
-      <x:c r="L1" s="91"/>
-      <x:c r="M1" s="91"/>
-      <x:c r="N1" s="91"/>
-      <x:c r="O1" s="91"/>
-      <x:c r="P1" s="91"/>
+      <x:c r="B1" s="113"/>
+      <x:c r="C1" s="113"/>
+      <x:c r="D1" s="113"/>
+      <x:c r="E1" s="113"/>
+      <x:c r="F1" s="113"/>
+      <x:c r="G1" s="113"/>
+      <x:c r="H1" s="113"/>
+      <x:c r="I1" s="113"/>
+      <x:c r="J1" s="113"/>
+      <x:c r="K1" s="113"/>
+      <x:c r="L1" s="113"/>
+      <x:c r="M1" s="113"/>
+      <x:c r="N1" s="113"/>
+      <x:c r="O1" s="113"/>
+      <x:c r="P1" s="113"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="94" t="str">
+      <x:c r="A3" s="114" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="94"/>
-      <x:c r="C3" s="94"/>
-      <x:c r="D3" s="94"/>
-      <x:c r="E3" s="94"/>
-      <x:c r="F3" s="94"/>
-      <x:c r="G3" s="94"/>
-      <x:c r="H3" s="94"/>
-      <x:c r="I3" s="94"/>
-      <x:c r="J3" s="94"/>
-      <x:c r="K3" s="94"/>
-      <x:c r="L3" s="94"/>
-      <x:c r="M3" s="94"/>
-      <x:c r="N3" s="94"/>
-      <x:c r="O3" s="94"/>
-      <x:c r="P3" s="94"/>
+      <x:c r="B3" s="114"/>
+      <x:c r="C3" s="114"/>
+      <x:c r="D3" s="114"/>
+      <x:c r="E3" s="114"/>
+      <x:c r="F3" s="114"/>
+      <x:c r="G3" s="114"/>
+      <x:c r="H3" s="114"/>
+      <x:c r="I3" s="114"/>
+      <x:c r="J3" s="114"/>
+      <x:c r="K3" s="114"/>
+      <x:c r="L3" s="114"/>
+      <x:c r="M3" s="114"/>
+      <x:c r="N3" s="114"/>
+      <x:c r="O3" s="114"/>
+      <x:c r="P3" s="114"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="97" t="str">
+      <x:c r="A5" s="115" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="97" t="str">
+      <x:c r="B5" s="115" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="97" t="str">
+      <x:c r="C5" s="115" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="97" t="str">
+      <x:c r="D5" s="115" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="97" t="str">
+      <x:c r="E5" s="115" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="97" t="str">
+      <x:c r="F5" s="115" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="97" t="str">
+      <x:c r="G5" s="115" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="97" t="str">
+      <x:c r="H5" s="115" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="97" t="str">
+      <x:c r="I5" s="115" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="97" t="str">
+      <x:c r="J5" s="115" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="97" t="str">
+      <x:c r="K5" s="115" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="97" t="str">
+      <x:c r="L5" s="115" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="97" t="str">
+      <x:c r="M5" s="115" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="97" t="str">
+      <x:c r="N5" s="115" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="97" t="str">
+      <x:c r="O5" s="115" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="97" t="str">
+      <x:c r="P5" s="115" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -3722,7 +3803,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="102" t="str">
+      <x:c r="O6" s="117" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -3772,7 +3853,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="103" t="str">
+      <x:c r="O7" s="118" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -3818,7 +3899,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="104" t="str">
+      <x:c r="O8" s="119" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -3868,44 +3949,94 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="103" t="str">
+      <x:c r="O9" s="118" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
         <x:v>50.7 s 동안 10.0 Hz, 시간축 1:1, 모든 드랍 원인 0</x:v>
       </x:c>
     </x:row>
+    <x:row r="10" ht="48" customHeight="1">
+      <x:c r="A10" s="100" t="str">
+        <x:v>cosmoke_capture_20260820_091833_148511.csv</x:v>
+      </x:c>
+      <x:c r="B10" s="100" t="str">
+        <x:v>CH1·CH2 0 입력 오프셋</x:v>
+      </x:c>
+      <x:c r="C10" s="100" t="str">
+        <x:v>4b7b1d3</x:v>
+      </x:c>
+      <x:c r="D10" s="100" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="100" t="n">
+        <x:v>4551</x:v>
+      </x:c>
+      <x:c r="F10" s="105" t="n">
+        <x:v>454.995</x:v>
+      </x:c>
+      <x:c r="G10" s="105" t="n">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="H10" s="105" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I10" s="105" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J10" s="105" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K10" s="100" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="L10" s="106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="100" t="str">
+        <x:v>CRC/SPI/DAC=0</x:v>
+      </x:c>
+      <x:c r="N10" s="100" t="str">
+        <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
+      </x:c>
+      <x:c r="O10" s="118" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="P10" s="100" t="str">
+        <x:v>보정 전 평균: I1 +12.466 mA, V1 -11.734 mV, I2 +11.331 mA, V2 +29.593 mV; OFFSET_UNITS 적용</x:v>
+      </x:c>
+    </x:row>
     <x:row r="11">
-      <x:c r="A11" s="108" t="str">
+      <x:c r="A11" s="120" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="108"/>
-      <x:c r="C11" s="108"/>
-      <x:c r="D11" s="108"/>
-      <x:c r="E11" s="108"/>
-      <x:c r="F11" s="108"/>
-      <x:c r="G11" s="108"/>
-      <x:c r="H11" s="108"/>
-      <x:c r="I11" s="108"/>
-      <x:c r="J11" s="108"/>
-      <x:c r="K11" s="108"/>
-      <x:c r="L11" s="108"/>
-      <x:c r="M11" s="108"/>
-      <x:c r="N11" s="108"/>
-      <x:c r="O11" s="108"/>
-      <x:c r="P11" s="108"/>
+      <x:c r="B11" s="120"/>
+      <x:c r="C11" s="120"/>
+      <x:c r="D11" s="120"/>
+      <x:c r="E11" s="120"/>
+      <x:c r="F11" s="120"/>
+      <x:c r="G11" s="120"/>
+      <x:c r="H11" s="120"/>
+      <x:c r="I11" s="120"/>
+      <x:c r="J11" s="120"/>
+      <x:c r="K11" s="120"/>
+      <x:c r="L11" s="120"/>
+      <x:c r="M11" s="120"/>
+      <x:c r="N11" s="120"/>
+      <x:c r="O11" s="120"/>
+      <x:c r="P11" s="120"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="109" t="str">
+      <x:c r="A12" s="121" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="109" t="str">
+      <x:c r="B12" s="121" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="109" t="str">
+      <x:c r="C12" s="121" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="109" t="str">
+      <x:c r="D12" s="121" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -3919,7 +4050,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="112" t="str">
+      <x:c r="D13" s="122" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -3933,7 +4064,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="112" t="str">
+      <x:c r="D14" s="122" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -3947,8 +4078,128 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="112" t="str">
+      <x:c r="D15" s="122" t="str">
         <x:v>검증됨</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="120" t="str">
+        <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
+      </x:c>
+      <x:c r="B17" s="120"/>
+      <x:c r="C17" s="120"/>
+      <x:c r="D17" s="120"/>
+      <x:c r="E17" s="120"/>
+      <x:c r="F17" s="120"/>
+      <x:c r="G17" s="120"/>
+      <x:c r="H17" s="120"/>
+      <x:c r="I17" s="120"/>
+      <x:c r="J17" s="120"/>
+      <x:c r="K17" s="120"/>
+      <x:c r="L17" s="120"/>
+      <x:c r="M17" s="120"/>
+      <x:c r="N17" s="120"/>
+      <x:c r="O17" s="120"/>
+      <x:c r="P17" s="120"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="121" t="str">
+        <x:v>채널</x:v>
+      </x:c>
+      <x:c r="B18" s="121" t="str">
+        <x:v>측정 평균</x:v>
+      </x:c>
+      <x:c r="C18" s="121" t="str">
+        <x:v>단위</x:v>
+      </x:c>
+      <x:c r="D18" s="121" t="str">
+        <x:v>펌웨어 매크로</x:v>
+      </x:c>
+      <x:c r="E18" s="121" t="str">
+        <x:v>적용 OFFSET_UNITS</x:v>
+      </x:c>
+      <x:c r="F18" s="121" t="str">
+        <x:v>CSV</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="110" t="str">
+        <x:v>CH1 Current</x:v>
+      </x:c>
+      <x:c r="B19" s="110" t="n">
+        <x:v>12.466</x:v>
+      </x:c>
+      <x:c r="C19" s="110" t="str">
+        <x:v>mA</x:v>
+      </x:c>
+      <x:c r="D19" s="110" t="str">
+        <x:v>APP_CH0_OFFSET_UNITS</x:v>
+      </x:c>
+      <x:c r="E19" s="126" t="n">
+        <x:v>-0.012466</x:v>
+      </x:c>
+      <x:c r="F19" s="110" t="str">
+        <x:v>091833_148511</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="110" t="str">
+        <x:v>CH1 Voltage</x:v>
+      </x:c>
+      <x:c r="B20" s="110" t="n">
+        <x:v>-11.734</x:v>
+      </x:c>
+      <x:c r="C20" s="110" t="str">
+        <x:v>mV</x:v>
+      </x:c>
+      <x:c r="D20" s="110" t="str">
+        <x:v>APP_CH1_OFFSET_UNITS</x:v>
+      </x:c>
+      <x:c r="E20" s="126" t="n">
+        <x:v>0.011734</x:v>
+      </x:c>
+      <x:c r="F20" s="110" t="str">
+        <x:v>091833_148511</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="110" t="str">
+        <x:v>CH2 Current</x:v>
+      </x:c>
+      <x:c r="B21" s="110" t="n">
+        <x:v>11.331</x:v>
+      </x:c>
+      <x:c r="C21" s="110" t="str">
+        <x:v>mA</x:v>
+      </x:c>
+      <x:c r="D21" s="110" t="str">
+        <x:v>APP_CH2_OFFSET_UNITS</x:v>
+      </x:c>
+      <x:c r="E21" s="126" t="n">
+        <x:v>-0.011331</x:v>
+      </x:c>
+      <x:c r="F21" s="110" t="str">
+        <x:v>091833_148511</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="110" t="str">
+        <x:v>CH2 Voltage</x:v>
+      </x:c>
+      <x:c r="B22" s="110" t="n">
+        <x:v>29.593</x:v>
+      </x:c>
+      <x:c r="C22" s="110" t="str">
+        <x:v>mV</x:v>
+      </x:c>
+      <x:c r="D22" s="110" t="str">
+        <x:v>APP_CH3_OFFSET_UNITS</x:v>
+      </x:c>
+      <x:c r="E22" s="126" t="n">
+        <x:v>-0.029593</x:v>
+      </x:c>
+      <x:c r="F22" s="110" t="str">
+        <x:v>091833_148511</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3956,6 +4207,7 @@
     <x:mergeCell ref="A1:P1"/>
     <x:mergeCell ref="A3:P3"/>
     <x:mergeCell ref="A11:P11"/>
+    <x:mergeCell ref="A17:P17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Record dual-channel load test and gain baseline
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3bb4e9d9b2c345f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R2f5082d810b343f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R6a67e313337044d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rfd699b596f8140f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R4c54b1ecbe5a4aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R6aa0f94d95eb4fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc967a9e506aa4eb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="Rece0d41565084d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="Rd3b79eb73da545ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R51fe58057fcb412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R88cb1ef9e88b45ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R0fed46371b8b4a62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -270,7 +300,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="127">
+  <x:cellXfs count="141">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -550,6 +580,36 @@
     <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="205" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="26" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="27" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="27" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -752,7 +812,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd79283ba94794f0b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5478fea5b1f4b05"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1103,7 +1163,7 @@
       </x:c>
       <x:c r="B8" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"FAIL")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
         <x:v>기능</x:v>
@@ -1127,7 +1187,7 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
@@ -1138,11 +1198,11 @@
       </x:c>
       <x:c r="F9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1310,7 +1370,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b5dac42a23f481e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8031251bcce0468f"/>
 </x:worksheet>
 </file>
 
@@ -2193,16 +2253,20 @@
       <x:c r="A8" s="25" t="str">
         <x:v>A-02</x:v>
       </x:c>
-      <x:c r="B8" s="58"/>
-      <x:c r="C8" s="57"/>
+      <x:c r="B8" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C8" s="57" t="str">
+        <x:v>4b7b1d3 (pre-gain)</x:v>
+      </x:c>
       <x:c r="D8" s="25" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
       <x:c r="E8" s="25" t="str">
-        <x:v>gain 오차</x:v>
+        <x:v>CH1·CH2 gain</x:v>
       </x:c>
       <x:c r="F8" s="25" t="str">
-        <x:v>100% span 오차</x:v>
+        <x:v>100% span 최대 오차</x:v>
       </x:c>
       <x:c r="G8" s="25" t="str">
         <x:v>%FS</x:v>
@@ -2213,25 +2277,43 @@
       <x:c r="I8" s="59" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J8" s="60"/>
-      <x:c r="K8" s="60"/>
-      <x:c r="L8" s="60"/>
-      <x:c r="M8" s="60"/>
-      <x:c r="N8" s="60"/>
-      <x:c r="O8" s="60"/>
-      <x:c r="P8" s="57"/>
+      <x:c r="J8" s="60" t="n">
+        <x:v>10.4435</x:v>
+      </x:c>
+      <x:c r="K8" s="60" t="n">
+        <x:v>3.3202</x:v>
+      </x:c>
+      <x:c r="L8" s="60" t="n">
+        <x:v>10.4435</x:v>
+      </x:c>
+      <x:c r="M8" s="60" t="n">
+        <x:v>7.3837</x:v>
+      </x:c>
+      <x:c r="N8" s="60" t="n">
+        <x:v>3.195</x:v>
+      </x:c>
+      <x:c r="O8" s="60" t="n">
+        <x:v>16577</x:v>
+      </x:c>
+      <x:c r="P8" s="57" t="str">
+        <x:v>11 V / 5 A; CH1+CH2; user-induced input interruption excluded</x:v>
+      </x:c>
       <x:c r="Q8" s="25" t="str">
         <x:f>IF(OR(H8="",I8="",J8=""),"INPUT",IF(I8="최대",IF(J8&lt;=H8,"PASS","FAIL"),IF(I8="최소",IF(J8&gt;=H8,"PASS","FAIL"),IF(I8="일치",IF(J8=H8,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="R8" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S8" s="57"/>
+        <x:v>보정 후 재검증 필요</x:v>
+      </x:c>
+      <x:c r="S8" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T8" s="57" t="str">
-        <x:v>보정 전/후 비교</x:v>
-      </x:c>
-      <x:c r="U8" s="57"/>
+        <x:v>보정 전: I1 +5.97%, V1 +9.80%, I2 +3.32%, V2 +10.44%. SCALE_TRIM은 f9ceb9a에 적용.</x:v>
+      </x:c>
+      <x:c r="U8" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="25" t="str">
@@ -2329,7 +2411,7 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="C11" s="57" t="str">
-        <x:v>0062af0</x:v>
+        <x:v>4b7b1d3</x:v>
       </x:c>
       <x:c r="D11" s="25" t="str">
         <x:v>시간 성능</x:v>
@@ -2350,35 +2432,35 @@
         <x:v>최소</x:v>
       </x:c>
       <x:c r="J11" s="60" t="n">
-        <x:v>1999.882</x:v>
+        <x:v>1999.931</x:v>
       </x:c>
       <x:c r="K11" s="60"/>
       <x:c r="L11" s="60"/>
       <x:c r="M11" s="60" t="n">
-        <x:v>1999.882</x:v>
+        <x:v>1999.931</x:v>
       </x:c>
       <x:c r="N11" s="60"/>
       <x:c r="O11" s="60" t="n">
-        <x:v>508</x:v>
+        <x:v>16621</x:v>
       </x:c>
       <x:c r="P11" s="57" t="str">
-        <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
+        <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
       <x:c r="Q11" s="25" t="str">
         <x:f>IF(J11&gt;=H11,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="R11" s="57" t="str">
-        <x:v>예비 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="S11" s="57" t="str">
         <x:v>지명환</x:v>
       </x:c>
       <x:c r="T11" s="57" t="str">
-        <x:v>50.7 s 최종 부팅 구간; PC 시간 대비 보드 시간 1:1</x:v>
+        <x:v>PC/보드 시간 1:1, ADC 1,999.931 Hz</x:v>
       </x:c>
       <x:c r="U11" s="57" t="str">
-        <x:v>logs/cosmoke_capture_20260820_090258_671647.csv</x:v>
+        <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2389,7 +2471,7 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="C12" s="57" t="str">
-        <x:v>0062af0</x:v>
+        <x:v>4b7b1d3</x:v>
       </x:c>
       <x:c r="D12" s="25" t="str">
         <x:v>시간 성능</x:v>
@@ -2425,26 +2507,26 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O12" s="60" t="n">
-        <x:v>508</x:v>
+        <x:v>16621</x:v>
       </x:c>
       <x:c r="P12" s="57" t="str">
-        <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
+        <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
       <x:c r="Q12" s="25" t="str">
         <x:f>IF(J12=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="R12" s="57" t="str">
-        <x:v>예비 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="S12" s="57" t="str">
         <x:v>지명환</x:v>
       </x:c>
       <x:c r="T12" s="57" t="str">
-        <x:v>DMA/Ring/Start/SPI error/DAC lock 모두 0; 10분 시험은 별도 수행</x:v>
+        <x:v>27.7 min 동안 모든 드롭 원인 0</x:v>
       </x:c>
       <x:c r="U12" s="57" t="str">
-        <x:v>logs/cosmoke_capture_20260820_090258_671647.csv</x:v>
+        <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2499,7 +2581,7 @@
         <x:v>46254</x:v>
       </x:c>
       <x:c r="C14" s="57" t="str">
-        <x:v>0062af0</x:v>
+        <x:v>4b7b1d3</x:v>
       </x:c>
       <x:c r="D14" s="25" t="str">
         <x:v>통신</x:v>
@@ -2520,41 +2602,41 @@
         <x:v>일치</x:v>
       </x:c>
       <x:c r="J14" s="60" t="n">
-        <x:v>100.002</x:v>
+        <x:v>99.999</x:v>
       </x:c>
       <x:c r="K14" s="60" t="n">
-        <x:v>98</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L14" s="60" t="n">
-        <x:v>102</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="M14" s="60" t="n">
-        <x:v>100.002</x:v>
+        <x:v>99.999</x:v>
       </x:c>
       <x:c r="N14" s="60" t="n">
-        <x:v>0.213</x:v>
+        <x:v>1.264</x:v>
       </x:c>
       <x:c r="O14" s="60" t="n">
-        <x:v>508</x:v>
+        <x:v>16620</x:v>
       </x:c>
       <x:c r="P14" s="57" t="str">
-        <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
+        <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
       <x:c r="Q14" s="25" t="str">
         <x:f>IF(AND(J14&gt;=95,J14&lt;=105),"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="R14" s="57" t="str">
-        <x:v>예비 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="S14" s="57" t="str">
         <x:v>지명환</x:v>
       </x:c>
       <x:c r="T14" s="57" t="str">
-        <x:v>최종 부팅 구간 50.7 s, 10.0 Hz; 1분 이상 시험은 별도 수행</x:v>
+        <x:v>평균 99.999 ms; PC 수신 타임스탬프 최대 gap 218 ms</x:v>
       </x:c>
       <x:c r="U14" s="57" t="str">
-        <x:v>logs/cosmoke_capture_20260820_090258_671647.csv</x:v>
+        <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -3671,92 +3753,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="113" t="str">
+      <x:c r="A1" s="127" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="113"/>
-      <x:c r="C1" s="113"/>
-      <x:c r="D1" s="113"/>
-      <x:c r="E1" s="113"/>
-      <x:c r="F1" s="113"/>
-      <x:c r="G1" s="113"/>
-      <x:c r="H1" s="113"/>
-      <x:c r="I1" s="113"/>
-      <x:c r="J1" s="113"/>
-      <x:c r="K1" s="113"/>
-      <x:c r="L1" s="113"/>
-      <x:c r="M1" s="113"/>
-      <x:c r="N1" s="113"/>
-      <x:c r="O1" s="113"/>
-      <x:c r="P1" s="113"/>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+      <x:c r="E1" s="127"/>
+      <x:c r="F1" s="127"/>
+      <x:c r="G1" s="127"/>
+      <x:c r="H1" s="127"/>
+      <x:c r="I1" s="127"/>
+      <x:c r="J1" s="127"/>
+      <x:c r="K1" s="127"/>
+      <x:c r="L1" s="127"/>
+      <x:c r="M1" s="127"/>
+      <x:c r="N1" s="127"/>
+      <x:c r="O1" s="127"/>
+      <x:c r="P1" s="127"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="114" t="str">
+      <x:c r="A3" s="128" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="114"/>
-      <x:c r="C3" s="114"/>
-      <x:c r="D3" s="114"/>
-      <x:c r="E3" s="114"/>
-      <x:c r="F3" s="114"/>
-      <x:c r="G3" s="114"/>
-      <x:c r="H3" s="114"/>
-      <x:c r="I3" s="114"/>
-      <x:c r="J3" s="114"/>
-      <x:c r="K3" s="114"/>
-      <x:c r="L3" s="114"/>
-      <x:c r="M3" s="114"/>
-      <x:c r="N3" s="114"/>
-      <x:c r="O3" s="114"/>
-      <x:c r="P3" s="114"/>
+      <x:c r="B3" s="128"/>
+      <x:c r="C3" s="128"/>
+      <x:c r="D3" s="128"/>
+      <x:c r="E3" s="128"/>
+      <x:c r="F3" s="128"/>
+      <x:c r="G3" s="128"/>
+      <x:c r="H3" s="128"/>
+      <x:c r="I3" s="128"/>
+      <x:c r="J3" s="128"/>
+      <x:c r="K3" s="128"/>
+      <x:c r="L3" s="128"/>
+      <x:c r="M3" s="128"/>
+      <x:c r="N3" s="128"/>
+      <x:c r="O3" s="128"/>
+      <x:c r="P3" s="128"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="115" t="str">
+      <x:c r="A5" s="129" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="115" t="str">
+      <x:c r="B5" s="129" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="115" t="str">
+      <x:c r="C5" s="129" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="115" t="str">
+      <x:c r="D5" s="129" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="115" t="str">
+      <x:c r="E5" s="129" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="115" t="str">
+      <x:c r="F5" s="129" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="115" t="str">
+      <x:c r="G5" s="129" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="115" t="str">
+      <x:c r="H5" s="129" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="115" t="str">
+      <x:c r="I5" s="129" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="115" t="str">
+      <x:c r="J5" s="129" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="115" t="str">
+      <x:c r="K5" s="129" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="115" t="str">
+      <x:c r="L5" s="129" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="115" t="str">
+      <x:c r="M5" s="129" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="115" t="str">
+      <x:c r="N5" s="129" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="115" t="str">
+      <x:c r="O5" s="129" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="115" t="str">
+      <x:c r="P5" s="129" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -3803,7 +3885,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="117" t="str">
+      <x:c r="O6" s="130" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -3853,7 +3935,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="118" t="str">
+      <x:c r="O7" s="131" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -3899,7 +3981,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="119" t="str">
+      <x:c r="O8" s="132" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -3949,7 +4031,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="118" t="str">
+      <x:c r="O9" s="131" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -3999,7 +4081,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="118" t="str">
+      <x:c r="O10" s="131" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4007,36 +4089,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="120" t="str">
+      <x:c r="A11" s="133" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="120"/>
-      <x:c r="C11" s="120"/>
-      <x:c r="D11" s="120"/>
-      <x:c r="E11" s="120"/>
-      <x:c r="F11" s="120"/>
-      <x:c r="G11" s="120"/>
-      <x:c r="H11" s="120"/>
-      <x:c r="I11" s="120"/>
-      <x:c r="J11" s="120"/>
-      <x:c r="K11" s="120"/>
-      <x:c r="L11" s="120"/>
-      <x:c r="M11" s="120"/>
-      <x:c r="N11" s="120"/>
-      <x:c r="O11" s="120"/>
-      <x:c r="P11" s="120"/>
+      <x:c r="B11" s="133"/>
+      <x:c r="C11" s="133"/>
+      <x:c r="D11" s="133"/>
+      <x:c r="E11" s="133"/>
+      <x:c r="F11" s="133"/>
+      <x:c r="G11" s="133"/>
+      <x:c r="H11" s="133"/>
+      <x:c r="I11" s="133"/>
+      <x:c r="J11" s="133"/>
+      <x:c r="K11" s="133"/>
+      <x:c r="L11" s="133"/>
+      <x:c r="M11" s="133"/>
+      <x:c r="N11" s="133"/>
+      <x:c r="O11" s="133"/>
+      <x:c r="P11" s="133"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="121" t="str">
+      <x:c r="A12" s="134" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="121" t="str">
+      <x:c r="B12" s="134" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="121" t="str">
+      <x:c r="C12" s="134" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="121" t="str">
+      <x:c r="D12" s="134" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4050,7 +4132,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="122" t="str">
+      <x:c r="D13" s="135" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4064,7 +4146,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="122" t="str">
+      <x:c r="D14" s="135" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4078,47 +4160,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="122" t="str">
+      <x:c r="D15" s="135" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="120" t="str">
+      <x:c r="A17" s="133" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="120"/>
-      <x:c r="C17" s="120"/>
-      <x:c r="D17" s="120"/>
-      <x:c r="E17" s="120"/>
-      <x:c r="F17" s="120"/>
-      <x:c r="G17" s="120"/>
-      <x:c r="H17" s="120"/>
-      <x:c r="I17" s="120"/>
-      <x:c r="J17" s="120"/>
-      <x:c r="K17" s="120"/>
-      <x:c r="L17" s="120"/>
-      <x:c r="M17" s="120"/>
-      <x:c r="N17" s="120"/>
-      <x:c r="O17" s="120"/>
-      <x:c r="P17" s="120"/>
+      <x:c r="B17" s="133"/>
+      <x:c r="C17" s="133"/>
+      <x:c r="D17" s="133"/>
+      <x:c r="E17" s="133"/>
+      <x:c r="F17" s="133"/>
+      <x:c r="G17" s="133"/>
+      <x:c r="H17" s="133"/>
+      <x:c r="I17" s="133"/>
+      <x:c r="J17" s="133"/>
+      <x:c r="K17" s="133"/>
+      <x:c r="L17" s="133"/>
+      <x:c r="M17" s="133"/>
+      <x:c r="N17" s="133"/>
+      <x:c r="O17" s="133"/>
+      <x:c r="P17" s="133"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="121" t="str">
+      <x:c r="A18" s="134" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="121" t="str">
+      <x:c r="B18" s="134" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="121" t="str">
+      <x:c r="C18" s="134" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="121" t="str">
+      <x:c r="D18" s="134" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="121" t="str">
+      <x:c r="E18" s="134" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="121" t="str">
+      <x:c r="F18" s="134" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4200,6 +4282,126 @@
       </x:c>
       <x:c r="F22" s="110" t="str">
         <x:v>091833_148511</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="133" t="str">
+        <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
+      </x:c>
+      <x:c r="B24" s="133"/>
+      <x:c r="C24" s="133"/>
+      <x:c r="D24" s="133"/>
+      <x:c r="E24" s="133"/>
+      <x:c r="F24" s="133"/>
+      <x:c r="G24" s="133"/>
+      <x:c r="H24" s="133"/>
+      <x:c r="I24" s="133"/>
+      <x:c r="J24" s="133"/>
+      <x:c r="K24" s="133"/>
+      <x:c r="L24" s="133"/>
+      <x:c r="M24" s="133"/>
+      <x:c r="N24" s="133"/>
+      <x:c r="O24" s="133"/>
+      <x:c r="P24" s="133"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="129" t="str">
+        <x:v>CSV 파일</x:v>
+      </x:c>
+      <x:c r="B25" s="129" t="str">
+        <x:v>시험 목적</x:v>
+      </x:c>
+      <x:c r="C25" s="129" t="str">
+        <x:v>FW commit</x:v>
+      </x:c>
+      <x:c r="D25" s="129" t="str">
+        <x:v>부팅 구간</x:v>
+      </x:c>
+      <x:c r="E25" s="129" t="str">
+        <x:v>프레임</x:v>
+      </x:c>
+      <x:c r="F25" s="129" t="str">
+        <x:v>PC 시간 (s)</x:v>
+      </x:c>
+      <x:c r="G25" s="129" t="str">
+        <x:v>보드 시간 (s)</x:v>
+      </x:c>
+      <x:c r="H25" s="129" t="str">
+        <x:v>시간비</x:v>
+      </x:c>
+      <x:c r="I25" s="129" t="str">
+        <x:v>ADC rate (Hz)</x:v>
+      </x:c>
+      <x:c r="J25" s="129" t="str">
+        <x:v>UDP 평균 (ms)</x:v>
+      </x:c>
+      <x:c r="K25" s="129" t="str">
+        <x:v>UDP 범위 (ms)</x:v>
+      </x:c>
+      <x:c r="L25" s="129" t="str">
+        <x:v>드랍 최대</x:v>
+      </x:c>
+      <x:c r="M25" s="129" t="str">
+        <x:v>오류</x:v>
+      </x:c>
+      <x:c r="N25" s="129" t="str">
+        <x:v>입력/조건</x:v>
+      </x:c>
+      <x:c r="O25" s="129" t="str">
+        <x:v>판정</x:v>
+      </x:c>
+      <x:c r="P25" s="129" t="str">
+        <x:v>분석 메모</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="52" customHeight="1">
+      <x:c r="A26" s="100" t="str">
+        <x:v>cosmoke_capture_20260820_094031_980220.csv</x:v>
+      </x:c>
+      <x:c r="B26" s="100" t="str">
+        <x:v>양 채널 11 V / 5 A 27.7분</x:v>
+      </x:c>
+      <x:c r="C26" s="100" t="str">
+        <x:v>4b7b1d3 (pre-gain)</x:v>
+      </x:c>
+      <x:c r="D26" s="100" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="100" t="n">
+        <x:v>16621</x:v>
+      </x:c>
+      <x:c r="F26" s="105" t="n">
+        <x:v>1661.982</x:v>
+      </x:c>
+      <x:c r="G26" s="105" t="n">
+        <x:v>1662</x:v>
+      </x:c>
+      <x:c r="H26" s="105" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I26" s="105" t="n">
+        <x:v>1999.931</x:v>
+      </x:c>
+      <x:c r="J26" s="105" t="n">
+        <x:v>99.999</x:v>
+      </x:c>
+      <x:c r="K26" s="100" t="str">
+        <x:v>0–218</x:v>
+      </x:c>
+      <x:c r="L26" s="106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M26" s="100" t="str">
+        <x:v>CRC/SPI/DAC=0</x:v>
+      </x:c>
+      <x:c r="N26" s="100" t="str">
+        <x:v>CH1+CH2 11 V / 5 A</x:v>
+      </x:c>
+      <x:c r="O26" s="131" t="str">
+        <x:v>PASS (안정성)</x:v>
+      </x:c>
+      <x:c r="P26" s="100" t="str">
+        <x:v>0 입력 구간 44프레임 제외. 게인 오차: I1 +5.97%, V1 +9.80%, I2 +3.32%, V2 +10.44%; SCALE_TRIM 적용 후 재시험 필요</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4208,6 +4410,7 @@
     <x:mergeCell ref="A3:P3"/>
     <x:mergeCell ref="A11:P11"/>
     <x:mergeCell ref="A17:P17"/>
+    <x:mergeCell ref="A24:P24"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Defer gain verification to field validation
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc967a9e506aa4eb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="Rece0d41565084d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="Rd3b79eb73da545ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R51fe58057fcb412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R88cb1ef9e88b45ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R0fed46371b8b4a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rca8f6eb0b04746fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="Rbdd0ebe7fe4441e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R8f98fd57ba7c4f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R3a70050716ea4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Rf889eea625ef4de5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R71ad1e9752e34edb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="30">
+  <x:fills count="36">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -300,7 +330,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="141">
+  <x:cellXfs count="150">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -610,6 +640,27 @@
     <x:xf numFmtId="0" fontId="0" fillId="27" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="32" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -812,7 +863,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5478fea5b1f4b05"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5623979d32dc4911"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1163,7 +1214,7 @@
       </x:c>
       <x:c r="B8" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"FAIL")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
         <x:v>기능</x:v>
@@ -1198,7 +1249,7 @@
       </x:c>
       <x:c r="F9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
@@ -1370,7 +1421,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8031251bcce0468f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99b796713ae64afe"/>
 </x:worksheet>
 </file>
 
@@ -2299,17 +2350,17 @@
         <x:v>11 V / 5 A; CH1+CH2; user-induced input interruption excluded</x:v>
       </x:c>
       <x:c r="Q8" s="25" t="str">
-        <x:f>IF(OR(H8="",I8="",J8=""),"INPUT",IF(I8="최대",IF(J8&lt;=H8,"PASS","FAIL"),IF(I8="최소",IF(J8&gt;=H8,"PASS","FAIL"),IF(I8="일치",IF(J8=H8,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>FAIL</x:v>
+        <x:f>"FIELD"</x:f>
+        <x:v>FIELD</x:v>
       </x:c>
       <x:c r="R8" s="57" t="str">
-        <x:v>보정 후 재검증 필요</x:v>
+        <x:v>현장 검증 이관</x:v>
       </x:c>
       <x:c r="S8" s="57" t="str">
         <x:v>지명환</x:v>
       </x:c>
       <x:c r="T8" s="57" t="str">
-        <x:v>보정 전: I1 +5.97%, V1 +9.80%, I2 +3.32%, V2 +10.44%. SCALE_TRIM은 f9ceb9a에 적용.</x:v>
+        <x:v>벤치 합격 판정에서는 제외. 보정 전 데이터와 SCALE_TRIM 적용 이력은 보존하며 실제 운용 환경에서 검증.</x:v>
       </x:c>
       <x:c r="U8" s="57" t="str">
         <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
@@ -3753,92 +3804,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="127" t="str">
+      <x:c r="A1" s="141" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="127"/>
-      <x:c r="C1" s="127"/>
-      <x:c r="D1" s="127"/>
-      <x:c r="E1" s="127"/>
-      <x:c r="F1" s="127"/>
-      <x:c r="G1" s="127"/>
-      <x:c r="H1" s="127"/>
-      <x:c r="I1" s="127"/>
-      <x:c r="J1" s="127"/>
-      <x:c r="K1" s="127"/>
-      <x:c r="L1" s="127"/>
-      <x:c r="M1" s="127"/>
-      <x:c r="N1" s="127"/>
-      <x:c r="O1" s="127"/>
-      <x:c r="P1" s="127"/>
+      <x:c r="B1" s="141"/>
+      <x:c r="C1" s="141"/>
+      <x:c r="D1" s="141"/>
+      <x:c r="E1" s="141"/>
+      <x:c r="F1" s="141"/>
+      <x:c r="G1" s="141"/>
+      <x:c r="H1" s="141"/>
+      <x:c r="I1" s="141"/>
+      <x:c r="J1" s="141"/>
+      <x:c r="K1" s="141"/>
+      <x:c r="L1" s="141"/>
+      <x:c r="M1" s="141"/>
+      <x:c r="N1" s="141"/>
+      <x:c r="O1" s="141"/>
+      <x:c r="P1" s="141"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="128" t="str">
+      <x:c r="A3" s="142" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="128"/>
-      <x:c r="C3" s="128"/>
-      <x:c r="D3" s="128"/>
-      <x:c r="E3" s="128"/>
-      <x:c r="F3" s="128"/>
-      <x:c r="G3" s="128"/>
-      <x:c r="H3" s="128"/>
-      <x:c r="I3" s="128"/>
-      <x:c r="J3" s="128"/>
-      <x:c r="K3" s="128"/>
-      <x:c r="L3" s="128"/>
-      <x:c r="M3" s="128"/>
-      <x:c r="N3" s="128"/>
-      <x:c r="O3" s="128"/>
-      <x:c r="P3" s="128"/>
+      <x:c r="B3" s="142"/>
+      <x:c r="C3" s="142"/>
+      <x:c r="D3" s="142"/>
+      <x:c r="E3" s="142"/>
+      <x:c r="F3" s="142"/>
+      <x:c r="G3" s="142"/>
+      <x:c r="H3" s="142"/>
+      <x:c r="I3" s="142"/>
+      <x:c r="J3" s="142"/>
+      <x:c r="K3" s="142"/>
+      <x:c r="L3" s="142"/>
+      <x:c r="M3" s="142"/>
+      <x:c r="N3" s="142"/>
+      <x:c r="O3" s="142"/>
+      <x:c r="P3" s="142"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="129" t="str">
+      <x:c r="A5" s="143" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="129" t="str">
+      <x:c r="B5" s="143" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="129" t="str">
+      <x:c r="C5" s="143" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="129" t="str">
+      <x:c r="D5" s="143" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="129" t="str">
+      <x:c r="E5" s="143" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="129" t="str">
+      <x:c r="F5" s="143" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="129" t="str">
+      <x:c r="G5" s="143" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="129" t="str">
+      <x:c r="H5" s="143" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="129" t="str">
+      <x:c r="I5" s="143" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="129" t="str">
+      <x:c r="J5" s="143" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="129" t="str">
+      <x:c r="K5" s="143" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="129" t="str">
+      <x:c r="L5" s="143" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="129" t="str">
+      <x:c r="M5" s="143" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="129" t="str">
+      <x:c r="N5" s="143" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="129" t="str">
+      <x:c r="O5" s="143" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="129" t="str">
+      <x:c r="P5" s="143" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -3885,7 +3936,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="130" t="str">
+      <x:c r="O6" s="144" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -3935,7 +3986,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="131" t="str">
+      <x:c r="O7" s="145" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -3981,7 +4032,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="132" t="str">
+      <x:c r="O8" s="146" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4031,7 +4082,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="131" t="str">
+      <x:c r="O9" s="145" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4081,7 +4132,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="131" t="str">
+      <x:c r="O10" s="145" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4089,36 +4140,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="133" t="str">
+      <x:c r="A11" s="147" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="133"/>
-      <x:c r="C11" s="133"/>
-      <x:c r="D11" s="133"/>
-      <x:c r="E11" s="133"/>
-      <x:c r="F11" s="133"/>
-      <x:c r="G11" s="133"/>
-      <x:c r="H11" s="133"/>
-      <x:c r="I11" s="133"/>
-      <x:c r="J11" s="133"/>
-      <x:c r="K11" s="133"/>
-      <x:c r="L11" s="133"/>
-      <x:c r="M11" s="133"/>
-      <x:c r="N11" s="133"/>
-      <x:c r="O11" s="133"/>
-      <x:c r="P11" s="133"/>
+      <x:c r="B11" s="147"/>
+      <x:c r="C11" s="147"/>
+      <x:c r="D11" s="147"/>
+      <x:c r="E11" s="147"/>
+      <x:c r="F11" s="147"/>
+      <x:c r="G11" s="147"/>
+      <x:c r="H11" s="147"/>
+      <x:c r="I11" s="147"/>
+      <x:c r="J11" s="147"/>
+      <x:c r="K11" s="147"/>
+      <x:c r="L11" s="147"/>
+      <x:c r="M11" s="147"/>
+      <x:c r="N11" s="147"/>
+      <x:c r="O11" s="147"/>
+      <x:c r="P11" s="147"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="134" t="str">
+      <x:c r="A12" s="148" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="134" t="str">
+      <x:c r="B12" s="148" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="134" t="str">
+      <x:c r="C12" s="148" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="134" t="str">
+      <x:c r="D12" s="148" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4132,7 +4183,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="135" t="str">
+      <x:c r="D13" s="149" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4146,7 +4197,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="135" t="str">
+      <x:c r="D14" s="149" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4160,47 +4211,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="135" t="str">
+      <x:c r="D15" s="149" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="133" t="str">
+      <x:c r="A17" s="147" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="133"/>
-      <x:c r="C17" s="133"/>
-      <x:c r="D17" s="133"/>
-      <x:c r="E17" s="133"/>
-      <x:c r="F17" s="133"/>
-      <x:c r="G17" s="133"/>
-      <x:c r="H17" s="133"/>
-      <x:c r="I17" s="133"/>
-      <x:c r="J17" s="133"/>
-      <x:c r="K17" s="133"/>
-      <x:c r="L17" s="133"/>
-      <x:c r="M17" s="133"/>
-      <x:c r="N17" s="133"/>
-      <x:c r="O17" s="133"/>
-      <x:c r="P17" s="133"/>
+      <x:c r="B17" s="147"/>
+      <x:c r="C17" s="147"/>
+      <x:c r="D17" s="147"/>
+      <x:c r="E17" s="147"/>
+      <x:c r="F17" s="147"/>
+      <x:c r="G17" s="147"/>
+      <x:c r="H17" s="147"/>
+      <x:c r="I17" s="147"/>
+      <x:c r="J17" s="147"/>
+      <x:c r="K17" s="147"/>
+      <x:c r="L17" s="147"/>
+      <x:c r="M17" s="147"/>
+      <x:c r="N17" s="147"/>
+      <x:c r="O17" s="147"/>
+      <x:c r="P17" s="147"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="134" t="str">
+      <x:c r="A18" s="148" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="134" t="str">
+      <x:c r="B18" s="148" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="134" t="str">
+      <x:c r="C18" s="148" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="134" t="str">
+      <x:c r="D18" s="148" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="134" t="str">
+      <x:c r="E18" s="148" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="134" t="str">
+      <x:c r="F18" s="148" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4285,72 +4336,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="133" t="str">
+      <x:c r="A24" s="147" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="133"/>
-      <x:c r="C24" s="133"/>
-      <x:c r="D24" s="133"/>
-      <x:c r="E24" s="133"/>
-      <x:c r="F24" s="133"/>
-      <x:c r="G24" s="133"/>
-      <x:c r="H24" s="133"/>
-      <x:c r="I24" s="133"/>
-      <x:c r="J24" s="133"/>
-      <x:c r="K24" s="133"/>
-      <x:c r="L24" s="133"/>
-      <x:c r="M24" s="133"/>
-      <x:c r="N24" s="133"/>
-      <x:c r="O24" s="133"/>
-      <x:c r="P24" s="133"/>
+      <x:c r="B24" s="147"/>
+      <x:c r="C24" s="147"/>
+      <x:c r="D24" s="147"/>
+      <x:c r="E24" s="147"/>
+      <x:c r="F24" s="147"/>
+      <x:c r="G24" s="147"/>
+      <x:c r="H24" s="147"/>
+      <x:c r="I24" s="147"/>
+      <x:c r="J24" s="147"/>
+      <x:c r="K24" s="147"/>
+      <x:c r="L24" s="147"/>
+      <x:c r="M24" s="147"/>
+      <x:c r="N24" s="147"/>
+      <x:c r="O24" s="147"/>
+      <x:c r="P24" s="147"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="129" t="str">
+      <x:c r="A25" s="143" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="129" t="str">
+      <x:c r="B25" s="143" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="129" t="str">
+      <x:c r="C25" s="143" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="129" t="str">
+      <x:c r="D25" s="143" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="129" t="str">
+      <x:c r="E25" s="143" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="129" t="str">
+      <x:c r="F25" s="143" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="129" t="str">
+      <x:c r="G25" s="143" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="129" t="str">
+      <x:c r="H25" s="143" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="129" t="str">
+      <x:c r="I25" s="143" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="129" t="str">
+      <x:c r="J25" s="143" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="129" t="str">
+      <x:c r="K25" s="143" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="129" t="str">
+      <x:c r="L25" s="143" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="129" t="str">
+      <x:c r="M25" s="143" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="129" t="str">
+      <x:c r="N25" s="143" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="129" t="str">
+      <x:c r="O25" s="143" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="129" t="str">
+      <x:c r="P25" s="143" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4397,7 +4448,7 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="131" t="str">
+      <x:c r="O26" s="145" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">

</xml_diff>

<commit_message>
Record noise and UDP loss test results
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rca8f6eb0b04746fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="Rbdd0ebe7fe4441e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R8f98fd57ba7c4f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R3a70050716ea4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Rf889eea625ef4de5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R71ad1e9752e34edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb5299ccd89f14f59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R5bf1242d7ab74f6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="Rf8960da39dc14715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R33f06b32f2d44e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Re7981bcb4d044446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R766ef6d788bc4a86"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="36">
+  <x:fills count="42">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -330,7 +360,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="150">
+  <x:cellXfs count="159">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -661,6 +691,27 @@
     <x:xf numFmtId="0" fontId="3" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="30" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="36" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="39" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -863,7 +914,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5623979d32dc4911"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bafa369f33e44c1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1193,7 +1244,7 @@
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"PASS")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>카테고리</x:v>
@@ -1238,14 +1289,14 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
       <x:c r="E9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
@@ -1253,7 +1304,7 @@
       </x:c>
       <x:c r="G9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1262,7 +1313,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>IFERROR(B7/B6,0)</x:f>
-        <x:v>0.23529411764705882</x:v>
+        <x:v>0.29411764705882354</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>시간 성능</x:v>
@@ -1421,7 +1472,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99b796713ae64afe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc178d52cde94182"/>
 </x:worksheet>
 </file>
 
@@ -2414,13 +2465,17 @@
       <x:c r="A10" s="25" t="str">
         <x:v>A-04</x:v>
       </x:c>
-      <x:c r="B10" s="58"/>
-      <x:c r="C10" s="57"/>
+      <x:c r="B10" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C10" s="57" t="str">
+        <x:v>4b7b1d3</x:v>
+      </x:c>
       <x:c r="D10" s="25" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
       <x:c r="E10" s="25" t="str">
-        <x:v>입력 노이즈</x:v>
+        <x:v>CH1·CH2 입력 노이즈</x:v>
       </x:c>
       <x:c r="F10" s="25" t="str">
         <x:v>RMS noise</x:v>
@@ -2434,25 +2489,43 @@
       <x:c r="I10" s="59" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J10" s="60"/>
-      <x:c r="K10" s="60"/>
-      <x:c r="L10" s="60"/>
-      <x:c r="M10" s="60"/>
-      <x:c r="N10" s="60"/>
-      <x:c r="O10" s="60"/>
-      <x:c r="P10" s="57"/>
+      <x:c r="J10" s="60" t="n">
+        <x:v>18.206</x:v>
+      </x:c>
+      <x:c r="K10" s="60" t="n">
+        <x:v>0.209</x:v>
+      </x:c>
+      <x:c r="L10" s="60" t="n">
+        <x:v>18.206</x:v>
+      </x:c>
+      <x:c r="M10" s="60" t="n">
+        <x:v>7.988</x:v>
+      </x:c>
+      <x:c r="N10" s="60" t="n">
+        <x:v>7.492</x:v>
+      </x:c>
+      <x:c r="O10" s="60" t="n">
+        <x:v>3001</x:v>
+      </x:c>
+      <x:c r="P10" s="57" t="str">
+        <x:v>11 V / 5 A; CH1+CH2; final stable 5 min</x:v>
+      </x:c>
       <x:c r="Q10" s="25" t="str">
         <x:f>IF(OR(H10="",I10="",J10=""),"INPUT",IF(I10="최대",IF(J10&lt;=H10,"PASS","FAIL"),IF(I10="최소",IF(J10&gt;=H10,"PASS","FAIL"),IF(I10="일치",IF(J10=H10,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R10" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S10" s="57"/>
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="S10" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T10" s="57" t="str">
-        <x:v>필터 설정 기록</x:v>
-      </x:c>
-      <x:c r="U10" s="57"/>
+        <x:v>RMS: I1 0.209 mA, V1 13.141 mV, I2 0.397 mA, V2 18.206 mV (최대값 판정).</x:v>
+      </x:c>
+      <x:c r="U10" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="25" t="str">
@@ -2694,8 +2767,12 @@
       <x:c r="A15" s="25" t="str">
         <x:v>N-02</x:v>
       </x:c>
-      <x:c r="B15" s="58"/>
-      <x:c r="C15" s="57"/>
+      <x:c r="B15" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C15" s="57" t="str">
+        <x:v>4b7b1d3</x:v>
+      </x:c>
       <x:c r="D15" s="25" t="str">
         <x:v>통신</x:v>
       </x:c>
@@ -2714,25 +2791,43 @@
       <x:c r="I15" s="59" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J15" s="60"/>
-      <x:c r="K15" s="60"/>
-      <x:c r="L15" s="60"/>
-      <x:c r="M15" s="60"/>
-      <x:c r="N15" s="60"/>
-      <x:c r="O15" s="60"/>
-      <x:c r="P15" s="57"/>
+      <x:c r="J15" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K15" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L15" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M15" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N15" s="60" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O15" s="60" t="n">
+        <x:v>16620</x:v>
+      </x:c>
+      <x:c r="P15" s="57" t="str">
+        <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
+      </x:c>
       <x:c r="Q15" s="25" t="str">
         <x:f>IF(OR(H15="",I15="",J15=""),"INPUT",IF(I15="최대",IF(J15&lt;=H15,"PASS","FAIL"),IF(I15="최소",IF(J15&gt;=H15,"PASS","FAIL"),IF(I15="일치",IF(J15=H15,"PASS","FAIL"),"CHECK"))))</x:f>
         <x:v>INPUT</x:v>
       </x:c>
       <x:c r="R15" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S15" s="57"/>
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="S15" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T15" s="57" t="str">
-        <x:v>동일 LAN 기준</x:v>
-      </x:c>
-      <x:c r="U15" s="57"/>
+        <x:v>ADC sequence 간격 최대 201 (정상 200)으로 UDP 손실 0%. PC 수신 gap 218 ms 1회는 호스트 지연으로 분리.</x:v>
+      </x:c>
+      <x:c r="U15" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="25" t="str">
@@ -3804,92 +3899,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="141" t="str">
+      <x:c r="A1" s="150" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="141"/>
-      <x:c r="C1" s="141"/>
-      <x:c r="D1" s="141"/>
-      <x:c r="E1" s="141"/>
-      <x:c r="F1" s="141"/>
-      <x:c r="G1" s="141"/>
-      <x:c r="H1" s="141"/>
-      <x:c r="I1" s="141"/>
-      <x:c r="J1" s="141"/>
-      <x:c r="K1" s="141"/>
-      <x:c r="L1" s="141"/>
-      <x:c r="M1" s="141"/>
-      <x:c r="N1" s="141"/>
-      <x:c r="O1" s="141"/>
-      <x:c r="P1" s="141"/>
+      <x:c r="B1" s="150"/>
+      <x:c r="C1" s="150"/>
+      <x:c r="D1" s="150"/>
+      <x:c r="E1" s="150"/>
+      <x:c r="F1" s="150"/>
+      <x:c r="G1" s="150"/>
+      <x:c r="H1" s="150"/>
+      <x:c r="I1" s="150"/>
+      <x:c r="J1" s="150"/>
+      <x:c r="K1" s="150"/>
+      <x:c r="L1" s="150"/>
+      <x:c r="M1" s="150"/>
+      <x:c r="N1" s="150"/>
+      <x:c r="O1" s="150"/>
+      <x:c r="P1" s="150"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="142" t="str">
+      <x:c r="A3" s="151" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="142"/>
-      <x:c r="C3" s="142"/>
-      <x:c r="D3" s="142"/>
-      <x:c r="E3" s="142"/>
-      <x:c r="F3" s="142"/>
-      <x:c r="G3" s="142"/>
-      <x:c r="H3" s="142"/>
-      <x:c r="I3" s="142"/>
-      <x:c r="J3" s="142"/>
-      <x:c r="K3" s="142"/>
-      <x:c r="L3" s="142"/>
-      <x:c r="M3" s="142"/>
-      <x:c r="N3" s="142"/>
-      <x:c r="O3" s="142"/>
-      <x:c r="P3" s="142"/>
+      <x:c r="B3" s="151"/>
+      <x:c r="C3" s="151"/>
+      <x:c r="D3" s="151"/>
+      <x:c r="E3" s="151"/>
+      <x:c r="F3" s="151"/>
+      <x:c r="G3" s="151"/>
+      <x:c r="H3" s="151"/>
+      <x:c r="I3" s="151"/>
+      <x:c r="J3" s="151"/>
+      <x:c r="K3" s="151"/>
+      <x:c r="L3" s="151"/>
+      <x:c r="M3" s="151"/>
+      <x:c r="N3" s="151"/>
+      <x:c r="O3" s="151"/>
+      <x:c r="P3" s="151"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="143" t="str">
+      <x:c r="A5" s="152" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="143" t="str">
+      <x:c r="B5" s="152" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="143" t="str">
+      <x:c r="C5" s="152" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="143" t="str">
+      <x:c r="D5" s="152" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="143" t="str">
+      <x:c r="E5" s="152" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="143" t="str">
+      <x:c r="F5" s="152" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="143" t="str">
+      <x:c r="G5" s="152" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="143" t="str">
+      <x:c r="H5" s="152" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="143" t="str">
+      <x:c r="I5" s="152" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="143" t="str">
+      <x:c r="J5" s="152" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="143" t="str">
+      <x:c r="K5" s="152" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="143" t="str">
+      <x:c r="L5" s="152" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="143" t="str">
+      <x:c r="M5" s="152" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="143" t="str">
+      <x:c r="N5" s="152" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="143" t="str">
+      <x:c r="O5" s="152" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="143" t="str">
+      <x:c r="P5" s="152" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -3936,7 +4031,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="144" t="str">
+      <x:c r="O6" s="153" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -3986,7 +4081,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="145" t="str">
+      <x:c r="O7" s="154" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -4032,7 +4127,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="146" t="str">
+      <x:c r="O8" s="155" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4082,7 +4177,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="145" t="str">
+      <x:c r="O9" s="154" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4132,7 +4227,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="145" t="str">
+      <x:c r="O10" s="154" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4140,36 +4235,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="147" t="str">
+      <x:c r="A11" s="156" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="147"/>
-      <x:c r="C11" s="147"/>
-      <x:c r="D11" s="147"/>
-      <x:c r="E11" s="147"/>
-      <x:c r="F11" s="147"/>
-      <x:c r="G11" s="147"/>
-      <x:c r="H11" s="147"/>
-      <x:c r="I11" s="147"/>
-      <x:c r="J11" s="147"/>
-      <x:c r="K11" s="147"/>
-      <x:c r="L11" s="147"/>
-      <x:c r="M11" s="147"/>
-      <x:c r="N11" s="147"/>
-      <x:c r="O11" s="147"/>
-      <x:c r="P11" s="147"/>
+      <x:c r="B11" s="156"/>
+      <x:c r="C11" s="156"/>
+      <x:c r="D11" s="156"/>
+      <x:c r="E11" s="156"/>
+      <x:c r="F11" s="156"/>
+      <x:c r="G11" s="156"/>
+      <x:c r="H11" s="156"/>
+      <x:c r="I11" s="156"/>
+      <x:c r="J11" s="156"/>
+      <x:c r="K11" s="156"/>
+      <x:c r="L11" s="156"/>
+      <x:c r="M11" s="156"/>
+      <x:c r="N11" s="156"/>
+      <x:c r="O11" s="156"/>
+      <x:c r="P11" s="156"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="148" t="str">
+      <x:c r="A12" s="157" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="148" t="str">
+      <x:c r="B12" s="157" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="148" t="str">
+      <x:c r="C12" s="157" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="148" t="str">
+      <x:c r="D12" s="157" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4183,7 +4278,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="149" t="str">
+      <x:c r="D13" s="158" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4197,7 +4292,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="149" t="str">
+      <x:c r="D14" s="158" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4211,47 +4306,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="149" t="str">
+      <x:c r="D15" s="158" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="147" t="str">
+      <x:c r="A17" s="156" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="147"/>
-      <x:c r="C17" s="147"/>
-      <x:c r="D17" s="147"/>
-      <x:c r="E17" s="147"/>
-      <x:c r="F17" s="147"/>
-      <x:c r="G17" s="147"/>
-      <x:c r="H17" s="147"/>
-      <x:c r="I17" s="147"/>
-      <x:c r="J17" s="147"/>
-      <x:c r="K17" s="147"/>
-      <x:c r="L17" s="147"/>
-      <x:c r="M17" s="147"/>
-      <x:c r="N17" s="147"/>
-      <x:c r="O17" s="147"/>
-      <x:c r="P17" s="147"/>
+      <x:c r="B17" s="156"/>
+      <x:c r="C17" s="156"/>
+      <x:c r="D17" s="156"/>
+      <x:c r="E17" s="156"/>
+      <x:c r="F17" s="156"/>
+      <x:c r="G17" s="156"/>
+      <x:c r="H17" s="156"/>
+      <x:c r="I17" s="156"/>
+      <x:c r="J17" s="156"/>
+      <x:c r="K17" s="156"/>
+      <x:c r="L17" s="156"/>
+      <x:c r="M17" s="156"/>
+      <x:c r="N17" s="156"/>
+      <x:c r="O17" s="156"/>
+      <x:c r="P17" s="156"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="148" t="str">
+      <x:c r="A18" s="157" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="148" t="str">
+      <x:c r="B18" s="157" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="148" t="str">
+      <x:c r="C18" s="157" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="148" t="str">
+      <x:c r="D18" s="157" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="148" t="str">
+      <x:c r="E18" s="157" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="148" t="str">
+      <x:c r="F18" s="157" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4336,72 +4431,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="147" t="str">
+      <x:c r="A24" s="156" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="147"/>
-      <x:c r="C24" s="147"/>
-      <x:c r="D24" s="147"/>
-      <x:c r="E24" s="147"/>
-      <x:c r="F24" s="147"/>
-      <x:c r="G24" s="147"/>
-      <x:c r="H24" s="147"/>
-      <x:c r="I24" s="147"/>
-      <x:c r="J24" s="147"/>
-      <x:c r="K24" s="147"/>
-      <x:c r="L24" s="147"/>
-      <x:c r="M24" s="147"/>
-      <x:c r="N24" s="147"/>
-      <x:c r="O24" s="147"/>
-      <x:c r="P24" s="147"/>
+      <x:c r="B24" s="156"/>
+      <x:c r="C24" s="156"/>
+      <x:c r="D24" s="156"/>
+      <x:c r="E24" s="156"/>
+      <x:c r="F24" s="156"/>
+      <x:c r="G24" s="156"/>
+      <x:c r="H24" s="156"/>
+      <x:c r="I24" s="156"/>
+      <x:c r="J24" s="156"/>
+      <x:c r="K24" s="156"/>
+      <x:c r="L24" s="156"/>
+      <x:c r="M24" s="156"/>
+      <x:c r="N24" s="156"/>
+      <x:c r="O24" s="156"/>
+      <x:c r="P24" s="156"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="143" t="str">
+      <x:c r="A25" s="152" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="143" t="str">
+      <x:c r="B25" s="152" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="143" t="str">
+      <x:c r="C25" s="152" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="143" t="str">
+      <x:c r="D25" s="152" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="143" t="str">
+      <x:c r="E25" s="152" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="143" t="str">
+      <x:c r="F25" s="152" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="143" t="str">
+      <x:c r="G25" s="152" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="143" t="str">
+      <x:c r="H25" s="152" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="143" t="str">
+      <x:c r="I25" s="152" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="143" t="str">
+      <x:c r="J25" s="152" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="143" t="str">
+      <x:c r="K25" s="152" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="143" t="str">
+      <x:c r="L25" s="152" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="143" t="str">
+      <x:c r="M25" s="152" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="143" t="str">
+      <x:c r="N25" s="152" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="143" t="str">
+      <x:c r="O25" s="152" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="143" t="str">
+      <x:c r="P25" s="152" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4448,7 +4543,7 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="145" t="str">
+      <x:c r="O26" s="154" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">

</xml_diff>

<commit_message>
Record boot state transition test
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb5299ccd89f14f59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R5bf1242d7ab74f6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="Rf8960da39dc14715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R33f06b32f2d44e7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Re7981bcb4d044446"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R766ef6d788bc4a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4a985c4443954036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R2d8181c6c3034e75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R2b24b832644146f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R902e5eacc7704731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R0106ecab1590483b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R4a7450cc045b4d33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="42">
+  <x:fills count="48">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -360,7 +390,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="159">
+  <x:cellXfs count="168">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -712,6 +742,27 @@
     <x:xf numFmtId="0" fontId="3" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="36" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="39" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="44" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="46" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="42" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -914,7 +965,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bafa369f33e44c1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e88b91ceea04ee6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1244,7 +1295,7 @@
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"PASS")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>카테고리</x:v>
@@ -1272,7 +1323,7 @@
       </x:c>
       <x:c r="E8" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F8" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
@@ -1280,7 +1331,7 @@
       </x:c>
       <x:c r="G8" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1289,7 +1340,7 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
@@ -1313,7 +1364,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>IFERROR(B7/B6,0)</x:f>
-        <x:v>0.29411764705882354</x:v>
+        <x:v>0.35294117647058826</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>시간 성능</x:v>
@@ -1472,7 +1523,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc178d52cde94182"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8167c00aab24a1b"/>
 </x:worksheet>
 </file>
 
@@ -1587,7 +1638,7 @@
         <x:v>s</x:v>
       </x:c>
       <x:c r="F6" s="56" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="55" t="str">
         <x:v>최대</x:v>
@@ -1599,7 +1650,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="J6" s="55" t="str">
-        <x:v>10 정상 프레임 및 DAC health 확인</x:v>
+        <x:v>GUI 첫 VALID 텔레메트리 기준 3초 이내</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2245,8 +2296,12 @@
       <x:c r="A6" s="25" t="str">
         <x:v>F-01</x:v>
       </x:c>
-      <x:c r="B6" s="58"/>
-      <x:c r="C6" s="57"/>
+      <x:c r="B6" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C6" s="57" t="str">
+        <x:v>4b7b1d3</x:v>
+      </x:c>
       <x:c r="D6" s="25" t="str">
         <x:v>기능</x:v>
       </x:c>
@@ -2260,30 +2315,42 @@
         <x:v>s</x:v>
       </x:c>
       <x:c r="H6" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I6" s="59" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J6" s="60"/>
+      <x:c r="J6" s="60" t="n">
+        <x:v>2.312</x:v>
+      </x:c>
       <x:c r="K6" s="60"/>
       <x:c r="L6" s="60"/>
-      <x:c r="M6" s="60"/>
+      <x:c r="M6" s="60" t="n">
+        <x:v>2.312</x:v>
+      </x:c>
       <x:c r="N6" s="60"/>
-      <x:c r="O6" s="60"/>
-      <x:c r="P6" s="57"/>
+      <x:c r="O6" s="60" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P6" s="57" t="str">
+        <x:v>Reset 후 GUI 첫 VALID 텔레메트리</x:v>
+      </x:c>
       <x:c r="Q6" s="25" t="str">
         <x:f>IF(OR(H6="",I6="",J6=""),"INPUT",IF(I6="최대",IF(J6&lt;=H6,"PASS","FAIL"),IF(I6="최소",IF(J6&gt;=H6,"PASS","FAIL"),IF(I6="일치",IF(J6=H6,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R6" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S6" s="57"/>
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="S6" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T6" s="57" t="str">
-        <x:v>10 정상 프레임 및 DAC health 확인</x:v>
-      </x:c>
-      <x:c r="U6" s="57"/>
+        <x:v>반복 부팅 관찰상 GUI 첫 정상 데이터가 보드 시간 약 2–3초. 대표 CSV 첫 VALID 2.312초.</x:v>
+      </x:c>
+      <x:c r="U6" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_091833_148511.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="25" t="str">
@@ -3899,92 +3966,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="150" t="str">
+      <x:c r="A1" s="159" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="150"/>
-      <x:c r="C1" s="150"/>
-      <x:c r="D1" s="150"/>
-      <x:c r="E1" s="150"/>
-      <x:c r="F1" s="150"/>
-      <x:c r="G1" s="150"/>
-      <x:c r="H1" s="150"/>
-      <x:c r="I1" s="150"/>
-      <x:c r="J1" s="150"/>
-      <x:c r="K1" s="150"/>
-      <x:c r="L1" s="150"/>
-      <x:c r="M1" s="150"/>
-      <x:c r="N1" s="150"/>
-      <x:c r="O1" s="150"/>
-      <x:c r="P1" s="150"/>
+      <x:c r="B1" s="159"/>
+      <x:c r="C1" s="159"/>
+      <x:c r="D1" s="159"/>
+      <x:c r="E1" s="159"/>
+      <x:c r="F1" s="159"/>
+      <x:c r="G1" s="159"/>
+      <x:c r="H1" s="159"/>
+      <x:c r="I1" s="159"/>
+      <x:c r="J1" s="159"/>
+      <x:c r="K1" s="159"/>
+      <x:c r="L1" s="159"/>
+      <x:c r="M1" s="159"/>
+      <x:c r="N1" s="159"/>
+      <x:c r="O1" s="159"/>
+      <x:c r="P1" s="159"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="151" t="str">
+      <x:c r="A3" s="160" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="151"/>
-      <x:c r="C3" s="151"/>
-      <x:c r="D3" s="151"/>
-      <x:c r="E3" s="151"/>
-      <x:c r="F3" s="151"/>
-      <x:c r="G3" s="151"/>
-      <x:c r="H3" s="151"/>
-      <x:c r="I3" s="151"/>
-      <x:c r="J3" s="151"/>
-      <x:c r="K3" s="151"/>
-      <x:c r="L3" s="151"/>
-      <x:c r="M3" s="151"/>
-      <x:c r="N3" s="151"/>
-      <x:c r="O3" s="151"/>
-      <x:c r="P3" s="151"/>
+      <x:c r="B3" s="160"/>
+      <x:c r="C3" s="160"/>
+      <x:c r="D3" s="160"/>
+      <x:c r="E3" s="160"/>
+      <x:c r="F3" s="160"/>
+      <x:c r="G3" s="160"/>
+      <x:c r="H3" s="160"/>
+      <x:c r="I3" s="160"/>
+      <x:c r="J3" s="160"/>
+      <x:c r="K3" s="160"/>
+      <x:c r="L3" s="160"/>
+      <x:c r="M3" s="160"/>
+      <x:c r="N3" s="160"/>
+      <x:c r="O3" s="160"/>
+      <x:c r="P3" s="160"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="152" t="str">
+      <x:c r="A5" s="161" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="152" t="str">
+      <x:c r="B5" s="161" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="152" t="str">
+      <x:c r="C5" s="161" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="152" t="str">
+      <x:c r="D5" s="161" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="152" t="str">
+      <x:c r="E5" s="161" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="152" t="str">
+      <x:c r="F5" s="161" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="152" t="str">
+      <x:c r="G5" s="161" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="152" t="str">
+      <x:c r="H5" s="161" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="152" t="str">
+      <x:c r="I5" s="161" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="152" t="str">
+      <x:c r="J5" s="161" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="152" t="str">
+      <x:c r="K5" s="161" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="152" t="str">
+      <x:c r="L5" s="161" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="152" t="str">
+      <x:c r="M5" s="161" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="152" t="str">
+      <x:c r="N5" s="161" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="152" t="str">
+      <x:c r="O5" s="161" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="152" t="str">
+      <x:c r="P5" s="161" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4031,7 +4098,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="153" t="str">
+      <x:c r="O6" s="162" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -4081,7 +4148,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="154" t="str">
+      <x:c r="O7" s="163" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -4127,7 +4194,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="155" t="str">
+      <x:c r="O8" s="164" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4177,7 +4244,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="154" t="str">
+      <x:c r="O9" s="163" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4227,7 +4294,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="154" t="str">
+      <x:c r="O10" s="163" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4235,36 +4302,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="156" t="str">
+      <x:c r="A11" s="165" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="156"/>
-      <x:c r="C11" s="156"/>
-      <x:c r="D11" s="156"/>
-      <x:c r="E11" s="156"/>
-      <x:c r="F11" s="156"/>
-      <x:c r="G11" s="156"/>
-      <x:c r="H11" s="156"/>
-      <x:c r="I11" s="156"/>
-      <x:c r="J11" s="156"/>
-      <x:c r="K11" s="156"/>
-      <x:c r="L11" s="156"/>
-      <x:c r="M11" s="156"/>
-      <x:c r="N11" s="156"/>
-      <x:c r="O11" s="156"/>
-      <x:c r="P11" s="156"/>
+      <x:c r="B11" s="165"/>
+      <x:c r="C11" s="165"/>
+      <x:c r="D11" s="165"/>
+      <x:c r="E11" s="165"/>
+      <x:c r="F11" s="165"/>
+      <x:c r="G11" s="165"/>
+      <x:c r="H11" s="165"/>
+      <x:c r="I11" s="165"/>
+      <x:c r="J11" s="165"/>
+      <x:c r="K11" s="165"/>
+      <x:c r="L11" s="165"/>
+      <x:c r="M11" s="165"/>
+      <x:c r="N11" s="165"/>
+      <x:c r="O11" s="165"/>
+      <x:c r="P11" s="165"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="157" t="str">
+      <x:c r="A12" s="166" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="157" t="str">
+      <x:c r="B12" s="166" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="157" t="str">
+      <x:c r="C12" s="166" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="157" t="str">
+      <x:c r="D12" s="166" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4278,7 +4345,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="158" t="str">
+      <x:c r="D13" s="167" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4292,7 +4359,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="158" t="str">
+      <x:c r="D14" s="167" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4306,47 +4373,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="158" t="str">
+      <x:c r="D15" s="167" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="156" t="str">
+      <x:c r="A17" s="165" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="156"/>
-      <x:c r="C17" s="156"/>
-      <x:c r="D17" s="156"/>
-      <x:c r="E17" s="156"/>
-      <x:c r="F17" s="156"/>
-      <x:c r="G17" s="156"/>
-      <x:c r="H17" s="156"/>
-      <x:c r="I17" s="156"/>
-      <x:c r="J17" s="156"/>
-      <x:c r="K17" s="156"/>
-      <x:c r="L17" s="156"/>
-      <x:c r="M17" s="156"/>
-      <x:c r="N17" s="156"/>
-      <x:c r="O17" s="156"/>
-      <x:c r="P17" s="156"/>
+      <x:c r="B17" s="165"/>
+      <x:c r="C17" s="165"/>
+      <x:c r="D17" s="165"/>
+      <x:c r="E17" s="165"/>
+      <x:c r="F17" s="165"/>
+      <x:c r="G17" s="165"/>
+      <x:c r="H17" s="165"/>
+      <x:c r="I17" s="165"/>
+      <x:c r="J17" s="165"/>
+      <x:c r="K17" s="165"/>
+      <x:c r="L17" s="165"/>
+      <x:c r="M17" s="165"/>
+      <x:c r="N17" s="165"/>
+      <x:c r="O17" s="165"/>
+      <x:c r="P17" s="165"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="157" t="str">
+      <x:c r="A18" s="166" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="157" t="str">
+      <x:c r="B18" s="166" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="157" t="str">
+      <x:c r="C18" s="166" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="157" t="str">
+      <x:c r="D18" s="166" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="157" t="str">
+      <x:c r="E18" s="166" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="157" t="str">
+      <x:c r="F18" s="166" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4431,72 +4498,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="156" t="str">
+      <x:c r="A24" s="165" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="156"/>
-      <x:c r="C24" s="156"/>
-      <x:c r="D24" s="156"/>
-      <x:c r="E24" s="156"/>
-      <x:c r="F24" s="156"/>
-      <x:c r="G24" s="156"/>
-      <x:c r="H24" s="156"/>
-      <x:c r="I24" s="156"/>
-      <x:c r="J24" s="156"/>
-      <x:c r="K24" s="156"/>
-      <x:c r="L24" s="156"/>
-      <x:c r="M24" s="156"/>
-      <x:c r="N24" s="156"/>
-      <x:c r="O24" s="156"/>
-      <x:c r="P24" s="156"/>
+      <x:c r="B24" s="165"/>
+      <x:c r="C24" s="165"/>
+      <x:c r="D24" s="165"/>
+      <x:c r="E24" s="165"/>
+      <x:c r="F24" s="165"/>
+      <x:c r="G24" s="165"/>
+      <x:c r="H24" s="165"/>
+      <x:c r="I24" s="165"/>
+      <x:c r="J24" s="165"/>
+      <x:c r="K24" s="165"/>
+      <x:c r="L24" s="165"/>
+      <x:c r="M24" s="165"/>
+      <x:c r="N24" s="165"/>
+      <x:c r="O24" s="165"/>
+      <x:c r="P24" s="165"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="152" t="str">
+      <x:c r="A25" s="161" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="152" t="str">
+      <x:c r="B25" s="161" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="152" t="str">
+      <x:c r="C25" s="161" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="152" t="str">
+      <x:c r="D25" s="161" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="152" t="str">
+      <x:c r="E25" s="161" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="152" t="str">
+      <x:c r="F25" s="161" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="152" t="str">
+      <x:c r="G25" s="161" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="152" t="str">
+      <x:c r="H25" s="161" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="152" t="str">
+      <x:c r="I25" s="161" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="152" t="str">
+      <x:c r="J25" s="161" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="152" t="str">
+      <x:c r="K25" s="161" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="152" t="str">
+      <x:c r="L25" s="161" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="152" t="str">
+      <x:c r="M25" s="161" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="152" t="str">
+      <x:c r="N25" s="161" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="152" t="str">
+      <x:c r="O25" s="161" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="152" t="str">
+      <x:c r="P25" s="161" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4543,7 +4610,7 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="154" t="str">
+      <x:c r="O26" s="163" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">

</xml_diff>

<commit_message>
Record three-point linearity test
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4a985c4443954036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R2d8181c6c3034e75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R2b24b832644146f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R902e5eacc7704731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R0106ecab1590483b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R4a7450cc045b4d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5e685c84705b4d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="Rbbeeba7158f74781"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R96a8063a2f4e4284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R2f4772bec6374f28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Rdc872c198a004c68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="Rdb49b82e06934174"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="48">
+  <x:fills count="54">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -390,7 +420,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="168">
+  <x:cellXfs count="182">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -763,6 +793,36 @@
     <x:xf numFmtId="0" fontId="3" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="42" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="48" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="51" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -965,7 +1025,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e88b91ceea04ee6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbad03ef8bdcd4400"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1295,7 +1355,7 @@
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"PASS")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>카테고리</x:v>
@@ -1340,14 +1400,14 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
       <x:c r="E9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
@@ -1355,7 +1415,7 @@
       </x:c>
       <x:c r="G9" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1364,7 +1424,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>IFERROR(B7/B6,0)</x:f>
-        <x:v>0.35294117647058826</x:v>
+        <x:v>0.4117647058823529</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>시간 성능</x:v>
@@ -1523,7 +1583,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8167c00aab24a1b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd1f214a836e4aac"/>
 </x:worksheet>
 </file>
 
@@ -2488,13 +2548,17 @@
       <x:c r="A9" s="25" t="str">
         <x:v>A-03</x:v>
       </x:c>
-      <x:c r="B9" s="58"/>
-      <x:c r="C9" s="57"/>
+      <x:c r="B9" s="58" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C9" s="57" t="str">
+        <x:v>f9ceb9a</x:v>
+      </x:c>
       <x:c r="D9" s="25" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
       <x:c r="E9" s="25" t="str">
-        <x:v>선형성</x:v>
+        <x:v>CH1·CH2 선형성</x:v>
       </x:c>
       <x:c r="F9" s="25" t="str">
         <x:v>0/50/100% 최대 편차</x:v>
@@ -2508,25 +2572,43 @@
       <x:c r="I9" s="59" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J9" s="60"/>
-      <x:c r="K9" s="60"/>
-      <x:c r="L9" s="60"/>
-      <x:c r="M9" s="60"/>
-      <x:c r="N9" s="60"/>
-      <x:c r="O9" s="60"/>
-      <x:c r="P9" s="57"/>
+      <x:c r="J9" s="60" t="n">
+        <x:v>0.2803</x:v>
+      </x:c>
+      <x:c r="K9" s="60" t="n">
+        <x:v>0.0098</x:v>
+      </x:c>
+      <x:c r="L9" s="60" t="n">
+        <x:v>0.2803</x:v>
+      </x:c>
+      <x:c r="M9" s="60" t="n">
+        <x:v>0.14135</x:v>
+      </x:c>
+      <x:c r="N9" s="60" t="n">
+        <x:v>0.1275</x:v>
+      </x:c>
+      <x:c r="O9" s="60" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P9" s="57" t="str">
+        <x:v>CH1+CH2; CSV 구간 0 V / 약 5 V / 약 10 V</x:v>
+      </x:c>
       <x:c r="Q9" s="25" t="str">
         <x:f>IF(OR(H9="",I9="",J9=""),"INPUT",IF(I9="최대",IF(J9&lt;=H9,"PASS","FAIL"),IF(I9="최소",IF(J9&gt;=H9,"PASS","FAIL"),IF(I9="일치",IF(J9=H9,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R9" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
-      <x:c r="S9" s="57"/>
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="S9" s="57" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
       <x:c r="T9" s="57" t="str">
-        <x:v>다점 결과 첨부</x:v>
-      </x:c>
-      <x:c r="U9" s="57"/>
+        <x:v>50% 점 편차: I1 0.2803%, V1 0.0184%, I2 0.2569%, V2 0.0098%FS. 절대 게인은 현장 검증 이관.</x:v>
+      </x:c>
+      <x:c r="U9" s="57" t="str">
+        <x:v>logs/cosmoke_capture_20260820_103337_769201.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="25" t="str">
@@ -3966,92 +4048,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="159" t="str">
+      <x:c r="A1" s="168" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="159"/>
-      <x:c r="C1" s="159"/>
-      <x:c r="D1" s="159"/>
-      <x:c r="E1" s="159"/>
-      <x:c r="F1" s="159"/>
-      <x:c r="G1" s="159"/>
-      <x:c r="H1" s="159"/>
-      <x:c r="I1" s="159"/>
-      <x:c r="J1" s="159"/>
-      <x:c r="K1" s="159"/>
-      <x:c r="L1" s="159"/>
-      <x:c r="M1" s="159"/>
-      <x:c r="N1" s="159"/>
-      <x:c r="O1" s="159"/>
-      <x:c r="P1" s="159"/>
+      <x:c r="B1" s="168"/>
+      <x:c r="C1" s="168"/>
+      <x:c r="D1" s="168"/>
+      <x:c r="E1" s="168"/>
+      <x:c r="F1" s="168"/>
+      <x:c r="G1" s="168"/>
+      <x:c r="H1" s="168"/>
+      <x:c r="I1" s="168"/>
+      <x:c r="J1" s="168"/>
+      <x:c r="K1" s="168"/>
+      <x:c r="L1" s="168"/>
+      <x:c r="M1" s="168"/>
+      <x:c r="N1" s="168"/>
+      <x:c r="O1" s="168"/>
+      <x:c r="P1" s="168"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="160" t="str">
+      <x:c r="A3" s="169" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="160"/>
-      <x:c r="C3" s="160"/>
-      <x:c r="D3" s="160"/>
-      <x:c r="E3" s="160"/>
-      <x:c r="F3" s="160"/>
-      <x:c r="G3" s="160"/>
-      <x:c r="H3" s="160"/>
-      <x:c r="I3" s="160"/>
-      <x:c r="J3" s="160"/>
-      <x:c r="K3" s="160"/>
-      <x:c r="L3" s="160"/>
-      <x:c r="M3" s="160"/>
-      <x:c r="N3" s="160"/>
-      <x:c r="O3" s="160"/>
-      <x:c r="P3" s="160"/>
+      <x:c r="B3" s="169"/>
+      <x:c r="C3" s="169"/>
+      <x:c r="D3" s="169"/>
+      <x:c r="E3" s="169"/>
+      <x:c r="F3" s="169"/>
+      <x:c r="G3" s="169"/>
+      <x:c r="H3" s="169"/>
+      <x:c r="I3" s="169"/>
+      <x:c r="J3" s="169"/>
+      <x:c r="K3" s="169"/>
+      <x:c r="L3" s="169"/>
+      <x:c r="M3" s="169"/>
+      <x:c r="N3" s="169"/>
+      <x:c r="O3" s="169"/>
+      <x:c r="P3" s="169"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="161" t="str">
+      <x:c r="A5" s="170" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="161" t="str">
+      <x:c r="B5" s="170" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="161" t="str">
+      <x:c r="C5" s="170" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="161" t="str">
+      <x:c r="D5" s="170" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="161" t="str">
+      <x:c r="E5" s="170" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="161" t="str">
+      <x:c r="F5" s="170" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="161" t="str">
+      <x:c r="G5" s="170" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="161" t="str">
+      <x:c r="H5" s="170" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="161" t="str">
+      <x:c r="I5" s="170" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="161" t="str">
+      <x:c r="J5" s="170" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="161" t="str">
+      <x:c r="K5" s="170" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="161" t="str">
+      <x:c r="L5" s="170" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="161" t="str">
+      <x:c r="M5" s="170" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="161" t="str">
+      <x:c r="N5" s="170" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="161" t="str">
+      <x:c r="O5" s="170" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="161" t="str">
+      <x:c r="P5" s="170" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4098,7 +4180,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="162" t="str">
+      <x:c r="O6" s="171" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -4148,7 +4230,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="163" t="str">
+      <x:c r="O7" s="172" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -4194,7 +4276,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="164" t="str">
+      <x:c r="O8" s="173" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4244,7 +4326,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="163" t="str">
+      <x:c r="O9" s="172" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4294,7 +4376,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="163" t="str">
+      <x:c r="O10" s="172" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4302,36 +4384,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="165" t="str">
+      <x:c r="A11" s="174" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="165"/>
-      <x:c r="C11" s="165"/>
-      <x:c r="D11" s="165"/>
-      <x:c r="E11" s="165"/>
-      <x:c r="F11" s="165"/>
-      <x:c r="G11" s="165"/>
-      <x:c r="H11" s="165"/>
-      <x:c r="I11" s="165"/>
-      <x:c r="J11" s="165"/>
-      <x:c r="K11" s="165"/>
-      <x:c r="L11" s="165"/>
-      <x:c r="M11" s="165"/>
-      <x:c r="N11" s="165"/>
-      <x:c r="O11" s="165"/>
-      <x:c r="P11" s="165"/>
+      <x:c r="B11" s="174"/>
+      <x:c r="C11" s="174"/>
+      <x:c r="D11" s="174"/>
+      <x:c r="E11" s="174"/>
+      <x:c r="F11" s="174"/>
+      <x:c r="G11" s="174"/>
+      <x:c r="H11" s="174"/>
+      <x:c r="I11" s="174"/>
+      <x:c r="J11" s="174"/>
+      <x:c r="K11" s="174"/>
+      <x:c r="L11" s="174"/>
+      <x:c r="M11" s="174"/>
+      <x:c r="N11" s="174"/>
+      <x:c r="O11" s="174"/>
+      <x:c r="P11" s="174"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="166" t="str">
+      <x:c r="A12" s="175" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="166" t="str">
+      <x:c r="B12" s="175" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="166" t="str">
+      <x:c r="C12" s="175" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="166" t="str">
+      <x:c r="D12" s="175" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4345,7 +4427,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="167" t="str">
+      <x:c r="D13" s="176" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4359,7 +4441,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="167" t="str">
+      <x:c r="D14" s="176" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4373,47 +4455,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="167" t="str">
+      <x:c r="D15" s="176" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="165" t="str">
+      <x:c r="A17" s="174" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="165"/>
-      <x:c r="C17" s="165"/>
-      <x:c r="D17" s="165"/>
-      <x:c r="E17" s="165"/>
-      <x:c r="F17" s="165"/>
-      <x:c r="G17" s="165"/>
-      <x:c r="H17" s="165"/>
-      <x:c r="I17" s="165"/>
-      <x:c r="J17" s="165"/>
-      <x:c r="K17" s="165"/>
-      <x:c r="L17" s="165"/>
-      <x:c r="M17" s="165"/>
-      <x:c r="N17" s="165"/>
-      <x:c r="O17" s="165"/>
-      <x:c r="P17" s="165"/>
+      <x:c r="B17" s="174"/>
+      <x:c r="C17" s="174"/>
+      <x:c r="D17" s="174"/>
+      <x:c r="E17" s="174"/>
+      <x:c r="F17" s="174"/>
+      <x:c r="G17" s="174"/>
+      <x:c r="H17" s="174"/>
+      <x:c r="I17" s="174"/>
+      <x:c r="J17" s="174"/>
+      <x:c r="K17" s="174"/>
+      <x:c r="L17" s="174"/>
+      <x:c r="M17" s="174"/>
+      <x:c r="N17" s="174"/>
+      <x:c r="O17" s="174"/>
+      <x:c r="P17" s="174"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="166" t="str">
+      <x:c r="A18" s="175" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="166" t="str">
+      <x:c r="B18" s="175" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="166" t="str">
+      <x:c r="C18" s="175" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="166" t="str">
+      <x:c r="D18" s="175" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="166" t="str">
+      <x:c r="E18" s="175" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="166" t="str">
+      <x:c r="F18" s="175" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4498,72 +4580,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="165" t="str">
+      <x:c r="A24" s="174" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="165"/>
-      <x:c r="C24" s="165"/>
-      <x:c r="D24" s="165"/>
-      <x:c r="E24" s="165"/>
-      <x:c r="F24" s="165"/>
-      <x:c r="G24" s="165"/>
-      <x:c r="H24" s="165"/>
-      <x:c r="I24" s="165"/>
-      <x:c r="J24" s="165"/>
-      <x:c r="K24" s="165"/>
-      <x:c r="L24" s="165"/>
-      <x:c r="M24" s="165"/>
-      <x:c r="N24" s="165"/>
-      <x:c r="O24" s="165"/>
-      <x:c r="P24" s="165"/>
+      <x:c r="B24" s="174"/>
+      <x:c r="C24" s="174"/>
+      <x:c r="D24" s="174"/>
+      <x:c r="E24" s="174"/>
+      <x:c r="F24" s="174"/>
+      <x:c r="G24" s="174"/>
+      <x:c r="H24" s="174"/>
+      <x:c r="I24" s="174"/>
+      <x:c r="J24" s="174"/>
+      <x:c r="K24" s="174"/>
+      <x:c r="L24" s="174"/>
+      <x:c r="M24" s="174"/>
+      <x:c r="N24" s="174"/>
+      <x:c r="O24" s="174"/>
+      <x:c r="P24" s="174"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="161" t="str">
+      <x:c r="A25" s="170" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="161" t="str">
+      <x:c r="B25" s="170" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="161" t="str">
+      <x:c r="C25" s="170" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="161" t="str">
+      <x:c r="D25" s="170" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="161" t="str">
+      <x:c r="E25" s="170" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="161" t="str">
+      <x:c r="F25" s="170" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="161" t="str">
+      <x:c r="G25" s="170" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="161" t="str">
+      <x:c r="H25" s="170" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="161" t="str">
+      <x:c r="I25" s="170" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="161" t="str">
+      <x:c r="J25" s="170" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="161" t="str">
+      <x:c r="K25" s="170" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="161" t="str">
+      <x:c r="L25" s="170" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="161" t="str">
+      <x:c r="M25" s="170" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="161" t="str">
+      <x:c r="N25" s="170" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="161" t="str">
+      <x:c r="O25" s="170" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="161" t="str">
+      <x:c r="P25" s="170" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4610,11 +4692,131 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="163" t="str">
+      <x:c r="O26" s="172" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">
         <x:v>0 입력 구간 44프레임 제외. 게인 오차: I1 +5.97%, V1 +9.80%, I2 +3.32%, V2 +10.44%; SCALE_TRIM 적용 후 재시험 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="174" t="str">
+        <x:v>추가 캡처: 3점 상대 선형성 시험</x:v>
+      </x:c>
+      <x:c r="B28" s="174"/>
+      <x:c r="C28" s="174"/>
+      <x:c r="D28" s="174"/>
+      <x:c r="E28" s="174"/>
+      <x:c r="F28" s="174"/>
+      <x:c r="G28" s="174"/>
+      <x:c r="H28" s="174"/>
+      <x:c r="I28" s="174"/>
+      <x:c r="J28" s="174"/>
+      <x:c r="K28" s="174"/>
+      <x:c r="L28" s="174"/>
+      <x:c r="M28" s="174"/>
+      <x:c r="N28" s="174"/>
+      <x:c r="O28" s="174"/>
+      <x:c r="P28" s="174"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="170" t="str">
+        <x:v>CSV 파일</x:v>
+      </x:c>
+      <x:c r="B29" s="170" t="str">
+        <x:v>시험 목적</x:v>
+      </x:c>
+      <x:c r="C29" s="170" t="str">
+        <x:v>FW commit</x:v>
+      </x:c>
+      <x:c r="D29" s="170" t="str">
+        <x:v>부팅 구간</x:v>
+      </x:c>
+      <x:c r="E29" s="170" t="str">
+        <x:v>프레임</x:v>
+      </x:c>
+      <x:c r="F29" s="170" t="str">
+        <x:v>PC 시간 (s)</x:v>
+      </x:c>
+      <x:c r="G29" s="170" t="str">
+        <x:v>보드 시간 (s)</x:v>
+      </x:c>
+      <x:c r="H29" s="170" t="str">
+        <x:v>시간비</x:v>
+      </x:c>
+      <x:c r="I29" s="170" t="str">
+        <x:v>ADC rate (Hz)</x:v>
+      </x:c>
+      <x:c r="J29" s="170" t="str">
+        <x:v>UDP 평균 (ms)</x:v>
+      </x:c>
+      <x:c r="K29" s="170" t="str">
+        <x:v>UDP 범위 (ms)</x:v>
+      </x:c>
+      <x:c r="L29" s="170" t="str">
+        <x:v>드랍 최대</x:v>
+      </x:c>
+      <x:c r="M29" s="170" t="str">
+        <x:v>오류</x:v>
+      </x:c>
+      <x:c r="N29" s="170" t="str">
+        <x:v>입력/조건</x:v>
+      </x:c>
+      <x:c r="O29" s="170" t="str">
+        <x:v>판정</x:v>
+      </x:c>
+      <x:c r="P29" s="170" t="str">
+        <x:v>분석 메모</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="48" customHeight="1">
+      <x:c r="A30" s="100" t="str">
+        <x:v>cosmoke_capture_20260820_103337_769201.csv</x:v>
+      </x:c>
+      <x:c r="B30" s="100" t="str">
+        <x:v>CH1·CH2 3점 상대 선형성</x:v>
+      </x:c>
+      <x:c r="C30" s="100" t="str">
+        <x:v>f9ceb9a</x:v>
+      </x:c>
+      <x:c r="D30" s="100" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E30" s="100" t="n">
+        <x:v>3135</x:v>
+      </x:c>
+      <x:c r="F30" s="105" t="n">
+        <x:v>313.399</x:v>
+      </x:c>
+      <x:c r="G30" s="105" t="n">
+        <x:v>313.4</x:v>
+      </x:c>
+      <x:c r="H30" s="105" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I30" s="105" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J30" s="105" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K30" s="100" t="str">
+        <x:v>99–101</x:v>
+      </x:c>
+      <x:c r="L30" s="106" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="100" t="str">
+        <x:v>CRC/SPI/DAC=0</x:v>
+      </x:c>
+      <x:c r="N30" s="100" t="str">
+        <x:v>0 V / 약 5 V / 약 10 V</x:v>
+      </x:c>
+      <x:c r="O30" s="172" t="str">
+        <x:v>PASS (상대 선형성)</x:v>
+      </x:c>
+      <x:c r="P30" s="100" t="str">
+        <x:v>50%FS 최대 편차 0.2803% (기준 1%). 절대 전압·전류 기준값은 현장 검증 이관.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4624,6 +4826,7 @@
     <x:mergeCell ref="A11:P11"/>
     <x:mergeCell ref="A17:P17"/>
     <x:mergeCell ref="A24:P24"/>
+    <x:mergeCell ref="A28:P28"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Remove DAC response test from bench plan
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5e685c84705b4d21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="Rbbeeba7158f74781"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R96a8063a2f4e4284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R2f4772bec6374f28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Rdc872c198a004c68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="Rdb49b82e06934174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re1bf95d1adfd4e7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R8953be38cb2e4817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R3a5b6bfc62644572"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rf379f3416bbf4163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R8e9e20bdafba407a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="Rb112bbe406b345bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="54">
+  <x:fills count="60">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -420,7 +450,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="182">
+  <x:cellXfs count="191">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -823,6 +853,27 @@
     <x:xf numFmtId="0" fontId="0" fillId="51" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="56" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="58" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1025,7 +1076,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbad03ef8bdcd4400"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re707023819774079"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1325,7 +1376,7 @@
       </x:c>
       <x:c r="B6" s="17" t="n">
         <x:f>COUNTA('Test Log'!A2:A201)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
         <x:v>카테고리별 결과</x:v>
@@ -1400,7 +1451,7 @@
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
@@ -1424,7 +1475,7 @@
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f>IFERROR(B7/B6,0)</x:f>
-        <x:v>0.4117647058823529</x:v>
+        <x:v>0.4375</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>시간 성능</x:v>
@@ -1439,7 +1490,7 @@
       </x:c>
       <x:c r="G10" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1583,7 +1634,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd1f214a836e4aac"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9577d22f5ac749ce"/>
 </x:worksheet>
 </file>
 
@@ -1906,36 +1957,16 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="55" t="str">
-        <x:v>T-03</x:v>
-      </x:c>
-      <x:c r="B13" s="55" t="str">
-        <x:v>시간 성능</x:v>
-      </x:c>
-      <x:c r="C13" s="55" t="str">
-        <x:v>DAC 응답</x:v>
-      </x:c>
-      <x:c r="D13" s="55" t="str">
-        <x:v>입력 step→출력 안정화</x:v>
-      </x:c>
-      <x:c r="E13" s="55" t="str">
-        <x:v>ms</x:v>
-      </x:c>
-      <x:c r="F13" s="56" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="G13" s="55" t="str">
-        <x:v>최대</x:v>
-      </x:c>
-      <x:c r="H13" s="55" t="str">
-        <x:v>oscilloscope</x:v>
-      </x:c>
-      <x:c r="I13" s="55" t="str">
-        <x:v>P1</x:v>
-      </x:c>
-      <x:c r="J13" s="55" t="str">
-        <x:v>필터 포함 end-to-end</x:v>
-      </x:c>
+      <x:c r="A13" s="55"/>
+      <x:c r="B13" s="55"/>
+      <x:c r="C13" s="55"/>
+      <x:c r="D13" s="55"/>
+      <x:c r="E13" s="55"/>
+      <x:c r="F13" s="56"/>
+      <x:c r="G13" s="55"/>
+      <x:c r="H13" s="55"/>
+      <x:c r="I13" s="55"/>
+      <x:c r="J13" s="55"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="55" t="str">
@@ -2803,29 +2834,15 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="25" t="str">
-        <x:v>T-03</x:v>
-      </x:c>
+      <x:c r="A13" s="25"/>
       <x:c r="B13" s="58"/>
       <x:c r="C13" s="57"/>
-      <x:c r="D13" s="25" t="str">
-        <x:v>시간 성능</x:v>
-      </x:c>
-      <x:c r="E13" s="25" t="str">
-        <x:v>DAC 응답</x:v>
-      </x:c>
-      <x:c r="F13" s="25" t="str">
-        <x:v>입력 step→출력 안정화</x:v>
-      </x:c>
-      <x:c r="G13" s="25" t="str">
-        <x:v>ms</x:v>
-      </x:c>
-      <x:c r="H13" s="59" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="I13" s="59" t="str">
-        <x:v>최대</x:v>
-      </x:c>
+      <x:c r="D13" s="25"/>
+      <x:c r="E13" s="25"/>
+      <x:c r="F13" s="25"/>
+      <x:c r="G13" s="25"/>
+      <x:c r="H13" s="59"/>
+      <x:c r="I13" s="59"/>
       <x:c r="J13" s="60"/>
       <x:c r="K13" s="60"/>
       <x:c r="L13" s="60"/>
@@ -2833,17 +2850,10 @@
       <x:c r="N13" s="60"/>
       <x:c r="O13" s="60"/>
       <x:c r="P13" s="57"/>
-      <x:c r="Q13" s="25" t="str">
-        <x:f>IF(OR(H13="",I13="",J13=""),"INPUT",IF(I13="최대",IF(J13&lt;=H13,"PASS","FAIL"),IF(I13="최소",IF(J13&gt;=H13,"PASS","FAIL"),IF(I13="일치",IF(J13=H13,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
-      </x:c>
-      <x:c r="R13" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
+      <x:c r="Q13" s="25"/>
+      <x:c r="R13" s="57"/>
       <x:c r="S13" s="57"/>
-      <x:c r="T13" s="57" t="str">
-        <x:v>필터 포함 end-to-end</x:v>
-      </x:c>
+      <x:c r="T13" s="57"/>
       <x:c r="U13" s="57"/>
     </x:row>
     <x:row r="14">
@@ -4048,92 +4058,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="168" t="str">
+      <x:c r="A1" s="182" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="168"/>
-      <x:c r="C1" s="168"/>
-      <x:c r="D1" s="168"/>
-      <x:c r="E1" s="168"/>
-      <x:c r="F1" s="168"/>
-      <x:c r="G1" s="168"/>
-      <x:c r="H1" s="168"/>
-      <x:c r="I1" s="168"/>
-      <x:c r="J1" s="168"/>
-      <x:c r="K1" s="168"/>
-      <x:c r="L1" s="168"/>
-      <x:c r="M1" s="168"/>
-      <x:c r="N1" s="168"/>
-      <x:c r="O1" s="168"/>
-      <x:c r="P1" s="168"/>
+      <x:c r="B1" s="182"/>
+      <x:c r="C1" s="182"/>
+      <x:c r="D1" s="182"/>
+      <x:c r="E1" s="182"/>
+      <x:c r="F1" s="182"/>
+      <x:c r="G1" s="182"/>
+      <x:c r="H1" s="182"/>
+      <x:c r="I1" s="182"/>
+      <x:c r="J1" s="182"/>
+      <x:c r="K1" s="182"/>
+      <x:c r="L1" s="182"/>
+      <x:c r="M1" s="182"/>
+      <x:c r="N1" s="182"/>
+      <x:c r="O1" s="182"/>
+      <x:c r="P1" s="182"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="169" t="str">
+      <x:c r="A3" s="183" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="169"/>
-      <x:c r="C3" s="169"/>
-      <x:c r="D3" s="169"/>
-      <x:c r="E3" s="169"/>
-      <x:c r="F3" s="169"/>
-      <x:c r="G3" s="169"/>
-      <x:c r="H3" s="169"/>
-      <x:c r="I3" s="169"/>
-      <x:c r="J3" s="169"/>
-      <x:c r="K3" s="169"/>
-      <x:c r="L3" s="169"/>
-      <x:c r="M3" s="169"/>
-      <x:c r="N3" s="169"/>
-      <x:c r="O3" s="169"/>
-      <x:c r="P3" s="169"/>
+      <x:c r="B3" s="183"/>
+      <x:c r="C3" s="183"/>
+      <x:c r="D3" s="183"/>
+      <x:c r="E3" s="183"/>
+      <x:c r="F3" s="183"/>
+      <x:c r="G3" s="183"/>
+      <x:c r="H3" s="183"/>
+      <x:c r="I3" s="183"/>
+      <x:c r="J3" s="183"/>
+      <x:c r="K3" s="183"/>
+      <x:c r="L3" s="183"/>
+      <x:c r="M3" s="183"/>
+      <x:c r="N3" s="183"/>
+      <x:c r="O3" s="183"/>
+      <x:c r="P3" s="183"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="170" t="str">
+      <x:c r="A5" s="184" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="170" t="str">
+      <x:c r="B5" s="184" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="170" t="str">
+      <x:c r="C5" s="184" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="170" t="str">
+      <x:c r="D5" s="184" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="170" t="str">
+      <x:c r="E5" s="184" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="170" t="str">
+      <x:c r="F5" s="184" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="170" t="str">
+      <x:c r="G5" s="184" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="170" t="str">
+      <x:c r="H5" s="184" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="170" t="str">
+      <x:c r="I5" s="184" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="170" t="str">
+      <x:c r="J5" s="184" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="170" t="str">
+      <x:c r="K5" s="184" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="170" t="str">
+      <x:c r="L5" s="184" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="170" t="str">
+      <x:c r="M5" s="184" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="170" t="str">
+      <x:c r="N5" s="184" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="170" t="str">
+      <x:c r="O5" s="184" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="170" t="str">
+      <x:c r="P5" s="184" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4180,7 +4190,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="171" t="str">
+      <x:c r="O6" s="185" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -4230,7 +4240,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="172" t="str">
+      <x:c r="O7" s="186" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -4276,7 +4286,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="173" t="str">
+      <x:c r="O8" s="187" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4326,7 +4336,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="172" t="str">
+      <x:c r="O9" s="186" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4376,7 +4386,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="172" t="str">
+      <x:c r="O10" s="186" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4384,36 +4394,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="174" t="str">
+      <x:c r="A11" s="188" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="174"/>
-      <x:c r="C11" s="174"/>
-      <x:c r="D11" s="174"/>
-      <x:c r="E11" s="174"/>
-      <x:c r="F11" s="174"/>
-      <x:c r="G11" s="174"/>
-      <x:c r="H11" s="174"/>
-      <x:c r="I11" s="174"/>
-      <x:c r="J11" s="174"/>
-      <x:c r="K11" s="174"/>
-      <x:c r="L11" s="174"/>
-      <x:c r="M11" s="174"/>
-      <x:c r="N11" s="174"/>
-      <x:c r="O11" s="174"/>
-      <x:c r="P11" s="174"/>
+      <x:c r="B11" s="188"/>
+      <x:c r="C11" s="188"/>
+      <x:c r="D11" s="188"/>
+      <x:c r="E11" s="188"/>
+      <x:c r="F11" s="188"/>
+      <x:c r="G11" s="188"/>
+      <x:c r="H11" s="188"/>
+      <x:c r="I11" s="188"/>
+      <x:c r="J11" s="188"/>
+      <x:c r="K11" s="188"/>
+      <x:c r="L11" s="188"/>
+      <x:c r="M11" s="188"/>
+      <x:c r="N11" s="188"/>
+      <x:c r="O11" s="188"/>
+      <x:c r="P11" s="188"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="175" t="str">
+      <x:c r="A12" s="189" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="175" t="str">
+      <x:c r="B12" s="189" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="175" t="str">
+      <x:c r="C12" s="189" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="175" t="str">
+      <x:c r="D12" s="189" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4427,7 +4437,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="176" t="str">
+      <x:c r="D13" s="190" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4441,7 +4451,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="176" t="str">
+      <x:c r="D14" s="190" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4455,47 +4465,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="176" t="str">
+      <x:c r="D15" s="190" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="174" t="str">
+      <x:c r="A17" s="188" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="174"/>
-      <x:c r="C17" s="174"/>
-      <x:c r="D17" s="174"/>
-      <x:c r="E17" s="174"/>
-      <x:c r="F17" s="174"/>
-      <x:c r="G17" s="174"/>
-      <x:c r="H17" s="174"/>
-      <x:c r="I17" s="174"/>
-      <x:c r="J17" s="174"/>
-      <x:c r="K17" s="174"/>
-      <x:c r="L17" s="174"/>
-      <x:c r="M17" s="174"/>
-      <x:c r="N17" s="174"/>
-      <x:c r="O17" s="174"/>
-      <x:c r="P17" s="174"/>
+      <x:c r="B17" s="188"/>
+      <x:c r="C17" s="188"/>
+      <x:c r="D17" s="188"/>
+      <x:c r="E17" s="188"/>
+      <x:c r="F17" s="188"/>
+      <x:c r="G17" s="188"/>
+      <x:c r="H17" s="188"/>
+      <x:c r="I17" s="188"/>
+      <x:c r="J17" s="188"/>
+      <x:c r="K17" s="188"/>
+      <x:c r="L17" s="188"/>
+      <x:c r="M17" s="188"/>
+      <x:c r="N17" s="188"/>
+      <x:c r="O17" s="188"/>
+      <x:c r="P17" s="188"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="175" t="str">
+      <x:c r="A18" s="189" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="175" t="str">
+      <x:c r="B18" s="189" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="175" t="str">
+      <x:c r="C18" s="189" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="175" t="str">
+      <x:c r="D18" s="189" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="175" t="str">
+      <x:c r="E18" s="189" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="175" t="str">
+      <x:c r="F18" s="189" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4580,72 +4590,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="174" t="str">
+      <x:c r="A24" s="188" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="174"/>
-      <x:c r="C24" s="174"/>
-      <x:c r="D24" s="174"/>
-      <x:c r="E24" s="174"/>
-      <x:c r="F24" s="174"/>
-      <x:c r="G24" s="174"/>
-      <x:c r="H24" s="174"/>
-      <x:c r="I24" s="174"/>
-      <x:c r="J24" s="174"/>
-      <x:c r="K24" s="174"/>
-      <x:c r="L24" s="174"/>
-      <x:c r="M24" s="174"/>
-      <x:c r="N24" s="174"/>
-      <x:c r="O24" s="174"/>
-      <x:c r="P24" s="174"/>
+      <x:c r="B24" s="188"/>
+      <x:c r="C24" s="188"/>
+      <x:c r="D24" s="188"/>
+      <x:c r="E24" s="188"/>
+      <x:c r="F24" s="188"/>
+      <x:c r="G24" s="188"/>
+      <x:c r="H24" s="188"/>
+      <x:c r="I24" s="188"/>
+      <x:c r="J24" s="188"/>
+      <x:c r="K24" s="188"/>
+      <x:c r="L24" s="188"/>
+      <x:c r="M24" s="188"/>
+      <x:c r="N24" s="188"/>
+      <x:c r="O24" s="188"/>
+      <x:c r="P24" s="188"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="170" t="str">
+      <x:c r="A25" s="184" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="170" t="str">
+      <x:c r="B25" s="184" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="170" t="str">
+      <x:c r="C25" s="184" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="170" t="str">
+      <x:c r="D25" s="184" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="170" t="str">
+      <x:c r="E25" s="184" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="170" t="str">
+      <x:c r="F25" s="184" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="170" t="str">
+      <x:c r="G25" s="184" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="170" t="str">
+      <x:c r="H25" s="184" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="170" t="str">
+      <x:c r="I25" s="184" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="170" t="str">
+      <x:c r="J25" s="184" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="170" t="str">
+      <x:c r="K25" s="184" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="170" t="str">
+      <x:c r="L25" s="184" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="170" t="str">
+      <x:c r="M25" s="184" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="170" t="str">
+      <x:c r="N25" s="184" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="170" t="str">
+      <x:c r="O25" s="184" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="170" t="str">
+      <x:c r="P25" s="184" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4692,7 +4702,7 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="172" t="str">
+      <x:c r="O26" s="186" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">
@@ -4700,72 +4710,72 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="174" t="str">
+      <x:c r="A28" s="188" t="str">
         <x:v>추가 캡처: 3점 상대 선형성 시험</x:v>
       </x:c>
-      <x:c r="B28" s="174"/>
-      <x:c r="C28" s="174"/>
-      <x:c r="D28" s="174"/>
-      <x:c r="E28" s="174"/>
-      <x:c r="F28" s="174"/>
-      <x:c r="G28" s="174"/>
-      <x:c r="H28" s="174"/>
-      <x:c r="I28" s="174"/>
-      <x:c r="J28" s="174"/>
-      <x:c r="K28" s="174"/>
-      <x:c r="L28" s="174"/>
-      <x:c r="M28" s="174"/>
-      <x:c r="N28" s="174"/>
-      <x:c r="O28" s="174"/>
-      <x:c r="P28" s="174"/>
+      <x:c r="B28" s="188"/>
+      <x:c r="C28" s="188"/>
+      <x:c r="D28" s="188"/>
+      <x:c r="E28" s="188"/>
+      <x:c r="F28" s="188"/>
+      <x:c r="G28" s="188"/>
+      <x:c r="H28" s="188"/>
+      <x:c r="I28" s="188"/>
+      <x:c r="J28" s="188"/>
+      <x:c r="K28" s="188"/>
+      <x:c r="L28" s="188"/>
+      <x:c r="M28" s="188"/>
+      <x:c r="N28" s="188"/>
+      <x:c r="O28" s="188"/>
+      <x:c r="P28" s="188"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="170" t="str">
+      <x:c r="A29" s="184" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B29" s="170" t="str">
+      <x:c r="B29" s="184" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C29" s="170" t="str">
+      <x:c r="C29" s="184" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D29" s="170" t="str">
+      <x:c r="D29" s="184" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E29" s="170" t="str">
+      <x:c r="E29" s="184" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F29" s="170" t="str">
+      <x:c r="F29" s="184" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G29" s="170" t="str">
+      <x:c r="G29" s="184" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H29" s="170" t="str">
+      <x:c r="H29" s="184" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I29" s="170" t="str">
+      <x:c r="I29" s="184" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J29" s="170" t="str">
+      <x:c r="J29" s="184" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K29" s="170" t="str">
+      <x:c r="K29" s="184" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L29" s="170" t="str">
+      <x:c r="L29" s="184" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M29" s="170" t="str">
+      <x:c r="M29" s="184" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N29" s="170" t="str">
+      <x:c r="N29" s="184" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O29" s="170" t="str">
+      <x:c r="O29" s="184" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P29" s="170" t="str">
+      <x:c r="P29" s="184" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4812,7 +4822,7 @@
       <x:c r="N30" s="100" t="str">
         <x:v>0 V / 약 5 V / 약 10 V</x:v>
       </x:c>
-      <x:c r="O30" s="172" t="str">
+      <x:c r="O30" s="186" t="str">
         <x:v>PASS (상대 선형성)</x:v>
       </x:c>
       <x:c r="P30" s="100" t="str">

</xml_diff>

<commit_message>
Remove fault-injection tests from bench scope
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re1bf95d1adfd4e7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R8953be38cb2e4817"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R3a5b6bfc62644572"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rf379f3416bbf4163"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R8e9e20bdafba407a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="Rb112bbe406b345bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R92685b5c69584f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R520d6fc0f8de4b26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="Rf510f0a7a7e64e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R8918c58f6e384c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R4584ea02a62440b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R5aa9754e99e64d6d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="60">
+  <x:fills count="66">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -450,7 +480,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="191">
+  <x:cellXfs count="200">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -874,6 +904,27 @@
     <x:xf numFmtId="0" fontId="3" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="57" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="62" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="60" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1076,7 +1127,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re707023819774079"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bc3df6faae5463a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1375,8 +1426,8 @@
         <x:v>총 시험 항목</x:v>
       </x:c>
       <x:c r="B6" s="17" t="n">
-        <x:f>COUNTA('Test Log'!A2:A201)</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTIF('Test Log'!Q6:Q20,"PASS")+COUNTIF('Test Log'!Q6:Q20,"FAIL")+COUNTIF('Test Log'!Q6:Q20,"INPUT")</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
         <x:v>카테고리별 결과</x:v>
@@ -1405,8 +1456,8 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
-        <x:f>COUNTIF('Test Log'!Q2:Q201,"PASS")</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIF('Test Log'!Q6:Q20,"PASS")</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>카테고리</x:v>
@@ -1426,7 +1477,7 @@
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="B8" s="17" t="n">
-        <x:f>COUNTIF('Test Log'!Q2:Q201,"FAIL")</x:f>
+        <x:f>COUNTIF('Test Log'!Q6:Q20,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
@@ -1450,8 +1501,8 @@
         <x:v>입력 대기</x:v>
       </x:c>
       <x:c r="B9" s="17" t="n">
-        <x:f>COUNTIF('Test Log'!Q2:Q201,"INPUT")+COUNTIF('Test Log'!Q2:Q201,"CHECK")</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTIF('Test Log'!Q6:Q20,"INPUT")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>계측 정확도</x:v>
@@ -1474,8 +1525,8 @@
         <x:v>합격률</x:v>
       </x:c>
       <x:c r="B10" s="18" t="n">
-        <x:f>IFERROR(B7/B6,0)</x:f>
-        <x:v>0.4375</x:v>
+        <x:f>IF(B6=0,0,B7/B6)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="26" t="str">
         <x:v>시간 성능</x:v>
@@ -1499,7 +1550,7 @@
       </x:c>
       <x:c r="E11" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F11" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
@@ -1507,7 +1558,7 @@
       </x:c>
       <x:c r="G11" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1524,7 +1575,7 @@
       </x:c>
       <x:c r="G12" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D12,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D12,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1541,7 +1592,7 @@
       </x:c>
       <x:c r="G13" s="25" t="n">
         <x:f>COUNTIFS('Test Log'!D$2:D$201,D13,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D13,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
@@ -1634,7 +1685,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9577d22f5ac749ce"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea2ae2fd7e3442f4"/>
 </x:worksheet>
 </file>
 
@@ -2033,164 +2084,64 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="55" t="str">
-        <x:v>R-01</x:v>
-      </x:c>
-      <x:c r="B16" s="55" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="C16" s="55" t="str">
-        <x:v>ADC DRDY 정지</x:v>
-      </x:c>
-      <x:c r="D16" s="55" t="str">
-        <x:v>MUTED 전이 시간</x:v>
-      </x:c>
-      <x:c r="E16" s="55" t="str">
-        <x:v>ms</x:v>
-      </x:c>
-      <x:c r="F16" s="56" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="G16" s="55" t="str">
-        <x:v>최대</x:v>
-      </x:c>
-      <x:c r="H16" s="55" t="str">
-        <x:v>signal disconnect/log</x:v>
-      </x:c>
-      <x:c r="I16" s="55" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="J16" s="55" t="str">
-        <x:v>safe output 확인</x:v>
-      </x:c>
+      <x:c r="A16" s="55"/>
+      <x:c r="B16" s="55"/>
+      <x:c r="C16" s="55"/>
+      <x:c r="D16" s="55"/>
+      <x:c r="E16" s="55"/>
+      <x:c r="F16" s="56"/>
+      <x:c r="G16" s="55"/>
+      <x:c r="H16" s="55"/>
+      <x:c r="I16" s="55"/>
+      <x:c r="J16" s="55"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="55" t="str">
-        <x:v>R-02</x:v>
-      </x:c>
-      <x:c r="B17" s="55" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="C17" s="55" t="str">
-        <x:v>SPI 장애</x:v>
-      </x:c>
-      <x:c r="D17" s="55" t="str">
-        <x:v>recovery 성공 시간</x:v>
-      </x:c>
-      <x:c r="E17" s="55" t="str">
-        <x:v>s</x:v>
-      </x:c>
-      <x:c r="F17" s="56" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G17" s="55" t="str">
-        <x:v>최대</x:v>
-      </x:c>
-      <x:c r="H17" s="55" t="str">
-        <x:v>fault injection</x:v>
-      </x:c>
-      <x:c r="I17" s="55" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="J17" s="55" t="str">
-        <x:v>backoff 포함</x:v>
-      </x:c>
+      <x:c r="A17" s="55"/>
+      <x:c r="B17" s="55"/>
+      <x:c r="C17" s="55"/>
+      <x:c r="D17" s="55"/>
+      <x:c r="E17" s="55"/>
+      <x:c r="F17" s="56"/>
+      <x:c r="G17" s="55"/>
+      <x:c r="H17" s="55"/>
+      <x:c r="I17" s="55"/>
+      <x:c r="J17" s="55"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="55" t="str">
-        <x:v>R-03</x:v>
-      </x:c>
-      <x:c r="B18" s="55" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="C18" s="55" t="str">
-        <x:v>DAC 통신 장애</x:v>
-      </x:c>
-      <x:c r="D18" s="55" t="str">
-        <x:v>DAC fault 전이</x:v>
-      </x:c>
-      <x:c r="E18" s="55" t="str">
-        <x:v>ms</x:v>
-      </x:c>
-      <x:c r="F18" s="56" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="G18" s="55" t="str">
-        <x:v>최대</x:v>
-      </x:c>
-      <x:c r="H18" s="55" t="str">
-        <x:v>fault injection</x:v>
-      </x:c>
-      <x:c r="I18" s="55" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="J18" s="55" t="str">
-        <x:v>출력 안전 상태 확인</x:v>
-      </x:c>
+      <x:c r="A18" s="55"/>
+      <x:c r="B18" s="55"/>
+      <x:c r="C18" s="55"/>
+      <x:c r="D18" s="55"/>
+      <x:c r="E18" s="55"/>
+      <x:c r="F18" s="56"/>
+      <x:c r="G18" s="55"/>
+      <x:c r="H18" s="55"/>
+      <x:c r="I18" s="55"/>
+      <x:c r="J18" s="55"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="55" t="str">
-        <x:v>R-04</x:v>
-      </x:c>
-      <x:c r="B19" s="55" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="C19" s="55" t="str">
-        <x:v>LAN 미연결</x:v>
-      </x:c>
-      <x:c r="D19" s="55" t="str">
-        <x:v>watchdog 재부팅 반복</x:v>
-      </x:c>
-      <x:c r="E19" s="55" t="str">
-        <x:v>count</x:v>
-      </x:c>
-      <x:c r="F19" s="56" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="55" t="str">
-        <x:v>일치</x:v>
-      </x:c>
-      <x:c r="H19" s="55" t="str">
-        <x:v>Ethernet unplug</x:v>
-      </x:c>
-      <x:c r="I19" s="55" t="str">
-        <x:v>P1</x:v>
-      </x:c>
-      <x:c r="J19" s="55" t="str">
-        <x:v>10분 관찰</x:v>
-      </x:c>
+      <x:c r="A19" s="55"/>
+      <x:c r="B19" s="55"/>
+      <x:c r="C19" s="55"/>
+      <x:c r="D19" s="55"/>
+      <x:c r="E19" s="55"/>
+      <x:c r="F19" s="56"/>
+      <x:c r="G19" s="55"/>
+      <x:c r="H19" s="55"/>
+      <x:c r="I19" s="55"/>
+      <x:c r="J19" s="55"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="55" t="str">
-        <x:v>L-01</x:v>
-      </x:c>
-      <x:c r="B20" s="55" t="str">
-        <x:v>장시간 안정성</x:v>
-      </x:c>
-      <x:c r="C20" s="55" t="str">
-        <x:v>Soak test</x:v>
-      </x:c>
-      <x:c r="D20" s="55" t="str">
-        <x:v>연속 동작 시간</x:v>
-      </x:c>
-      <x:c r="E20" s="55" t="str">
-        <x:v>h</x:v>
-      </x:c>
-      <x:c r="F20" s="56" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="G20" s="55" t="str">
-        <x:v>최소</x:v>
-      </x:c>
-      <x:c r="H20" s="55" t="str">
-        <x:v>24h logger</x:v>
-      </x:c>
-      <x:c r="I20" s="55" t="str">
-        <x:v>P1</x:v>
-      </x:c>
-      <x:c r="J20" s="55" t="str">
-        <x:v>reset/error/drop 기록</x:v>
-      </x:c>
+      <x:c r="A20" s="55"/>
+      <x:c r="B20" s="55"/>
+      <x:c r="C20" s="55"/>
+      <x:c r="D20" s="55"/>
+      <x:c r="E20" s="55"/>
+      <x:c r="F20" s="56"/>
+      <x:c r="G20" s="55"/>
+      <x:c r="H20" s="55"/>
+      <x:c r="I20" s="55"/>
+      <x:c r="J20" s="55"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2972,8 +2923,8 @@
         <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
       <x:c r="Q15" s="25" t="str">
-        <x:f>IF(OR(H15="",I15="",J15=""),"INPUT",IF(I15="최대",IF(J15&lt;=H15,"PASS","FAIL"),IF(I15="최소",IF(J15&gt;=H15,"PASS","FAIL"),IF(I15="일치",IF(J15=H15,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
+        <x:f>IF(J15&lt;=H15,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R15" s="57" t="str">
         <x:v>통과</x:v>
@@ -2989,29 +2940,15 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="25" t="str">
-        <x:v>R-01</x:v>
-      </x:c>
+      <x:c r="A16" s="25"/>
       <x:c r="B16" s="58"/>
       <x:c r="C16" s="57"/>
-      <x:c r="D16" s="25" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="E16" s="25" t="str">
-        <x:v>ADC DRDY 정지</x:v>
-      </x:c>
-      <x:c r="F16" s="25" t="str">
-        <x:v>MUTED 전이 시간</x:v>
-      </x:c>
-      <x:c r="G16" s="25" t="str">
-        <x:v>ms</x:v>
-      </x:c>
-      <x:c r="H16" s="59" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="I16" s="59" t="str">
-        <x:v>최대</x:v>
-      </x:c>
+      <x:c r="D16" s="25"/>
+      <x:c r="E16" s="25"/>
+      <x:c r="F16" s="25"/>
+      <x:c r="G16" s="25"/>
+      <x:c r="H16" s="59"/>
+      <x:c r="I16" s="59"/>
       <x:c r="J16" s="60"/>
       <x:c r="K16" s="60"/>
       <x:c r="L16" s="60"/>
@@ -3019,43 +2956,22 @@
       <x:c r="N16" s="60"/>
       <x:c r="O16" s="60"/>
       <x:c r="P16" s="57"/>
-      <x:c r="Q16" s="25" t="str">
-        <x:f>IF(OR(H16="",I16="",J16=""),"INPUT",IF(I16="최대",IF(J16&lt;=H16,"PASS","FAIL"),IF(I16="최소",IF(J16&gt;=H16,"PASS","FAIL"),IF(I16="일치",IF(J16=H16,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
-      </x:c>
-      <x:c r="R16" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
+      <x:c r="Q16" s="25"/>
+      <x:c r="R16" s="57"/>
       <x:c r="S16" s="57"/>
-      <x:c r="T16" s="57" t="str">
-        <x:v>safe output 확인</x:v>
-      </x:c>
+      <x:c r="T16" s="57"/>
       <x:c r="U16" s="57"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="25" t="str">
-        <x:v>R-02</x:v>
-      </x:c>
+      <x:c r="A17" s="25"/>
       <x:c r="B17" s="58"/>
       <x:c r="C17" s="57"/>
-      <x:c r="D17" s="25" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="E17" s="25" t="str">
-        <x:v>SPI 장애</x:v>
-      </x:c>
-      <x:c r="F17" s="25" t="str">
-        <x:v>recovery 성공 시간</x:v>
-      </x:c>
-      <x:c r="G17" s="25" t="str">
-        <x:v>s</x:v>
-      </x:c>
-      <x:c r="H17" s="59" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I17" s="59" t="str">
-        <x:v>최대</x:v>
-      </x:c>
+      <x:c r="D17" s="25"/>
+      <x:c r="E17" s="25"/>
+      <x:c r="F17" s="25"/>
+      <x:c r="G17" s="25"/>
+      <x:c r="H17" s="59"/>
+      <x:c r="I17" s="59"/>
       <x:c r="J17" s="60"/>
       <x:c r="K17" s="60"/>
       <x:c r="L17" s="60"/>
@@ -3063,43 +2979,22 @@
       <x:c r="N17" s="60"/>
       <x:c r="O17" s="60"/>
       <x:c r="P17" s="57"/>
-      <x:c r="Q17" s="25" t="str">
-        <x:f>IF(OR(H17="",I17="",J17=""),"INPUT",IF(I17="최대",IF(J17&lt;=H17,"PASS","FAIL"),IF(I17="최소",IF(J17&gt;=H17,"PASS","FAIL"),IF(I17="일치",IF(J17=H17,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
-      </x:c>
-      <x:c r="R17" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
+      <x:c r="Q17" s="25"/>
+      <x:c r="R17" s="57"/>
       <x:c r="S17" s="57"/>
-      <x:c r="T17" s="57" t="str">
-        <x:v>backoff 포함</x:v>
-      </x:c>
+      <x:c r="T17" s="57"/>
       <x:c r="U17" s="57"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="25" t="str">
-        <x:v>R-03</x:v>
-      </x:c>
+      <x:c r="A18" s="25"/>
       <x:c r="B18" s="58"/>
       <x:c r="C18" s="57"/>
-      <x:c r="D18" s="25" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="E18" s="25" t="str">
-        <x:v>DAC 통신 장애</x:v>
-      </x:c>
-      <x:c r="F18" s="25" t="str">
-        <x:v>DAC fault 전이</x:v>
-      </x:c>
-      <x:c r="G18" s="25" t="str">
-        <x:v>ms</x:v>
-      </x:c>
-      <x:c r="H18" s="59" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="I18" s="59" t="str">
-        <x:v>최대</x:v>
-      </x:c>
+      <x:c r="D18" s="25"/>
+      <x:c r="E18" s="25"/>
+      <x:c r="F18" s="25"/>
+      <x:c r="G18" s="25"/>
+      <x:c r="H18" s="59"/>
+      <x:c r="I18" s="59"/>
       <x:c r="J18" s="60"/>
       <x:c r="K18" s="60"/>
       <x:c r="L18" s="60"/>
@@ -3107,43 +3002,22 @@
       <x:c r="N18" s="60"/>
       <x:c r="O18" s="60"/>
       <x:c r="P18" s="57"/>
-      <x:c r="Q18" s="25" t="str">
-        <x:f>IF(OR(H18="",I18="",J18=""),"INPUT",IF(I18="최대",IF(J18&lt;=H18,"PASS","FAIL"),IF(I18="최소",IF(J18&gt;=H18,"PASS","FAIL"),IF(I18="일치",IF(J18=H18,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
-      </x:c>
-      <x:c r="R18" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
+      <x:c r="Q18" s="25"/>
+      <x:c r="R18" s="57"/>
       <x:c r="S18" s="57"/>
-      <x:c r="T18" s="57" t="str">
-        <x:v>출력 안전 상태 확인</x:v>
-      </x:c>
+      <x:c r="T18" s="57"/>
       <x:c r="U18" s="57"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="25" t="str">
-        <x:v>R-04</x:v>
-      </x:c>
+      <x:c r="A19" s="25"/>
       <x:c r="B19" s="58"/>
       <x:c r="C19" s="57"/>
-      <x:c r="D19" s="25" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="E19" s="25" t="str">
-        <x:v>LAN 미연결</x:v>
-      </x:c>
-      <x:c r="F19" s="25" t="str">
-        <x:v>watchdog 재부팅 반복</x:v>
-      </x:c>
-      <x:c r="G19" s="25" t="str">
-        <x:v>count</x:v>
-      </x:c>
-      <x:c r="H19" s="59" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I19" s="59" t="str">
-        <x:v>일치</x:v>
-      </x:c>
+      <x:c r="D19" s="25"/>
+      <x:c r="E19" s="25"/>
+      <x:c r="F19" s="25"/>
+      <x:c r="G19" s="25"/>
+      <x:c r="H19" s="59"/>
+      <x:c r="I19" s="59"/>
       <x:c r="J19" s="60"/>
       <x:c r="K19" s="60"/>
       <x:c r="L19" s="60"/>
@@ -3151,43 +3025,22 @@
       <x:c r="N19" s="60"/>
       <x:c r="O19" s="60"/>
       <x:c r="P19" s="57"/>
-      <x:c r="Q19" s="25" t="str">
-        <x:f>IF(OR(H19="",I19="",J19=""),"INPUT",IF(I19="최대",IF(J19&lt;=H19,"PASS","FAIL"),IF(I19="최소",IF(J19&gt;=H19,"PASS","FAIL"),IF(I19="일치",IF(J19=H19,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
-      </x:c>
-      <x:c r="R19" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
+      <x:c r="Q19" s="25"/>
+      <x:c r="R19" s="57"/>
       <x:c r="S19" s="57"/>
-      <x:c r="T19" s="57" t="str">
-        <x:v>10분 관찰</x:v>
-      </x:c>
+      <x:c r="T19" s="57"/>
       <x:c r="U19" s="57"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="25" t="str">
-        <x:v>L-01</x:v>
-      </x:c>
+      <x:c r="A20" s="25"/>
       <x:c r="B20" s="58"/>
       <x:c r="C20" s="57"/>
-      <x:c r="D20" s="25" t="str">
-        <x:v>장시간 안정성</x:v>
-      </x:c>
-      <x:c r="E20" s="25" t="str">
-        <x:v>Soak test</x:v>
-      </x:c>
-      <x:c r="F20" s="25" t="str">
-        <x:v>연속 동작 시간</x:v>
-      </x:c>
-      <x:c r="G20" s="25" t="str">
-        <x:v>h</x:v>
-      </x:c>
-      <x:c r="H20" s="59" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="I20" s="59" t="str">
-        <x:v>최소</x:v>
-      </x:c>
+      <x:c r="D20" s="25"/>
+      <x:c r="E20" s="25"/>
+      <x:c r="F20" s="25"/>
+      <x:c r="G20" s="25"/>
+      <x:c r="H20" s="59"/>
+      <x:c r="I20" s="59"/>
       <x:c r="J20" s="60"/>
       <x:c r="K20" s="60"/>
       <x:c r="L20" s="60"/>
@@ -3195,17 +3048,10 @@
       <x:c r="N20" s="60"/>
       <x:c r="O20" s="60"/>
       <x:c r="P20" s="57"/>
-      <x:c r="Q20" s="25" t="str">
-        <x:f>IF(OR(H20="",I20="",J20=""),"INPUT",IF(I20="최대",IF(J20&lt;=H20,"PASS","FAIL"),IF(I20="최소",IF(J20&gt;=H20,"PASS","FAIL"),IF(I20="일치",IF(J20=H20,"PASS","FAIL"),"CHECK"))))</x:f>
-        <x:v>INPUT</x:v>
-      </x:c>
-      <x:c r="R20" s="57" t="str">
-        <x:v>미실행</x:v>
-      </x:c>
+      <x:c r="Q20" s="25"/>
+      <x:c r="R20" s="57"/>
       <x:c r="S20" s="57"/>
-      <x:c r="T20" s="57" t="str">
-        <x:v>reset/error/drop 기록</x:v>
-      </x:c>
+      <x:c r="T20" s="57"/>
       <x:c r="U20" s="57"/>
     </x:row>
   </x:sheetData>
@@ -4058,92 +3904,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="182" t="str">
+      <x:c r="A1" s="191" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="182"/>
-      <x:c r="C1" s="182"/>
-      <x:c r="D1" s="182"/>
-      <x:c r="E1" s="182"/>
-      <x:c r="F1" s="182"/>
-      <x:c r="G1" s="182"/>
-      <x:c r="H1" s="182"/>
-      <x:c r="I1" s="182"/>
-      <x:c r="J1" s="182"/>
-      <x:c r="K1" s="182"/>
-      <x:c r="L1" s="182"/>
-      <x:c r="M1" s="182"/>
-      <x:c r="N1" s="182"/>
-      <x:c r="O1" s="182"/>
-      <x:c r="P1" s="182"/>
+      <x:c r="B1" s="191"/>
+      <x:c r="C1" s="191"/>
+      <x:c r="D1" s="191"/>
+      <x:c r="E1" s="191"/>
+      <x:c r="F1" s="191"/>
+      <x:c r="G1" s="191"/>
+      <x:c r="H1" s="191"/>
+      <x:c r="I1" s="191"/>
+      <x:c r="J1" s="191"/>
+      <x:c r="K1" s="191"/>
+      <x:c r="L1" s="191"/>
+      <x:c r="M1" s="191"/>
+      <x:c r="N1" s="191"/>
+      <x:c r="O1" s="191"/>
+      <x:c r="P1" s="191"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="183" t="str">
+      <x:c r="A3" s="192" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="183"/>
-      <x:c r="C3" s="183"/>
-      <x:c r="D3" s="183"/>
-      <x:c r="E3" s="183"/>
-      <x:c r="F3" s="183"/>
-      <x:c r="G3" s="183"/>
-      <x:c r="H3" s="183"/>
-      <x:c r="I3" s="183"/>
-      <x:c r="J3" s="183"/>
-      <x:c r="K3" s="183"/>
-      <x:c r="L3" s="183"/>
-      <x:c r="M3" s="183"/>
-      <x:c r="N3" s="183"/>
-      <x:c r="O3" s="183"/>
-      <x:c r="P3" s="183"/>
+      <x:c r="B3" s="192"/>
+      <x:c r="C3" s="192"/>
+      <x:c r="D3" s="192"/>
+      <x:c r="E3" s="192"/>
+      <x:c r="F3" s="192"/>
+      <x:c r="G3" s="192"/>
+      <x:c r="H3" s="192"/>
+      <x:c r="I3" s="192"/>
+      <x:c r="J3" s="192"/>
+      <x:c r="K3" s="192"/>
+      <x:c r="L3" s="192"/>
+      <x:c r="M3" s="192"/>
+      <x:c r="N3" s="192"/>
+      <x:c r="O3" s="192"/>
+      <x:c r="P3" s="192"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="184" t="str">
+      <x:c r="A5" s="193" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="184" t="str">
+      <x:c r="B5" s="193" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="184" t="str">
+      <x:c r="C5" s="193" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="184" t="str">
+      <x:c r="D5" s="193" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="184" t="str">
+      <x:c r="E5" s="193" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="184" t="str">
+      <x:c r="F5" s="193" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="184" t="str">
+      <x:c r="G5" s="193" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="184" t="str">
+      <x:c r="H5" s="193" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="184" t="str">
+      <x:c r="I5" s="193" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="184" t="str">
+      <x:c r="J5" s="193" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="184" t="str">
+      <x:c r="K5" s="193" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="184" t="str">
+      <x:c r="L5" s="193" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="184" t="str">
+      <x:c r="M5" s="193" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="184" t="str">
+      <x:c r="N5" s="193" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="184" t="str">
+      <x:c r="O5" s="193" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="184" t="str">
+      <x:c r="P5" s="193" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4190,7 +4036,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="185" t="str">
+      <x:c r="O6" s="194" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -4240,7 +4086,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="186" t="str">
+      <x:c r="O7" s="195" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -4286,7 +4132,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="187" t="str">
+      <x:c r="O8" s="196" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4336,7 +4182,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="186" t="str">
+      <x:c r="O9" s="195" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4386,7 +4232,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="186" t="str">
+      <x:c r="O10" s="195" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4394,36 +4240,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="188" t="str">
+      <x:c r="A11" s="197" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="188"/>
-      <x:c r="C11" s="188"/>
-      <x:c r="D11" s="188"/>
-      <x:c r="E11" s="188"/>
-      <x:c r="F11" s="188"/>
-      <x:c r="G11" s="188"/>
-      <x:c r="H11" s="188"/>
-      <x:c r="I11" s="188"/>
-      <x:c r="J11" s="188"/>
-      <x:c r="K11" s="188"/>
-      <x:c r="L11" s="188"/>
-      <x:c r="M11" s="188"/>
-      <x:c r="N11" s="188"/>
-      <x:c r="O11" s="188"/>
-      <x:c r="P11" s="188"/>
+      <x:c r="B11" s="197"/>
+      <x:c r="C11" s="197"/>
+      <x:c r="D11" s="197"/>
+      <x:c r="E11" s="197"/>
+      <x:c r="F11" s="197"/>
+      <x:c r="G11" s="197"/>
+      <x:c r="H11" s="197"/>
+      <x:c r="I11" s="197"/>
+      <x:c r="J11" s="197"/>
+      <x:c r="K11" s="197"/>
+      <x:c r="L11" s="197"/>
+      <x:c r="M11" s="197"/>
+      <x:c r="N11" s="197"/>
+      <x:c r="O11" s="197"/>
+      <x:c r="P11" s="197"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="189" t="str">
+      <x:c r="A12" s="198" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="189" t="str">
+      <x:c r="B12" s="198" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="189" t="str">
+      <x:c r="C12" s="198" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="189" t="str">
+      <x:c r="D12" s="198" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4437,7 +4283,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="190" t="str">
+      <x:c r="D13" s="199" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4451,7 +4297,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="190" t="str">
+      <x:c r="D14" s="199" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4465,47 +4311,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="190" t="str">
+      <x:c r="D15" s="199" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="188" t="str">
+      <x:c r="A17" s="197" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="188"/>
-      <x:c r="C17" s="188"/>
-      <x:c r="D17" s="188"/>
-      <x:c r="E17" s="188"/>
-      <x:c r="F17" s="188"/>
-      <x:c r="G17" s="188"/>
-      <x:c r="H17" s="188"/>
-      <x:c r="I17" s="188"/>
-      <x:c r="J17" s="188"/>
-      <x:c r="K17" s="188"/>
-      <x:c r="L17" s="188"/>
-      <x:c r="M17" s="188"/>
-      <x:c r="N17" s="188"/>
-      <x:c r="O17" s="188"/>
-      <x:c r="P17" s="188"/>
+      <x:c r="B17" s="197"/>
+      <x:c r="C17" s="197"/>
+      <x:c r="D17" s="197"/>
+      <x:c r="E17" s="197"/>
+      <x:c r="F17" s="197"/>
+      <x:c r="G17" s="197"/>
+      <x:c r="H17" s="197"/>
+      <x:c r="I17" s="197"/>
+      <x:c r="J17" s="197"/>
+      <x:c r="K17" s="197"/>
+      <x:c r="L17" s="197"/>
+      <x:c r="M17" s="197"/>
+      <x:c r="N17" s="197"/>
+      <x:c r="O17" s="197"/>
+      <x:c r="P17" s="197"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="189" t="str">
+      <x:c r="A18" s="198" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="189" t="str">
+      <x:c r="B18" s="198" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="189" t="str">
+      <x:c r="C18" s="198" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="189" t="str">
+      <x:c r="D18" s="198" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="189" t="str">
+      <x:c r="E18" s="198" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="189" t="str">
+      <x:c r="F18" s="198" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4590,72 +4436,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="188" t="str">
+      <x:c r="A24" s="197" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="188"/>
-      <x:c r="C24" s="188"/>
-      <x:c r="D24" s="188"/>
-      <x:c r="E24" s="188"/>
-      <x:c r="F24" s="188"/>
-      <x:c r="G24" s="188"/>
-      <x:c r="H24" s="188"/>
-      <x:c r="I24" s="188"/>
-      <x:c r="J24" s="188"/>
-      <x:c r="K24" s="188"/>
-      <x:c r="L24" s="188"/>
-      <x:c r="M24" s="188"/>
-      <x:c r="N24" s="188"/>
-      <x:c r="O24" s="188"/>
-      <x:c r="P24" s="188"/>
+      <x:c r="B24" s="197"/>
+      <x:c r="C24" s="197"/>
+      <x:c r="D24" s="197"/>
+      <x:c r="E24" s="197"/>
+      <x:c r="F24" s="197"/>
+      <x:c r="G24" s="197"/>
+      <x:c r="H24" s="197"/>
+      <x:c r="I24" s="197"/>
+      <x:c r="J24" s="197"/>
+      <x:c r="K24" s="197"/>
+      <x:c r="L24" s="197"/>
+      <x:c r="M24" s="197"/>
+      <x:c r="N24" s="197"/>
+      <x:c r="O24" s="197"/>
+      <x:c r="P24" s="197"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="184" t="str">
+      <x:c r="A25" s="193" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="184" t="str">
+      <x:c r="B25" s="193" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="184" t="str">
+      <x:c r="C25" s="193" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="184" t="str">
+      <x:c r="D25" s="193" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="184" t="str">
+      <x:c r="E25" s="193" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="184" t="str">
+      <x:c r="F25" s="193" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="184" t="str">
+      <x:c r="G25" s="193" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="184" t="str">
+      <x:c r="H25" s="193" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="184" t="str">
+      <x:c r="I25" s="193" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="184" t="str">
+      <x:c r="J25" s="193" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="184" t="str">
+      <x:c r="K25" s="193" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="184" t="str">
+      <x:c r="L25" s="193" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="184" t="str">
+      <x:c r="M25" s="193" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="184" t="str">
+      <x:c r="N25" s="193" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="184" t="str">
+      <x:c r="O25" s="193" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="184" t="str">
+      <x:c r="P25" s="193" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4702,7 +4548,7 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="186" t="str">
+      <x:c r="O26" s="195" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">
@@ -4710,72 +4556,72 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="188" t="str">
+      <x:c r="A28" s="197" t="str">
         <x:v>추가 캡처: 3점 상대 선형성 시험</x:v>
       </x:c>
-      <x:c r="B28" s="188"/>
-      <x:c r="C28" s="188"/>
-      <x:c r="D28" s="188"/>
-      <x:c r="E28" s="188"/>
-      <x:c r="F28" s="188"/>
-      <x:c r="G28" s="188"/>
-      <x:c r="H28" s="188"/>
-      <x:c r="I28" s="188"/>
-      <x:c r="J28" s="188"/>
-      <x:c r="K28" s="188"/>
-      <x:c r="L28" s="188"/>
-      <x:c r="M28" s="188"/>
-      <x:c r="N28" s="188"/>
-      <x:c r="O28" s="188"/>
-      <x:c r="P28" s="188"/>
+      <x:c r="B28" s="197"/>
+      <x:c r="C28" s="197"/>
+      <x:c r="D28" s="197"/>
+      <x:c r="E28" s="197"/>
+      <x:c r="F28" s="197"/>
+      <x:c r="G28" s="197"/>
+      <x:c r="H28" s="197"/>
+      <x:c r="I28" s="197"/>
+      <x:c r="J28" s="197"/>
+      <x:c r="K28" s="197"/>
+      <x:c r="L28" s="197"/>
+      <x:c r="M28" s="197"/>
+      <x:c r="N28" s="197"/>
+      <x:c r="O28" s="197"/>
+      <x:c r="P28" s="197"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="184" t="str">
+      <x:c r="A29" s="193" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B29" s="184" t="str">
+      <x:c r="B29" s="193" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C29" s="184" t="str">
+      <x:c r="C29" s="193" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D29" s="184" t="str">
+      <x:c r="D29" s="193" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E29" s="184" t="str">
+      <x:c r="E29" s="193" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F29" s="184" t="str">
+      <x:c r="F29" s="193" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G29" s="184" t="str">
+      <x:c r="G29" s="193" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H29" s="184" t="str">
+      <x:c r="H29" s="193" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I29" s="184" t="str">
+      <x:c r="I29" s="193" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J29" s="184" t="str">
+      <x:c r="J29" s="193" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K29" s="184" t="str">
+      <x:c r="K29" s="193" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L29" s="184" t="str">
+      <x:c r="L29" s="193" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M29" s="184" t="str">
+      <x:c r="M29" s="193" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N29" s="184" t="str">
+      <x:c r="N29" s="193" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O29" s="184" t="str">
+      <x:c r="O29" s="193" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P29" s="184" t="str">
+      <x:c r="P29" s="193" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4822,7 +4668,7 @@
       <x:c r="N30" s="100" t="str">
         <x:v>0 V / 약 5 V / 약 10 V</x:v>
       </x:c>
-      <x:c r="O30" s="186" t="str">
+      <x:c r="O30" s="195" t="str">
         <x:v>PASS (상대 선형성)</x:v>
       </x:c>
       <x:c r="P30" s="100" t="str">

</xml_diff>

<commit_message>
Record thermal observation from load test
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R92685b5c69584f1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R520d6fc0f8de4b26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="Rf510f0a7a7e64e99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R8918c58f6e384c5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R4584ea02a62440b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R5aa9754e99e64d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6b76e2f56e304f4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R84eb57ead8f0401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R66b8697567d34d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rb25b39fb71a049f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Re4085fb988964699"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R871964fc51df43d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,13 +18,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="203" formatCode="0.000"/>
     <x:numFmt numFmtId="204" formatCode="#,##0"/>
     <x:numFmt numFmtId="205" formatCode="0.000000"/>
+    <x:numFmt numFmtId="206" formatCode="0.0"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -66,7 +67,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="66">
+  <x:fills count="72">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +122,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -480,7 +511,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="200">
+  <x:cellXfs count="216">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -925,6 +956,42 @@
     <x:xf numFmtId="0" fontId="3" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="60" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="63" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="68" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="70" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="69" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1127,7 +1194,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bc3df6faae5463a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcecc59c84ff74988"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1685,7 +1752,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea2ae2fd7e3442f4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a1181120e654137"/>
 </x:worksheet>
 </file>
 
@@ -3904,92 +3971,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="191" t="str">
+      <x:c r="A1" s="200" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="191"/>
-      <x:c r="C1" s="191"/>
-      <x:c r="D1" s="191"/>
-      <x:c r="E1" s="191"/>
-      <x:c r="F1" s="191"/>
-      <x:c r="G1" s="191"/>
-      <x:c r="H1" s="191"/>
-      <x:c r="I1" s="191"/>
-      <x:c r="J1" s="191"/>
-      <x:c r="K1" s="191"/>
-      <x:c r="L1" s="191"/>
-      <x:c r="M1" s="191"/>
-      <x:c r="N1" s="191"/>
-      <x:c r="O1" s="191"/>
-      <x:c r="P1" s="191"/>
+      <x:c r="B1" s="200"/>
+      <x:c r="C1" s="200"/>
+      <x:c r="D1" s="200"/>
+      <x:c r="E1" s="200"/>
+      <x:c r="F1" s="200"/>
+      <x:c r="G1" s="200"/>
+      <x:c r="H1" s="200"/>
+      <x:c r="I1" s="200"/>
+      <x:c r="J1" s="200"/>
+      <x:c r="K1" s="200"/>
+      <x:c r="L1" s="200"/>
+      <x:c r="M1" s="200"/>
+      <x:c r="N1" s="200"/>
+      <x:c r="O1" s="200"/>
+      <x:c r="P1" s="200"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="192" t="str">
+      <x:c r="A3" s="201" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="192"/>
-      <x:c r="C3" s="192"/>
-      <x:c r="D3" s="192"/>
-      <x:c r="E3" s="192"/>
-      <x:c r="F3" s="192"/>
-      <x:c r="G3" s="192"/>
-      <x:c r="H3" s="192"/>
-      <x:c r="I3" s="192"/>
-      <x:c r="J3" s="192"/>
-      <x:c r="K3" s="192"/>
-      <x:c r="L3" s="192"/>
-      <x:c r="M3" s="192"/>
-      <x:c r="N3" s="192"/>
-      <x:c r="O3" s="192"/>
-      <x:c r="P3" s="192"/>
+      <x:c r="B3" s="201"/>
+      <x:c r="C3" s="201"/>
+      <x:c r="D3" s="201"/>
+      <x:c r="E3" s="201"/>
+      <x:c r="F3" s="201"/>
+      <x:c r="G3" s="201"/>
+      <x:c r="H3" s="201"/>
+      <x:c r="I3" s="201"/>
+      <x:c r="J3" s="201"/>
+      <x:c r="K3" s="201"/>
+      <x:c r="L3" s="201"/>
+      <x:c r="M3" s="201"/>
+      <x:c r="N3" s="201"/>
+      <x:c r="O3" s="201"/>
+      <x:c r="P3" s="201"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="193" t="str">
+      <x:c r="A5" s="202" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="193" t="str">
+      <x:c r="B5" s="202" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="193" t="str">
+      <x:c r="C5" s="202" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="193" t="str">
+      <x:c r="D5" s="202" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="193" t="str">
+      <x:c r="E5" s="202" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="193" t="str">
+      <x:c r="F5" s="202" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="193" t="str">
+      <x:c r="G5" s="202" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="193" t="str">
+      <x:c r="H5" s="202" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="193" t="str">
+      <x:c r="I5" s="202" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="193" t="str">
+      <x:c r="J5" s="202" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="193" t="str">
+      <x:c r="K5" s="202" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="193" t="str">
+      <x:c r="L5" s="202" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="193" t="str">
+      <x:c r="M5" s="202" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="193" t="str">
+      <x:c r="N5" s="202" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="193" t="str">
+      <x:c r="O5" s="202" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="193" t="str">
+      <x:c r="P5" s="202" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4036,7 +4103,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="194" t="str">
+      <x:c r="O6" s="203" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -4086,7 +4153,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="195" t="str">
+      <x:c r="O7" s="204" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -4132,7 +4199,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="196" t="str">
+      <x:c r="O8" s="205" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4182,7 +4249,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="195" t="str">
+      <x:c r="O9" s="204" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4232,7 +4299,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="195" t="str">
+      <x:c r="O10" s="204" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4240,36 +4307,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="197" t="str">
+      <x:c r="A11" s="206" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="197"/>
-      <x:c r="C11" s="197"/>
-      <x:c r="D11" s="197"/>
-      <x:c r="E11" s="197"/>
-      <x:c r="F11" s="197"/>
-      <x:c r="G11" s="197"/>
-      <x:c r="H11" s="197"/>
-      <x:c r="I11" s="197"/>
-      <x:c r="J11" s="197"/>
-      <x:c r="K11" s="197"/>
-      <x:c r="L11" s="197"/>
-      <x:c r="M11" s="197"/>
-      <x:c r="N11" s="197"/>
-      <x:c r="O11" s="197"/>
-      <x:c r="P11" s="197"/>
+      <x:c r="B11" s="206"/>
+      <x:c r="C11" s="206"/>
+      <x:c r="D11" s="206"/>
+      <x:c r="E11" s="206"/>
+      <x:c r="F11" s="206"/>
+      <x:c r="G11" s="206"/>
+      <x:c r="H11" s="206"/>
+      <x:c r="I11" s="206"/>
+      <x:c r="J11" s="206"/>
+      <x:c r="K11" s="206"/>
+      <x:c r="L11" s="206"/>
+      <x:c r="M11" s="206"/>
+      <x:c r="N11" s="206"/>
+      <x:c r="O11" s="206"/>
+      <x:c r="P11" s="206"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="198" t="str">
+      <x:c r="A12" s="207" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="198" t="str">
+      <x:c r="B12" s="207" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="198" t="str">
+      <x:c r="C12" s="207" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="198" t="str">
+      <x:c r="D12" s="207" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4283,7 +4350,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="199" t="str">
+      <x:c r="D13" s="208" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4297,7 +4364,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="199" t="str">
+      <x:c r="D14" s="208" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4311,47 +4378,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="199" t="str">
+      <x:c r="D15" s="208" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="197" t="str">
+      <x:c r="A17" s="206" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="197"/>
-      <x:c r="C17" s="197"/>
-      <x:c r="D17" s="197"/>
-      <x:c r="E17" s="197"/>
-      <x:c r="F17" s="197"/>
-      <x:c r="G17" s="197"/>
-      <x:c r="H17" s="197"/>
-      <x:c r="I17" s="197"/>
-      <x:c r="J17" s="197"/>
-      <x:c r="K17" s="197"/>
-      <x:c r="L17" s="197"/>
-      <x:c r="M17" s="197"/>
-      <x:c r="N17" s="197"/>
-      <x:c r="O17" s="197"/>
-      <x:c r="P17" s="197"/>
+      <x:c r="B17" s="206"/>
+      <x:c r="C17" s="206"/>
+      <x:c r="D17" s="206"/>
+      <x:c r="E17" s="206"/>
+      <x:c r="F17" s="206"/>
+      <x:c r="G17" s="206"/>
+      <x:c r="H17" s="206"/>
+      <x:c r="I17" s="206"/>
+      <x:c r="J17" s="206"/>
+      <x:c r="K17" s="206"/>
+      <x:c r="L17" s="206"/>
+      <x:c r="M17" s="206"/>
+      <x:c r="N17" s="206"/>
+      <x:c r="O17" s="206"/>
+      <x:c r="P17" s="206"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="198" t="str">
+      <x:c r="A18" s="207" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="198" t="str">
+      <x:c r="B18" s="207" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="198" t="str">
+      <x:c r="C18" s="207" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="198" t="str">
+      <x:c r="D18" s="207" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="198" t="str">
+      <x:c r="E18" s="207" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="198" t="str">
+      <x:c r="F18" s="207" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4436,72 +4503,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="197" t="str">
+      <x:c r="A24" s="206" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="197"/>
-      <x:c r="C24" s="197"/>
-      <x:c r="D24" s="197"/>
-      <x:c r="E24" s="197"/>
-      <x:c r="F24" s="197"/>
-      <x:c r="G24" s="197"/>
-      <x:c r="H24" s="197"/>
-      <x:c r="I24" s="197"/>
-      <x:c r="J24" s="197"/>
-      <x:c r="K24" s="197"/>
-      <x:c r="L24" s="197"/>
-      <x:c r="M24" s="197"/>
-      <x:c r="N24" s="197"/>
-      <x:c r="O24" s="197"/>
-      <x:c r="P24" s="197"/>
+      <x:c r="B24" s="206"/>
+      <x:c r="C24" s="206"/>
+      <x:c r="D24" s="206"/>
+      <x:c r="E24" s="206"/>
+      <x:c r="F24" s="206"/>
+      <x:c r="G24" s="206"/>
+      <x:c r="H24" s="206"/>
+      <x:c r="I24" s="206"/>
+      <x:c r="J24" s="206"/>
+      <x:c r="K24" s="206"/>
+      <x:c r="L24" s="206"/>
+      <x:c r="M24" s="206"/>
+      <x:c r="N24" s="206"/>
+      <x:c r="O24" s="206"/>
+      <x:c r="P24" s="206"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="193" t="str">
+      <x:c r="A25" s="202" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="193" t="str">
+      <x:c r="B25" s="202" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="193" t="str">
+      <x:c r="C25" s="202" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="193" t="str">
+      <x:c r="D25" s="202" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="193" t="str">
+      <x:c r="E25" s="202" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="193" t="str">
+      <x:c r="F25" s="202" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="193" t="str">
+      <x:c r="G25" s="202" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="193" t="str">
+      <x:c r="H25" s="202" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="193" t="str">
+      <x:c r="I25" s="202" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="193" t="str">
+      <x:c r="J25" s="202" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="193" t="str">
+      <x:c r="K25" s="202" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="193" t="str">
+      <x:c r="L25" s="202" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="193" t="str">
+      <x:c r="M25" s="202" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="193" t="str">
+      <x:c r="N25" s="202" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="193" t="str">
+      <x:c r="O25" s="202" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="193" t="str">
+      <x:c r="P25" s="202" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4548,7 +4615,7 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="195" t="str">
+      <x:c r="O26" s="204" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">
@@ -4556,72 +4623,72 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="197" t="str">
+      <x:c r="A28" s="206" t="str">
         <x:v>추가 캡처: 3점 상대 선형성 시험</x:v>
       </x:c>
-      <x:c r="B28" s="197"/>
-      <x:c r="C28" s="197"/>
-      <x:c r="D28" s="197"/>
-      <x:c r="E28" s="197"/>
-      <x:c r="F28" s="197"/>
-      <x:c r="G28" s="197"/>
-      <x:c r="H28" s="197"/>
-      <x:c r="I28" s="197"/>
-      <x:c r="J28" s="197"/>
-      <x:c r="K28" s="197"/>
-      <x:c r="L28" s="197"/>
-      <x:c r="M28" s="197"/>
-      <x:c r="N28" s="197"/>
-      <x:c r="O28" s="197"/>
-      <x:c r="P28" s="197"/>
+      <x:c r="B28" s="206"/>
+      <x:c r="C28" s="206"/>
+      <x:c r="D28" s="206"/>
+      <x:c r="E28" s="206"/>
+      <x:c r="F28" s="206"/>
+      <x:c r="G28" s="206"/>
+      <x:c r="H28" s="206"/>
+      <x:c r="I28" s="206"/>
+      <x:c r="J28" s="206"/>
+      <x:c r="K28" s="206"/>
+      <x:c r="L28" s="206"/>
+      <x:c r="M28" s="206"/>
+      <x:c r="N28" s="206"/>
+      <x:c r="O28" s="206"/>
+      <x:c r="P28" s="206"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="193" t="str">
+      <x:c r="A29" s="202" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B29" s="193" t="str">
+      <x:c r="B29" s="202" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C29" s="193" t="str">
+      <x:c r="C29" s="202" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D29" s="193" t="str">
+      <x:c r="D29" s="202" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E29" s="193" t="str">
+      <x:c r="E29" s="202" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F29" s="193" t="str">
+      <x:c r="F29" s="202" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G29" s="193" t="str">
+      <x:c r="G29" s="202" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H29" s="193" t="str">
+      <x:c r="H29" s="202" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I29" s="193" t="str">
+      <x:c r="I29" s="202" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J29" s="193" t="str">
+      <x:c r="J29" s="202" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K29" s="193" t="str">
+      <x:c r="K29" s="202" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L29" s="193" t="str">
+      <x:c r="L29" s="202" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M29" s="193" t="str">
+      <x:c r="M29" s="202" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N29" s="193" t="str">
+      <x:c r="N29" s="202" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O29" s="193" t="str">
+      <x:c r="O29" s="202" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P29" s="193" t="str">
+      <x:c r="P29" s="202" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4668,11 +4735,123 @@
       <x:c r="N30" s="100" t="str">
         <x:v>0 V / 약 5 V / 약 10 V</x:v>
       </x:c>
-      <x:c r="O30" s="195" t="str">
+      <x:c r="O30" s="204" t="str">
         <x:v>PASS (상대 선형성)</x:v>
       </x:c>
       <x:c r="P30" s="100" t="str">
         <x:v>50%FS 최대 편차 0.2803% (기준 1%). 절대 전압·전류 기준값은 현장 검증 이관.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="206" t="str">
+        <x:v>열화상 참고 관찰: 양 채널 11 V / 5 A 부하 시험 말기</x:v>
+      </x:c>
+      <x:c r="B32" s="206"/>
+      <x:c r="C32" s="206"/>
+      <x:c r="D32" s="206"/>
+      <x:c r="E32" s="206"/>
+      <x:c r="F32" s="206"/>
+      <x:c r="G32" s="206"/>
+      <x:c r="H32" s="206"/>
+      <x:c r="I32" s="206"/>
+      <x:c r="J32" s="206"/>
+      <x:c r="K32" s="206"/>
+      <x:c r="L32" s="206"/>
+      <x:c r="M32" s="206"/>
+      <x:c r="N32" s="206"/>
+      <x:c r="O32" s="206"/>
+      <x:c r="P32" s="206"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="213" t="str">
+        <x:v>증빙 이미지</x:v>
+      </x:c>
+      <x:c r="B33" s="213" t="str">
+        <x:v>시험 조건</x:v>
+      </x:c>
+      <x:c r="C33" s="213" t="str">
+        <x:v>표시 최대 (°C)</x:v>
+      </x:c>
+      <x:c r="D33" s="213" t="str">
+        <x:v>중앙 측정점 (°C)</x:v>
+      </x:c>
+      <x:c r="E33" s="213" t="str">
+        <x:v>표시 하한/주변 (°C)</x:v>
+      </x:c>
+      <x:c r="F33" s="213" t="str">
+        <x:v>카메라 설정</x:v>
+      </x:c>
+      <x:c r="G33" s="213" t="str">
+        <x:v>판정/메모</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="48" customHeight="1">
+      <x:c r="A34" s="100" t="str">
+        <x:v>발열1.jpg</x:v>
+      </x:c>
+      <x:c r="B34" s="100" t="str">
+        <x:v>CH1+CH2 11 V / 5 A, 시험 말기</x:v>
+      </x:c>
+      <x:c r="C34" s="215" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="D34" s="215" t="n">
+        <x:v>33.5</x:v>
+      </x:c>
+      <x:c r="E34" s="215" t="n">
+        <x:v>26.9</x:v>
+      </x:c>
+      <x:c r="F34" s="100" t="str">
+        <x:v>Emissivity 0.95</x:v>
+      </x:c>
+      <x:c r="G34" s="100" t="str">
+        <x:v>국부 최고점 41.0°C 관찰; 부품 위치 미확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="48" customHeight="1">
+      <x:c r="A35" s="100" t="str">
+        <x:v>발열2.jpg</x:v>
+      </x:c>
+      <x:c r="B35" s="100" t="str">
+        <x:v>CH1+CH2 11 V / 5 A, 시험 말기</x:v>
+      </x:c>
+      <x:c r="C35" s="215" t="n">
+        <x:v>42.9</x:v>
+      </x:c>
+      <x:c r="D35" s="215" t="n">
+        <x:v>37.6</x:v>
+      </x:c>
+      <x:c r="E35" s="215" t="n">
+        <x:v>28.6</x:v>
+      </x:c>
+      <x:c r="F35" s="100" t="str">
+        <x:v>Emissivity 0.95</x:v>
+      </x:c>
+      <x:c r="G35" s="100" t="str">
+        <x:v>국부 최고점 42.9°C 관찰; 과열 징후 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="48" customHeight="1">
+      <x:c r="A36" s="100" t="str">
+        <x:v>발열3.jpg</x:v>
+      </x:c>
+      <x:c r="B36" s="100" t="str">
+        <x:v>CH1+CH2 11 V / 5 A, 시험 말기</x:v>
+      </x:c>
+      <x:c r="C36" s="215" t="n">
+        <x:v>42.9</x:v>
+      </x:c>
+      <x:c r="D36" s="215" t="n">
+        <x:v>34.2</x:v>
+      </x:c>
+      <x:c r="E36" s="215" t="n">
+        <x:v>27.6</x:v>
+      </x:c>
+      <x:c r="F36" s="100" t="str">
+        <x:v>Emissivity 0.95</x:v>
+      </x:c>
+      <x:c r="G36" s="100" t="str">
+        <x:v>국부 최고점 42.9°C 관찰; 정격 판정용이 아닌 참고 자료</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4683,6 +4862,7 @@
     <x:mergeCell ref="A17:P17"/>
     <x:mergeCell ref="A24:P24"/>
     <x:mergeCell ref="A28:P28"/>
+    <x:mergeCell ref="A32:P32"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Polish firmware test workbook and record stability run
</commit_message>
<xml_diff>
--- a/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
+++ b/docs/COSMOKE_H563_Firmware_Performance_Test_Record.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6b76e2f56e304f4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="R84eb57ead8f0401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R66b8697567d34d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="Rb25b39fb71a049f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="Re4085fb988964699"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R871964fc51df43d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1bd947e6767c4576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" r:id="Rc00a69b27e204d17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="Red6883c3d9574840"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Profiles" sheetId="4" r:id="R2b528896cd4a4ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Procedures" sheetId="5" r:id="R84dfa42f7b464c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capture History" sheetId="6" r:id="R44cc67f938e64d3a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27,7 +27,7 @@
     <x:numFmt numFmtId="205" formatCode="0.000000"/>
     <x:numFmt numFmtId="206" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -66,8 +66,101 @@
       <x:color rgb="FF49657A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="17"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17364D"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF17364D"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF3D4A55"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF17364D"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF5B4A00"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="72">
+  <x:fills count="79">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -424,8 +517,43 @@
         <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17364D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDF3E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="11">
+  <x:borders count="12">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -507,11 +635,25 @@
         <x:color rgb="FFD5E1EA"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E2EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7E2EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7E2EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7E2EA"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="216">
+  <x:cellXfs count="338">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -992,11 +1134,345 @@
     <x:xf numFmtId="206" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="74" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="75" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="13" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="75" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="75" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="74" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="74" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="76" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="76" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="72" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="76" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="76" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="76" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="76" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="76" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="76" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="72" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="72" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="72" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="18" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="8" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="78" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="76" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="76" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="5">
+  <x:dxfs count="7">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1025,6 +1501,28 @@
       <x:font>
         <x:color rgb="FF92400E"/>
       </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDDF3E4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF1BF"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
@@ -1061,7 +1559,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Dashboard'!$D$8:$D$13</c:f>
+              <c:f>'Dashboard'!$D$8:$D$12</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1069,7 +1567,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard'!$E$8:$E$13</c:f>
+              <c:f>'Dashboard'!$E$8:$E$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1085,7 +1583,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Dashboard'!$D$8:$D$13</c:f>
+              <c:f>'Dashboard'!$D$8:$D$12</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1093,7 +1591,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard'!$F$8:$F$13</c:f>
+              <c:f>'Dashboard'!$F$8:$F$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1194,7 +1692,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcecc59c84ff74988"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ba7616bd53b4d12"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1411,302 +1909,566 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
-      <x:c r="J1" s="4" t="str">
+      <x:c r="J1" s="239" t="str">
         <x:v>COSMOKE H563 펌웨어 성능 시험 기록표</x:v>
       </x:c>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="227"/>
+      <x:c r="B2" s="227"/>
+      <x:c r="C2" s="227"/>
+      <x:c r="D2" s="227"/>
+      <x:c r="E2" s="227"/>
+      <x:c r="F2" s="227"/>
+      <x:c r="G2" s="227"/>
+      <x:c r="H2" s="227"/>
+      <x:c r="I2" s="227"/>
+      <x:c r="J2" s="227"/>
+    </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="7" t="str">
+      <x:c r="A3" s="228" t="str">
         <x:v>시험 결과는 'Test Log' 탭에 입력합니다. Dashboard의 판정과 합격률은 자동 계산됩니다.</x:v>
       </x:c>
-      <x:c r="B3" s="7"/>
-      <x:c r="C3" s="7"/>
-      <x:c r="D3" s="7"/>
-      <x:c r="E3" s="7"/>
-      <x:c r="F3" s="7"/>
-      <x:c r="G3" s="7"/>
-      <x:c r="H3" s="7"/>
-      <x:c r="I3" s="7"/>
-      <x:c r="J3" s="7"/>
+      <x:c r="B3" s="228"/>
+      <x:c r="C3" s="228"/>
+      <x:c r="D3" s="228"/>
+      <x:c r="E3" s="228"/>
+      <x:c r="F3" s="228"/>
+      <x:c r="G3" s="228"/>
+      <x:c r="H3" s="228"/>
+      <x:c r="I3" s="228"/>
+      <x:c r="J3" s="228"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="227"/>
+      <x:c r="B4" s="227"/>
+      <x:c r="C4" s="227"/>
+      <x:c r="D4" s="227"/>
+      <x:c r="E4" s="227"/>
+      <x:c r="F4" s="227"/>
+      <x:c r="G4" s="227"/>
+      <x:c r="H4" s="227"/>
+      <x:c r="I4" s="227"/>
+      <x:c r="J4" s="227"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
-      <x:c r="A5" s="10" t="str">
+      <x:c r="A5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="B5" s="10" t="str">
+      <x:c r="B5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="C5" s="10" t="str">
+      <x:c r="C5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="D5" s="10" t="str">
+      <x:c r="D5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="E5" s="10" t="str">
+      <x:c r="E5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="F5" s="10" t="str">
+      <x:c r="F5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="G5" s="10" t="str">
+      <x:c r="G5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="H5" s="10" t="str">
+      <x:c r="H5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="I5" s="10" t="str">
+      <x:c r="I5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
-      <x:c r="J5" s="10" t="str">
+      <x:c r="J5" s="240" t="str">
         <x:v>시험 현황</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
-      <x:c r="A6" s="13" t="str">
+      <x:c r="A6" s="245" t="str">
         <x:v>총 시험 항목</x:v>
       </x:c>
-      <x:c r="B6" s="17" t="n">
+      <x:c r="B6" s="246" t="n">
         <x:f>COUNTIF('Test Log'!Q6:Q20,"PASS")+COUNTIF('Test Log'!Q6:Q20,"FAIL")+COUNTIF('Test Log'!Q6:Q20,"INPUT")</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D6" s="10" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C6" s="227"/>
+      <x:c r="D6" s="229" t="str">
         <x:v>카테고리별 결과</x:v>
       </x:c>
-      <x:c r="E6" s="10" t="str">
+      <x:c r="E6" s="229" t="str">
         <x:v>카테고리별 결과</x:v>
       </x:c>
-      <x:c r="F6" s="10" t="str">
+      <x:c r="F6" s="229" t="str">
         <x:v>카테고리별 결과</x:v>
       </x:c>
-      <x:c r="G6" s="10" t="str">
+      <x:c r="G6" s="229" t="str">
         <x:v>카테고리별 결과</x:v>
       </x:c>
-      <x:c r="H6" s="10" t="str">
+      <x:c r="H6" s="229" t="str">
         <x:v>카테고리별 결과</x:v>
       </x:c>
-      <x:c r="I6" s="10" t="str">
+      <x:c r="I6" s="229" t="str">
         <x:v>카테고리별 결과</x:v>
       </x:c>
-      <x:c r="J6" s="10" t="str">
+      <x:c r="J6" s="229" t="str">
         <x:v>카테고리별 결과</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="13" t="str">
+      <x:c r="A7" s="248" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="B7" s="17" t="n">
+      <x:c r="B7" s="249" t="n">
         <x:f>COUNTIF('Test Log'!Q6:Q20,"PASS")</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D7" s="23" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C7" s="227"/>
+      <x:c r="D7" s="258" t="str">
         <x:v>카테고리</x:v>
       </x:c>
-      <x:c r="E7" s="23" t="str">
+      <x:c r="E7" s="258" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="F7" s="23" t="str">
+      <x:c r="F7" s="258" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="G7" s="23" t="str">
+      <x:c r="G7" s="258" t="str">
         <x:v>미입력/확인</x:v>
       </x:c>
+      <x:c r="H7" s="227"/>
+      <x:c r="I7" s="227"/>
+      <x:c r="J7" s="227"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="13" t="str">
+      <x:c r="A8" s="250" t="str">
         <x:v>FAIL</x:v>
       </x:c>
-      <x:c r="B8" s="17" t="n">
+      <x:c r="B8" s="251" t="n">
         <x:f>COUNTIF('Test Log'!Q6:Q20,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D8" s="26" t="str">
+      <x:c r="C8" s="227"/>
+      <x:c r="D8" s="259" t="str">
         <x:v>기능</x:v>
       </x:c>
-      <x:c r="E8" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"PASS")</x:f>
+      <x:c r="E8" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D6:D20,D8,'Test Log'!Q6:Q20,"PASS")</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F8" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
+      <x:c r="F8" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D6:D20,D8,'Test Log'!Q6:Q20,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G8" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D8,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
+      <x:c r="G8" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D6:D20,D8,'Test Log'!Q6:Q20,"INPUT")</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="H8" s="227"/>
+      <x:c r="I8" s="227"/>
+      <x:c r="J8" s="227"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="13" t="str">
+      <x:c r="A9" s="252" t="str">
         <x:v>입력 대기</x:v>
       </x:c>
-      <x:c r="B9" s="17" t="n">
+      <x:c r="B9" s="253" t="n">
         <x:f>COUNTIF('Test Log'!Q6:Q20,"INPUT")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D9" s="26" t="str">
+      <x:c r="C9" s="227"/>
+      <x:c r="D9" s="259" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="E9" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"PASS")</x:f>
+      <x:c r="E9" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D7:D21,D9,'Test Log'!Q7:Q21,"PASS")</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F9" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
+      <x:c r="F9" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D7:D21,D9,'Test Log'!Q7:Q21,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G9" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D9,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
+      <x:c r="G9" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D7:D21,D9,'Test Log'!Q7:Q21,"INPUT")</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="H9" s="227"/>
+      <x:c r="I9" s="227"/>
+      <x:c r="J9" s="227"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="13" t="str">
+      <x:c r="A10" s="245" t="str">
         <x:v>합격률</x:v>
       </x:c>
-      <x:c r="B10" s="18" t="n">
+      <x:c r="B10" s="247" t="n">
         <x:f>IF(B6=0,0,B7/B6)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D10" s="26" t="str">
+      <x:c r="C10" s="227"/>
+      <x:c r="D10" s="259" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
-      <x:c r="E10" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"PASS")</x:f>
+      <x:c r="E10" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D8:D22,D10,'Test Log'!Q8:Q22,"PASS")</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F10" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
+      <x:c r="F10" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D8:D22,D10,'Test Log'!Q8:Q22,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G10" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D10,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
+      <x:c r="G10" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D8:D22,D10,'Test Log'!Q8:Q22,"INPUT")</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="H10" s="227"/>
+      <x:c r="I10" s="227"/>
+      <x:c r="J10" s="227"/>
     </x:row>
     <x:row r="11">
-      <x:c r="D11" s="26" t="str">
+      <x:c r="A11" s="227"/>
+      <x:c r="B11" s="227"/>
+      <x:c r="C11" s="227"/>
+      <x:c r="D11" s="259" t="str">
         <x:v>통신</x:v>
       </x:c>
-      <x:c r="E11" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"PASS")</x:f>
+      <x:c r="E11" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D9:D23,D11,'Test Log'!Q9:Q23,"PASS")</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F11" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
+      <x:c r="F11" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D9:D23,D11,'Test Log'!Q9:Q23,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G11" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D11,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
+      <x:c r="G11" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D9:D23,D11,'Test Log'!Q9:Q23,"INPUT")</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="H11" s="227"/>
+      <x:c r="I11" s="227"/>
+      <x:c r="J11" s="227"/>
     </x:row>
     <x:row r="12">
-      <x:c r="D12" s="26" t="str">
-        <x:v>복구·안전</x:v>
-      </x:c>
-      <x:c r="E12" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D12,'Test Log'!Q$2:Q$201,"PASS")</x:f>
+      <x:c r="A12" s="227"/>
+      <x:c r="B12" s="227"/>
+      <x:c r="C12" s="227"/>
+      <x:c r="D12" s="259" t="str">
+        <x:v>장시간 안정성</x:v>
+      </x:c>
+      <x:c r="E12" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D10:D24,D12,'Test Log'!Q10:Q24,"PASS")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F12" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D10:D24,D12,'Test Log'!Q10:Q24,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F12" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D12,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
+      <x:c r="G12" s="260" t="n">
+        <x:f>COUNTIFS('Test Log'!D10:D24,D12,'Test Log'!Q10:Q24,"INPUT")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G12" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D12,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D12,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="H12" s="227"/>
+      <x:c r="I12" s="227"/>
+      <x:c r="J12" s="227"/>
     </x:row>
     <x:row r="13">
-      <x:c r="D13" s="26" t="str">
-        <x:v>장시간 안정성</x:v>
-      </x:c>
-      <x:c r="E13" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D13,'Test Log'!Q$2:Q$201,"PASS")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F13" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D13,'Test Log'!Q$2:Q$201,"FAIL")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G13" s="25" t="n">
-        <x:f>COUNTIFS('Test Log'!D$2:D$201,D13,'Test Log'!Q$2:Q$201,"INPUT")+COUNTIFS('Test Log'!D$2:D$201,D13,'Test Log'!Q$2:Q$201,"CHECK")</x:f>
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="A13" s="227"/>
+      <x:c r="B13" s="227"/>
+      <x:c r="C13" s="227"/>
+      <x:c r="D13" s="259"/>
+      <x:c r="E13" s="260"/>
+      <x:c r="F13" s="260"/>
+      <x:c r="G13" s="260"/>
+      <x:c r="H13" s="227"/>
+      <x:c r="I13" s="227"/>
+      <x:c r="J13" s="227"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="227"/>
+      <x:c r="B14" s="227"/>
+      <x:c r="C14" s="227"/>
+      <x:c r="D14" s="227"/>
+      <x:c r="E14" s="227"/>
+      <x:c r="F14" s="227"/>
+      <x:c r="G14" s="227"/>
+      <x:c r="H14" s="227"/>
+      <x:c r="I14" s="227"/>
+      <x:c r="J14" s="227"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="227"/>
+      <x:c r="B15" s="227"/>
+      <x:c r="C15" s="227"/>
+      <x:c r="D15" s="227"/>
+      <x:c r="E15" s="227"/>
+      <x:c r="F15" s="227"/>
+      <x:c r="G15" s="227"/>
+      <x:c r="H15" s="227"/>
+      <x:c r="I15" s="227"/>
+      <x:c r="J15" s="227"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="227"/>
+      <x:c r="B16" s="227"/>
+      <x:c r="C16" s="227"/>
+      <x:c r="D16" s="227"/>
+      <x:c r="E16" s="227"/>
+      <x:c r="F16" s="227"/>
+      <x:c r="G16" s="227"/>
+      <x:c r="H16" s="227"/>
+      <x:c r="I16" s="227"/>
+      <x:c r="J16" s="227"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="227"/>
+      <x:c r="B17" s="227"/>
+      <x:c r="C17" s="227"/>
+      <x:c r="D17" s="227"/>
+      <x:c r="E17" s="227"/>
+      <x:c r="F17" s="227"/>
+      <x:c r="G17" s="227"/>
+      <x:c r="H17" s="227"/>
+      <x:c r="I17" s="227"/>
+      <x:c r="J17" s="227"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="227"/>
+      <x:c r="B18" s="227"/>
+      <x:c r="C18" s="227"/>
+      <x:c r="D18" s="227"/>
+      <x:c r="E18" s="227"/>
+      <x:c r="F18" s="227"/>
+      <x:c r="G18" s="227"/>
+      <x:c r="H18" s="227"/>
+      <x:c r="I18" s="227"/>
+      <x:c r="J18" s="227"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="227"/>
+      <x:c r="B19" s="227"/>
+      <x:c r="C19" s="227"/>
+      <x:c r="D19" s="227"/>
+      <x:c r="E19" s="227"/>
+      <x:c r="F19" s="227"/>
+      <x:c r="G19" s="227"/>
+      <x:c r="H19" s="227"/>
+      <x:c r="I19" s="227"/>
+      <x:c r="J19" s="227"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="227"/>
+      <x:c r="B20" s="227"/>
+      <x:c r="C20" s="227"/>
+      <x:c r="D20" s="227"/>
+      <x:c r="E20" s="227"/>
+      <x:c r="F20" s="227"/>
+      <x:c r="G20" s="227"/>
+      <x:c r="H20" s="227"/>
+      <x:c r="I20" s="227"/>
+      <x:c r="J20" s="227"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="227"/>
+      <x:c r="B21" s="227"/>
+      <x:c r="C21" s="227"/>
+      <x:c r="D21" s="227"/>
+      <x:c r="E21" s="227"/>
+      <x:c r="F21" s="227"/>
+      <x:c r="G21" s="227"/>
+      <x:c r="H21" s="227"/>
+      <x:c r="I21" s="227"/>
+      <x:c r="J21" s="227"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="227"/>
+      <x:c r="B22" s="227"/>
+      <x:c r="C22" s="227"/>
+      <x:c r="D22" s="227"/>
+      <x:c r="E22" s="227"/>
+      <x:c r="F22" s="227"/>
+      <x:c r="G22" s="227"/>
+      <x:c r="H22" s="227"/>
+      <x:c r="I22" s="227"/>
+      <x:c r="J22" s="227"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="227"/>
+      <x:c r="B23" s="227"/>
+      <x:c r="C23" s="227"/>
+      <x:c r="D23" s="227"/>
+      <x:c r="E23" s="227"/>
+      <x:c r="F23" s="227"/>
+      <x:c r="G23" s="227"/>
+      <x:c r="H23" s="227"/>
+      <x:c r="I23" s="227"/>
+      <x:c r="J23" s="227"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="227"/>
+      <x:c r="B24" s="227"/>
+      <x:c r="C24" s="227"/>
+      <x:c r="D24" s="227"/>
+      <x:c r="E24" s="227"/>
+      <x:c r="F24" s="227"/>
+      <x:c r="G24" s="227"/>
+      <x:c r="H24" s="227"/>
+      <x:c r="I24" s="227"/>
+      <x:c r="J24" s="227"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="227"/>
+      <x:c r="B25" s="227"/>
+      <x:c r="C25" s="227"/>
+      <x:c r="D25" s="227"/>
+      <x:c r="E25" s="227"/>
+      <x:c r="F25" s="227"/>
+      <x:c r="G25" s="227"/>
+      <x:c r="H25" s="227"/>
+      <x:c r="I25" s="227"/>
+      <x:c r="J25" s="227"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="227"/>
+      <x:c r="B26" s="227"/>
+      <x:c r="C26" s="227"/>
+      <x:c r="D26" s="227"/>
+      <x:c r="E26" s="227"/>
+      <x:c r="F26" s="227"/>
+      <x:c r="G26" s="227"/>
+      <x:c r="H26" s="227"/>
+      <x:c r="I26" s="227"/>
+      <x:c r="J26" s="227"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="227"/>
+      <x:c r="B27" s="227"/>
+      <x:c r="C27" s="227"/>
+      <x:c r="D27" s="227"/>
+      <x:c r="E27" s="227"/>
+      <x:c r="F27" s="227"/>
+      <x:c r="G27" s="227"/>
+      <x:c r="H27" s="227"/>
+      <x:c r="I27" s="227"/>
+      <x:c r="J27" s="227"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="227"/>
+      <x:c r="B28" s="227"/>
+      <x:c r="C28" s="227"/>
+      <x:c r="D28" s="227"/>
+      <x:c r="E28" s="227"/>
+      <x:c r="F28" s="227"/>
+      <x:c r="G28" s="227"/>
+      <x:c r="H28" s="227"/>
+      <x:c r="I28" s="227"/>
+      <x:c r="J28" s="227"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="227"/>
+      <x:c r="B29" s="227"/>
+      <x:c r="C29" s="227"/>
+      <x:c r="D29" s="227"/>
+      <x:c r="E29" s="227"/>
+      <x:c r="F29" s="227"/>
+      <x:c r="G29" s="227"/>
+      <x:c r="H29" s="227"/>
+      <x:c r="I29" s="227"/>
+      <x:c r="J29" s="227"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="227"/>
+      <x:c r="B30" s="227"/>
+      <x:c r="C30" s="227"/>
+      <x:c r="D30" s="227"/>
+      <x:c r="E30" s="227"/>
+      <x:c r="F30" s="227"/>
+      <x:c r="G30" s="227"/>
+      <x:c r="H30" s="227"/>
+      <x:c r="I30" s="227"/>
+      <x:c r="J30" s="227"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="227"/>
+      <x:c r="B31" s="227"/>
+      <x:c r="C31" s="227"/>
+      <x:c r="D31" s="227"/>
+      <x:c r="E31" s="227"/>
+      <x:c r="F31" s="227"/>
+      <x:c r="G31" s="227"/>
+      <x:c r="H31" s="227"/>
+      <x:c r="I31" s="227"/>
+      <x:c r="J31" s="227"/>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
-      <x:c r="A32" s="10" t="str">
+      <x:c r="A32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="B32" s="10" t="str">
+      <x:c r="B32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="C32" s="10" t="str">
+      <x:c r="C32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="D32" s="10" t="str">
+      <x:c r="D32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="E32" s="10" t="str">
+      <x:c r="E32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="F32" s="10" t="str">
+      <x:c r="F32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="G32" s="10" t="str">
+      <x:c r="G32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="H32" s="10" t="str">
+      <x:c r="H32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="I32" s="10" t="str">
+      <x:c r="I32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
-      <x:c r="J32" s="10" t="str">
+      <x:c r="J32" s="240" t="str">
         <x:v>시험 실행 메모</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="26" customHeight="1">
-      <x:c r="A33" s="45" t="str">
-        <x:v>시험 날짜, 보드 식별, 펌웨어 commit, 측정 장비, 온도·전원 조건을 Test Log에 반드시 남기십시오. 실제 부하 연결 전에는 WARMUP→ACTIVE, ADC/SPI/DAC fault, LAN 미연결, watchdog 동작을 벤치 환경에서 검증합니다.</x:v>
-      </x:c>
-      <x:c r="B33" s="46"/>
-      <x:c r="C33" s="46"/>
-      <x:c r="D33" s="46"/>
-      <x:c r="E33" s="46"/>
-      <x:c r="F33" s="46"/>
-      <x:c r="G33" s="46"/>
-      <x:c r="H33" s="46"/>
-      <x:c r="I33" s="46"/>
-      <x:c r="J33" s="47"/>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="264" t="str">
+        <x:v>시험 날짜, 보드 식별, 펌웨어 commit, 측정 장비, 온도·전원 조건을 Test Log에 남기십시오. 실부하 연결 전에는 WARMUP→ACTIVE와 기본 텔레메트리 상태를 확인합니다.</x:v>
+      </x:c>
+      <x:c r="B33" s="265"/>
+      <x:c r="C33" s="265"/>
+      <x:c r="D33" s="265"/>
+      <x:c r="E33" s="265"/>
+      <x:c r="F33" s="265"/>
+      <x:c r="G33" s="265"/>
+      <x:c r="H33" s="265"/>
+      <x:c r="I33" s="265"/>
+      <x:c r="J33" s="266"/>
     </x:row>
     <x:row r="34" ht="26" customHeight="1">
       <x:c r="A34" s="48"/>
@@ -1752,7 +2514,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a1181120e654137"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf394f5ee724c84"/>
 </x:worksheet>
 </file>
 
@@ -1763,404 +2525,448 @@
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="9" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
-      <x:c r="J1" s="4" t="str">
+      <x:c r="J1" s="270" t="str">
         <x:v>펌웨어 성능 시험 계획</x:v>
       </x:c>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="227"/>
+      <x:c r="B2" s="227"/>
+      <x:c r="C2" s="227"/>
+      <x:c r="D2" s="227"/>
+      <x:c r="E2" s="227"/>
+      <x:c r="F2" s="227"/>
+      <x:c r="G2" s="227"/>
+      <x:c r="H2" s="227"/>
+      <x:c r="I2" s="227"/>
+      <x:c r="J2" s="227"/>
+    </x:row>
     <x:row r="3">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="267" t="str">
         <x:v>목표값은 프로젝트 요구사항에 맞게 승인 후 수정하십시오. Test Log에 동일한 ID로 실제 결과를 기록합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="6"/>
-      <x:c r="C3" s="6"/>
-      <x:c r="D3" s="6"/>
-      <x:c r="E3" s="6"/>
-      <x:c r="F3" s="6"/>
-      <x:c r="G3" s="6"/>
-      <x:c r="H3" s="6"/>
-      <x:c r="I3" s="6"/>
-      <x:c r="J3" s="6"/>
+      <x:c r="B3" s="267"/>
+      <x:c r="C3" s="267"/>
+      <x:c r="D3" s="267"/>
+      <x:c r="E3" s="267"/>
+      <x:c r="F3" s="267"/>
+      <x:c r="G3" s="267"/>
+      <x:c r="H3" s="267"/>
+      <x:c r="I3" s="267"/>
+      <x:c r="J3" s="267"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="227"/>
+      <x:c r="B4" s="227"/>
+      <x:c r="C4" s="227"/>
+      <x:c r="D4" s="227"/>
+      <x:c r="E4" s="227"/>
+      <x:c r="F4" s="227"/>
+      <x:c r="G4" s="227"/>
+      <x:c r="H4" s="227"/>
+      <x:c r="I4" s="227"/>
+      <x:c r="J4" s="227"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="23" t="str">
+      <x:c r="A5" s="272" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="23" t="str">
+      <x:c r="B5" s="272" t="str">
         <x:v>카테고리</x:v>
       </x:c>
-      <x:c r="C5" s="23" t="str">
+      <x:c r="C5" s="272" t="str">
         <x:v>시험 항목</x:v>
       </x:c>
-      <x:c r="D5" s="23" t="str">
+      <x:c r="D5" s="272" t="str">
         <x:v>측정 지표</x:v>
       </x:c>
-      <x:c r="E5" s="23" t="str">
+      <x:c r="E5" s="272" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="F5" s="23" t="str">
+      <x:c r="F5" s="272" t="str">
         <x:v>권장 기준</x:v>
       </x:c>
-      <x:c r="G5" s="23" t="str">
+      <x:c r="G5" s="272" t="str">
         <x:v>비교</x:v>
       </x:c>
-      <x:c r="H5" s="23" t="str">
+      <x:c r="H5" s="272" t="str">
         <x:v>방법/장비</x:v>
       </x:c>
-      <x:c r="I5" s="23" t="str">
+      <x:c r="I5" s="272" t="str">
         <x:v>우선순위</x:v>
       </x:c>
-      <x:c r="J5" s="23" t="str">
+      <x:c r="J5" s="272" t="str">
         <x:v>비고</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="55" t="str">
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="279" t="str">
         <x:v>F-01</x:v>
       </x:c>
-      <x:c r="B6" s="55" t="str">
+      <x:c r="B6" s="275" t="str">
         <x:v>기능</x:v>
       </x:c>
-      <x:c r="C6" s="55" t="str">
+      <x:c r="C6" s="275" t="str">
         <x:v>부팅 상태 전이</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="str">
+      <x:c r="D6" s="275" t="str">
         <x:v>WARMUP→ACTIVE</x:v>
       </x:c>
-      <x:c r="E6" s="55" t="str">
+      <x:c r="E6" s="275" t="str">
         <x:v>s</x:v>
       </x:c>
-      <x:c r="F6" s="56" t="n">
+      <x:c r="F6" s="276" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="275" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="275" t="str">
         <x:v>UART/UDP 로그, 스톱워치</x:v>
       </x:c>
-      <x:c r="I6" s="55" t="str">
+      <x:c r="I6" s="275" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="J6" s="55" t="str">
+      <x:c r="J6" s="275" t="str">
         <x:v>GUI 첫 VALID 텔레메트리 기준 3초 이내</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="55" t="str">
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="279" t="str">
         <x:v>A-01</x:v>
       </x:c>
-      <x:c r="B7" s="55" t="str">
+      <x:c r="B7" s="275" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="C7" s="55" t="str">
+      <x:c r="C7" s="275" t="str">
         <x:v>영점 오차</x:v>
       </x:c>
-      <x:c r="D7" s="55" t="str">
+      <x:c r="D7" s="275" t="str">
         <x:v>0 입력 오차</x:v>
       </x:c>
-      <x:c r="E7" s="55" t="str">
+      <x:c r="E7" s="275" t="str">
         <x:v>%FS</x:v>
       </x:c>
-      <x:c r="F7" s="56" t="n">
+      <x:c r="F7" s="276" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="G7" s="55" t="str">
+      <x:c r="G7" s="275" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="H7" s="55" t="str">
+      <x:c r="H7" s="275" t="str">
         <x:v>정밀 DMM/캘리브레이터</x:v>
       </x:c>
-      <x:c r="I7" s="55" t="str">
+      <x:c r="I7" s="275" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="J7" s="55" t="str">
+      <x:c r="J7" s="275" t="str">
         <x:v>채널별 기록</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="55" t="str">
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="279" t="str">
         <x:v>A-02</x:v>
       </x:c>
-      <x:c r="B8" s="55" t="str">
+      <x:c r="B8" s="275" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="C8" s="55" t="str">
+      <x:c r="C8" s="275" t="str">
         <x:v>gain 오차</x:v>
       </x:c>
-      <x:c r="D8" s="55" t="str">
+      <x:c r="D8" s="275" t="str">
         <x:v>100% span 오차</x:v>
       </x:c>
-      <x:c r="E8" s="55" t="str">
+      <x:c r="E8" s="275" t="str">
         <x:v>%FS</x:v>
       </x:c>
-      <x:c r="F8" s="56" t="n">
+      <x:c r="F8" s="276" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="G8" s="55" t="str">
+      <x:c r="G8" s="275" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="H8" s="55" t="str">
+      <x:c r="H8" s="275" t="str">
         <x:v>정밀 전압·전류원</x:v>
       </x:c>
-      <x:c r="I8" s="55" t="str">
+      <x:c r="I8" s="275" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="J8" s="55" t="str">
+      <x:c r="J8" s="275" t="str">
         <x:v>보정 전/후 비교</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="55" t="str">
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="279" t="str">
         <x:v>A-03</x:v>
       </x:c>
-      <x:c r="B9" s="55" t="str">
+      <x:c r="B9" s="275" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="C9" s="55" t="str">
+      <x:c r="C9" s="275" t="str">
         <x:v>선형성</x:v>
       </x:c>
-      <x:c r="D9" s="55" t="str">
+      <x:c r="D9" s="275" t="str">
         <x:v>0/50/100% 최대 편차</x:v>
       </x:c>
-      <x:c r="E9" s="55" t="str">
+      <x:c r="E9" s="275" t="str">
         <x:v>%FS</x:v>
       </x:c>
-      <x:c r="F9" s="56" t="n">
+      <x:c r="F9" s="276" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G9" s="55" t="str">
+      <x:c r="G9" s="275" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="H9" s="55" t="str">
+      <x:c r="H9" s="275" t="str">
         <x:v>정밀 전압·전류원</x:v>
       </x:c>
-      <x:c r="I9" s="55" t="str">
+      <x:c r="I9" s="275" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="J9" s="55" t="str">
+      <x:c r="J9" s="275" t="str">
         <x:v>다점 결과 첨부</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="55" t="str">
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="279" t="str">
         <x:v>A-04</x:v>
       </x:c>
-      <x:c r="B10" s="55" t="str">
+      <x:c r="B10" s="275" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="C10" s="55" t="str">
+      <x:c r="C10" s="275" t="str">
         <x:v>입력 노이즈</x:v>
       </x:c>
-      <x:c r="D10" s="55" t="str">
+      <x:c r="D10" s="275" t="str">
         <x:v>RMS noise</x:v>
       </x:c>
-      <x:c r="E10" s="55" t="str">
+      <x:c r="E10" s="275" t="str">
         <x:v>mV/mA</x:v>
       </x:c>
-      <x:c r="F10" s="56" t="n">
+      <x:c r="F10" s="276" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="G10" s="55" t="str">
+      <x:c r="G10" s="275" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="H10" s="55" t="str">
+      <x:c r="H10" s="275" t="str">
         <x:v>고정 입력 10분 로그</x:v>
       </x:c>
-      <x:c r="I10" s="55" t="str">
+      <x:c r="I10" s="275" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="J10" s="55" t="str">
+      <x:c r="J10" s="275" t="str">
         <x:v>필터 설정 기록</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="55" t="str">
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="279" t="str">
         <x:v>T-01</x:v>
       </x:c>
-      <x:c r="B11" s="55" t="str">
+      <x:c r="B11" s="275" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
-      <x:c r="C11" s="55" t="str">
+      <x:c r="C11" s="275" t="str">
         <x:v>ADC 수집률</x:v>
       </x:c>
-      <x:c r="D11" s="55" t="str">
+      <x:c r="D11" s="275" t="str">
         <x:v>실제 sample rate</x:v>
       </x:c>
-      <x:c r="E11" s="55" t="str">
+      <x:c r="E11" s="275" t="str">
         <x:v>Hz</x:v>
       </x:c>
-      <x:c r="F11" s="56" t="n">
+      <x:c r="F11" s="276" t="n">
         <x:v>1980</x:v>
       </x:c>
-      <x:c r="G11" s="55" t="str">
+      <x:c r="G11" s="275" t="str">
         <x:v>최소</x:v>
       </x:c>
-      <x:c r="H11" s="55" t="str">
+      <x:c r="H11" s="275" t="str">
         <x:v>logic analyzer / timestamp</x:v>
       </x:c>
-      <x:c r="I11" s="55" t="str">
+      <x:c r="I11" s="275" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="J11" s="55" t="str">
+      <x:c r="J11" s="275" t="str">
         <x:v>명목 2 kSPS; 합격 기준은 1,980 Hz 이상 (±1%)</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="55" t="str">
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="279" t="str">
         <x:v>T-02</x:v>
       </x:c>
-      <x:c r="B12" s="55" t="str">
+      <x:c r="B12" s="275" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
-      <x:c r="C12" s="55" t="str">
+      <x:c r="C12" s="275" t="str">
         <x:v>DMA/링버퍼</x:v>
       </x:c>
-      <x:c r="D12" s="55" t="str">
+      <x:c r="D12" s="275" t="str">
         <x:v>dropped frames</x:v>
       </x:c>
-      <x:c r="E12" s="55" t="str">
+      <x:c r="E12" s="275" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="F12" s="56" t="n">
+      <x:c r="F12" s="276" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G12" s="55" t="str">
+      <x:c r="G12" s="275" t="str">
         <x:v>일치</x:v>
       </x:c>
-      <x:c r="H12" s="55" t="str">
+      <x:c r="H12" s="275" t="str">
         <x:v>telemetry counter</x:v>
       </x:c>
-      <x:c r="I12" s="55" t="str">
+      <x:c r="I12" s="275" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="J12" s="55" t="str">
+      <x:c r="J12" s="275" t="str">
         <x:v>10분 부하 시험</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="55"/>
-      <x:c r="B13" s="55"/>
-      <x:c r="C13" s="55"/>
-      <x:c r="D13" s="55"/>
-      <x:c r="E13" s="55"/>
-      <x:c r="F13" s="56"/>
-      <x:c r="G13" s="55"/>
-      <x:c r="H13" s="55"/>
-      <x:c r="I13" s="55"/>
-      <x:c r="J13" s="55"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="55" t="str">
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="279"/>
+      <x:c r="B13" s="275"/>
+      <x:c r="C13" s="275"/>
+      <x:c r="D13" s="275"/>
+      <x:c r="E13" s="275"/>
+      <x:c r="F13" s="276"/>
+      <x:c r="G13" s="275"/>
+      <x:c r="H13" s="275"/>
+      <x:c r="I13" s="275"/>
+      <x:c r="J13" s="275"/>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="279" t="str">
         <x:v>N-01</x:v>
       </x:c>
-      <x:c r="B14" s="55" t="str">
+      <x:c r="B14" s="275" t="str">
         <x:v>통신</x:v>
       </x:c>
-      <x:c r="C14" s="55" t="str">
+      <x:c r="C14" s="275" t="str">
         <x:v>UDP 전송률</x:v>
       </x:c>
-      <x:c r="D14" s="55" t="str">
+      <x:c r="D14" s="275" t="str">
         <x:v>송신 주기</x:v>
       </x:c>
-      <x:c r="E14" s="55" t="str">
+      <x:c r="E14" s="275" t="str">
         <x:v>ms</x:v>
       </x:c>
-      <x:c r="F14" s="56" t="n">
+      <x:c r="F14" s="276" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="G14" s="55" t="str">
+      <x:c r="G14" s="275" t="str">
         <x:v>일치</x:v>
       </x:c>
-      <x:c r="H14" s="55" t="str">
+      <x:c r="H14" s="275" t="str">
         <x:v>PC timestamp log</x:v>
       </x:c>
-      <x:c r="I14" s="55" t="str">
+      <x:c r="I14" s="275" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="J14" s="55" t="str">
+      <x:c r="J14" s="275" t="str">
         <x:v>명목 100 ms; 합격 범위는 평균 95–105 ms</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="55" t="str">
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="279" t="str">
         <x:v>N-02</x:v>
       </x:c>
-      <x:c r="B15" s="55" t="str">
+      <x:c r="B15" s="275" t="str">
         <x:v>통신</x:v>
       </x:c>
-      <x:c r="C15" s="55" t="str">
+      <x:c r="C15" s="275" t="str">
         <x:v>UDP 손실</x:v>
       </x:c>
-      <x:c r="D15" s="55" t="str">
+      <x:c r="D15" s="275" t="str">
         <x:v>sequence gap rate</x:v>
       </x:c>
-      <x:c r="E15" s="55" t="str">
+      <x:c r="E15" s="275" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="F15" s="56" t="n">
+      <x:c r="F15" s="276" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="G15" s="55" t="str">
+      <x:c r="G15" s="275" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="H15" s="55" t="str">
+      <x:c r="H15" s="275" t="str">
         <x:v>PC monitor</x:v>
       </x:c>
-      <x:c r="I15" s="55" t="str">
+      <x:c r="I15" s="275" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="J15" s="55" t="str">
+      <x:c r="J15" s="275" t="str">
         <x:v>동일 LAN 기준</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="55"/>
-      <x:c r="B16" s="55"/>
-      <x:c r="C16" s="55"/>
-      <x:c r="D16" s="55"/>
-      <x:c r="E16" s="55"/>
-      <x:c r="F16" s="56"/>
-      <x:c r="G16" s="55"/>
-      <x:c r="H16" s="55"/>
-      <x:c r="I16" s="55"/>
-      <x:c r="J16" s="55"/>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="279" t="str">
+        <x:v>L-01</x:v>
+      </x:c>
+      <x:c r="B16" s="275" t="str">
+        <x:v>장시간 안정성</x:v>
+      </x:c>
+      <x:c r="C16" s="275" t="str">
+        <x:v>양 채널 부하 안정성</x:v>
+      </x:c>
+      <x:c r="D16" s="275" t="str">
+        <x:v>연속 운전</x:v>
+      </x:c>
+      <x:c r="E16" s="275" t="str">
+        <x:v>min</x:v>
+      </x:c>
+      <x:c r="F16" s="276" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G16" s="275" t="str">
+        <x:v>최소</x:v>
+      </x:c>
+      <x:c r="H16" s="275" t="str">
+        <x:v>PC CSV / 대시보드</x:v>
+      </x:c>
+      <x:c r="I16" s="275" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J16" s="275" t="str">
+        <x:v>CH1+CH2 11 V / 5 A, 27.7분 검증; 다시간 soak은 범위 제외</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="55"/>
@@ -2224,810 +3030,897 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="8" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="9" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="12" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="11" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="11" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="12" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="13" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="38" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="44" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="I1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="J1" s="4" t="str">
+      <x:c r="J1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="K1" s="4" t="str">
+      <x:c r="K1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="L1" s="4" t="str">
+      <x:c r="L1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="M1" s="4" t="str">
+      <x:c r="M1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="N1" s="4" t="str">
+      <x:c r="N1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="O1" s="4" t="str">
+      <x:c r="O1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="P1" s="4" t="str">
+      <x:c r="P1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="Q1" s="4" t="str">
+      <x:c r="Q1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="R1" s="4" t="str">
+      <x:c r="R1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="S1" s="4" t="str">
+      <x:c r="S1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="T1" s="4" t="str">
+      <x:c r="T1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
-      <x:c r="U1" s="4" t="str">
+      <x:c r="U1" s="270" t="str">
         <x:v>성능 시험 결과 기록</x:v>
       </x:c>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="281"/>
+      <x:c r="B2" s="281"/>
+      <x:c r="C2" s="281"/>
+      <x:c r="D2" s="281"/>
+      <x:c r="E2" s="281"/>
+      <x:c r="F2" s="281"/>
+      <x:c r="G2" s="281"/>
+      <x:c r="H2" s="281"/>
+      <x:c r="I2" s="281"/>
+      <x:c r="J2" s="281"/>
+      <x:c r="K2" s="281"/>
+      <x:c r="L2" s="281"/>
+      <x:c r="M2" s="281"/>
+      <x:c r="N2" s="281"/>
+      <x:c r="O2" s="281"/>
+      <x:c r="P2" s="281"/>
+      <x:c r="Q2" s="281"/>
+      <x:c r="R2" s="281"/>
+      <x:c r="S2" s="281"/>
+      <x:c r="T2" s="281"/>
+      <x:c r="U2" s="281"/>
+    </x:row>
     <x:row r="3">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="282" t="str">
         <x:v>연한 파란색 열은 입력 영역입니다. Result는 Target/비교/측정값으로 자동 판정되며, 증빙 파일·로그 경로를 함께 남깁니다.</x:v>
       </x:c>
-      <x:c r="B3" s="6"/>
-      <x:c r="C3" s="6"/>
-      <x:c r="D3" s="6"/>
-      <x:c r="E3" s="6"/>
-      <x:c r="F3" s="6"/>
-      <x:c r="G3" s="6"/>
-      <x:c r="H3" s="6"/>
-      <x:c r="I3" s="6"/>
-      <x:c r="J3" s="6"/>
-      <x:c r="K3" s="6"/>
-      <x:c r="L3" s="6"/>
-      <x:c r="M3" s="6"/>
-      <x:c r="N3" s="6"/>
-      <x:c r="O3" s="6"/>
-      <x:c r="P3" s="6"/>
-      <x:c r="Q3" s="6"/>
-      <x:c r="R3" s="6"/>
-      <x:c r="S3" s="6"/>
-      <x:c r="T3" s="6"/>
-      <x:c r="U3" s="6"/>
-    </x:row>
-    <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="23" t="str">
+      <x:c r="B3" s="282"/>
+      <x:c r="C3" s="282"/>
+      <x:c r="D3" s="282"/>
+      <x:c r="E3" s="282"/>
+      <x:c r="F3" s="282"/>
+      <x:c r="G3" s="282"/>
+      <x:c r="H3" s="282"/>
+      <x:c r="I3" s="282"/>
+      <x:c r="J3" s="282"/>
+      <x:c r="K3" s="282"/>
+      <x:c r="L3" s="282"/>
+      <x:c r="M3" s="282"/>
+      <x:c r="N3" s="282"/>
+      <x:c r="O3" s="282"/>
+      <x:c r="P3" s="282"/>
+      <x:c r="Q3" s="282"/>
+      <x:c r="R3" s="282"/>
+      <x:c r="S3" s="282"/>
+      <x:c r="T3" s="282"/>
+      <x:c r="U3" s="282"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="281"/>
+      <x:c r="B4" s="281"/>
+      <x:c r="C4" s="281"/>
+      <x:c r="D4" s="281"/>
+      <x:c r="E4" s="281"/>
+      <x:c r="F4" s="281"/>
+      <x:c r="G4" s="281"/>
+      <x:c r="H4" s="281"/>
+      <x:c r="I4" s="281"/>
+      <x:c r="J4" s="281"/>
+      <x:c r="K4" s="281"/>
+      <x:c r="L4" s="281"/>
+      <x:c r="M4" s="281"/>
+      <x:c r="N4" s="281"/>
+      <x:c r="O4" s="281"/>
+      <x:c r="P4" s="281"/>
+      <x:c r="Q4" s="281"/>
+      <x:c r="R4" s="281"/>
+      <x:c r="S4" s="281"/>
+      <x:c r="T4" s="281"/>
+      <x:c r="U4" s="281"/>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="290" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="23" t="str">
+      <x:c r="B5" s="290" t="str">
         <x:v>시험일</x:v>
       </x:c>
-      <x:c r="C5" s="23" t="str">
+      <x:c r="C5" s="290" t="str">
         <x:v>FW 버전/commit</x:v>
       </x:c>
-      <x:c r="D5" s="23" t="str">
+      <x:c r="D5" s="290" t="str">
         <x:v>카테고리</x:v>
       </x:c>
-      <x:c r="E5" s="23" t="str">
+      <x:c r="E5" s="290" t="str">
         <x:v>시험 항목</x:v>
       </x:c>
-      <x:c r="F5" s="23" t="str">
+      <x:c r="F5" s="290" t="str">
         <x:v>측정 지표</x:v>
       </x:c>
-      <x:c r="G5" s="23" t="str">
+      <x:c r="G5" s="290" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="H5" s="23" t="str">
+      <x:c r="H5" s="290" t="str">
         <x:v>목표값</x:v>
       </x:c>
-      <x:c r="I5" s="23" t="str">
+      <x:c r="I5" s="290" t="str">
         <x:v>비교</x:v>
       </x:c>
-      <x:c r="J5" s="23" t="str">
+      <x:c r="J5" s="290" t="str">
         <x:v>측정값</x:v>
       </x:c>
-      <x:c r="K5" s="23" t="str">
+      <x:c r="K5" s="290" t="str">
         <x:v>최소</x:v>
       </x:c>
-      <x:c r="L5" s="23" t="str">
+      <x:c r="L5" s="290" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="M5" s="23" t="str">
+      <x:c r="M5" s="290" t="str">
         <x:v>평균</x:v>
       </x:c>
-      <x:c r="N5" s="23" t="str">
+      <x:c r="N5" s="290" t="str">
         <x:v>표준편차</x:v>
       </x:c>
-      <x:c r="O5" s="23" t="str">
+      <x:c r="O5" s="290" t="str">
         <x:v>샘플 수</x:v>
       </x:c>
-      <x:c r="P5" s="23" t="str">
+      <x:c r="P5" s="290" t="str">
         <x:v>환경/조건</x:v>
       </x:c>
-      <x:c r="Q5" s="23" t="str">
+      <x:c r="Q5" s="290" t="str">
         <x:v>Result</x:v>
       </x:c>
-      <x:c r="R5" s="23" t="str">
+      <x:c r="R5" s="290" t="str">
         <x:v>실행 상태</x:v>
       </x:c>
-      <x:c r="S5" s="23" t="str">
+      <x:c r="S5" s="290" t="str">
         <x:v>담당자</x:v>
       </x:c>
-      <x:c r="T5" s="23" t="str">
+      <x:c r="T5" s="290" t="str">
         <x:v>비고</x:v>
       </x:c>
-      <x:c r="U5" s="23" t="str">
+      <x:c r="U5" s="290" t="str">
         <x:v>증빙 경로</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="25" t="str">
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="308" t="str">
         <x:v>F-01</x:v>
       </x:c>
-      <x:c r="B6" s="58" t="n">
+      <x:c r="B6" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C6" s="57" t="str">
+      <x:c r="C6" s="303" t="str">
         <x:v>4b7b1d3</x:v>
       </x:c>
-      <x:c r="D6" s="25" t="str">
+      <x:c r="D6" s="301" t="str">
         <x:v>기능</x:v>
       </x:c>
-      <x:c r="E6" s="25" t="str">
+      <x:c r="E6" s="301" t="str">
         <x:v>부팅 상태 전이</x:v>
       </x:c>
-      <x:c r="F6" s="25" t="str">
+      <x:c r="F6" s="301" t="str">
         <x:v>WARMUP→ACTIVE</x:v>
       </x:c>
-      <x:c r="G6" s="25" t="str">
+      <x:c r="G6" s="301" t="str">
         <x:v>s</x:v>
       </x:c>
-      <x:c r="H6" s="59" t="n">
+      <x:c r="H6" s="309" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I6" s="59" t="str">
+      <x:c r="I6" s="304" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J6" s="60" t="n">
+      <x:c r="J6" s="310" t="n">
         <x:v>2.312</x:v>
       </x:c>
-      <x:c r="K6" s="60"/>
-      <x:c r="L6" s="60"/>
-      <x:c r="M6" s="60" t="n">
+      <x:c r="K6" s="310"/>
+      <x:c r="L6" s="310"/>
+      <x:c r="M6" s="310" t="n">
         <x:v>2.312</x:v>
       </x:c>
-      <x:c r="N6" s="60"/>
-      <x:c r="O6" s="60" t="n">
+      <x:c r="N6" s="310"/>
+      <x:c r="O6" s="310" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P6" s="57" t="str">
+      <x:c r="P6" s="303" t="str">
         <x:v>Reset 후 GUI 첫 VALID 텔레메트리</x:v>
       </x:c>
-      <x:c r="Q6" s="25" t="str">
+      <x:c r="Q6" s="311" t="str">
         <x:f>IF(OR(H6="",I6="",J6=""),"INPUT",IF(I6="최대",IF(J6&lt;=H6,"PASS","FAIL"),IF(I6="최소",IF(J6&gt;=H6,"PASS","FAIL"),IF(I6="일치",IF(J6=H6,"PASS","FAIL"),"CHECK"))))</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R6" s="57" t="str">
+      <x:c r="R6" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S6" s="57" t="str">
+      <x:c r="S6" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T6" s="57" t="str">
+      <x:c r="T6" s="303" t="str">
         <x:v>반복 부팅 관찰상 GUI 첫 정상 데이터가 보드 시간 약 2–3초. 대표 CSV 첫 VALID 2.312초.</x:v>
       </x:c>
-      <x:c r="U6" s="57" t="str">
+      <x:c r="U6" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_091833_148511.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="25" t="str">
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="308" t="str">
         <x:v>A-01</x:v>
       </x:c>
-      <x:c r="B7" s="58" t="n">
+      <x:c r="B7" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C7" s="57" t="str">
+      <x:c r="C7" s="303" t="str">
         <x:v>4b7b1d3</x:v>
       </x:c>
-      <x:c r="D7" s="25" t="str">
+      <x:c r="D7" s="301" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="E7" s="25" t="str">
+      <x:c r="E7" s="301" t="str">
         <x:v>CH1·CH2 영점</x:v>
       </x:c>
-      <x:c r="F7" s="25" t="str">
+      <x:c r="F7" s="301" t="str">
         <x:v>0 입력 최대 오차</x:v>
       </x:c>
-      <x:c r="G7" s="25" t="str">
+      <x:c r="G7" s="301" t="str">
         <x:v>%FS</x:v>
       </x:c>
-      <x:c r="H7" s="59" t="n">
+      <x:c r="H7" s="309" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="I7" s="59" t="str">
+      <x:c r="I7" s="304" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J7" s="60" t="n">
+      <x:c r="J7" s="310" t="n">
         <x:v>0.041553</x:v>
       </x:c>
-      <x:c r="K7" s="60" t="n">
+      <x:c r="K7" s="310" t="n">
         <x:v>0.004694</x:v>
       </x:c>
-      <x:c r="L7" s="60" t="n">
+      <x:c r="L7" s="310" t="n">
         <x:v>0.041553</x:v>
       </x:c>
-      <x:c r="M7" s="60" t="n">
+      <x:c r="M7" s="310" t="n">
         <x:v>0.023963</x:v>
       </x:c>
-      <x:c r="N7" s="60" t="n">
+      <x:c r="N7" s="310" t="n">
         <x:v>0.015</x:v>
       </x:c>
-      <x:c r="O7" s="60" t="n">
+      <x:c r="O7" s="310" t="n">
         <x:v>3001</x:v>
       </x:c>
-      <x:c r="P7" s="57" t="str">
+      <x:c r="P7" s="303" t="str">
         <x:v>0 V / 0 A; CH1+CH2; final 5 min</x:v>
       </x:c>
-      <x:c r="Q7" s="25" t="str">
+      <x:c r="Q7" s="311" t="str">
         <x:f>IF(OR(H7="",I7="",J7=""),"INPUT",IF(I7="최대",IF(J7&lt;=H7,"PASS","FAIL"),IF(I7="최소",IF(J7&gt;=H7,"PASS","FAIL"),IF(I7="일치",IF(J7=H7,"PASS","FAIL"),"CHECK"))))</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R7" s="57" t="str">
+      <x:c r="R7" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S7" s="57" t="str">
+      <x:c r="S7" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T7" s="57" t="str">
+      <x:c r="T7" s="303" t="str">
         <x:v>CH1 I +12.466 mA, V -11.734 mV; CH2 I +11.331 mA, V +29.593 mV. OFFSET_UNITS 적용.</x:v>
       </x:c>
-      <x:c r="U7" s="57" t="str">
+      <x:c r="U7" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_091833_148511.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="25" t="str">
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="308" t="str">
         <x:v>A-02</x:v>
       </x:c>
-      <x:c r="B8" s="58" t="n">
+      <x:c r="B8" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C8" s="57" t="str">
+      <x:c r="C8" s="303" t="str">
         <x:v>4b7b1d3 (pre-gain)</x:v>
       </x:c>
-      <x:c r="D8" s="25" t="str">
+      <x:c r="D8" s="301" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="E8" s="25" t="str">
+      <x:c r="E8" s="301" t="str">
         <x:v>CH1·CH2 gain</x:v>
       </x:c>
-      <x:c r="F8" s="25" t="str">
+      <x:c r="F8" s="301" t="str">
         <x:v>100% span 최대 오차</x:v>
       </x:c>
-      <x:c r="G8" s="25" t="str">
+      <x:c r="G8" s="301" t="str">
         <x:v>%FS</x:v>
       </x:c>
-      <x:c r="H8" s="59" t="n">
+      <x:c r="H8" s="309" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="I8" s="59" t="str">
+      <x:c r="I8" s="304" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J8" s="60" t="n">
+      <x:c r="J8" s="310" t="n">
         <x:v>10.4435</x:v>
       </x:c>
-      <x:c r="K8" s="60" t="n">
+      <x:c r="K8" s="310" t="n">
         <x:v>3.3202</x:v>
       </x:c>
-      <x:c r="L8" s="60" t="n">
+      <x:c r="L8" s="310" t="n">
         <x:v>10.4435</x:v>
       </x:c>
-      <x:c r="M8" s="60" t="n">
+      <x:c r="M8" s="310" t="n">
         <x:v>7.3837</x:v>
       </x:c>
-      <x:c r="N8" s="60" t="n">
+      <x:c r="N8" s="310" t="n">
         <x:v>3.195</x:v>
       </x:c>
-      <x:c r="O8" s="60" t="n">
+      <x:c r="O8" s="310" t="n">
         <x:v>16577</x:v>
       </x:c>
-      <x:c r="P8" s="57" t="str">
+      <x:c r="P8" s="303" t="str">
         <x:v>11 V / 5 A; CH1+CH2; user-induced input interruption excluded</x:v>
       </x:c>
-      <x:c r="Q8" s="25" t="str">
+      <x:c r="Q8" s="311" t="str">
         <x:f>"FIELD"</x:f>
         <x:v>FIELD</x:v>
       </x:c>
-      <x:c r="R8" s="57" t="str">
+      <x:c r="R8" s="312" t="str">
         <x:v>현장 검증 이관</x:v>
       </x:c>
-      <x:c r="S8" s="57" t="str">
+      <x:c r="S8" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T8" s="57" t="str">
+      <x:c r="T8" s="303" t="str">
         <x:v>벤치 합격 판정에서는 제외. 보정 전 데이터와 SCALE_TRIM 적용 이력은 보존하며 실제 운용 환경에서 검증.</x:v>
       </x:c>
-      <x:c r="U8" s="57" t="str">
+      <x:c r="U8" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="25" t="str">
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="308" t="str">
         <x:v>A-03</x:v>
       </x:c>
-      <x:c r="B9" s="58" t="n">
+      <x:c r="B9" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C9" s="57" t="str">
+      <x:c r="C9" s="303" t="str">
         <x:v>f9ceb9a</x:v>
       </x:c>
-      <x:c r="D9" s="25" t="str">
+      <x:c r="D9" s="301" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="E9" s="25" t="str">
+      <x:c r="E9" s="301" t="str">
         <x:v>CH1·CH2 선형성</x:v>
       </x:c>
-      <x:c r="F9" s="25" t="str">
+      <x:c r="F9" s="301" t="str">
         <x:v>0/50/100% 최대 편차</x:v>
       </x:c>
-      <x:c r="G9" s="25" t="str">
+      <x:c r="G9" s="301" t="str">
         <x:v>%FS</x:v>
       </x:c>
-      <x:c r="H9" s="59" t="n">
+      <x:c r="H9" s="309" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I9" s="59" t="str">
+      <x:c r="I9" s="304" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J9" s="60" t="n">
+      <x:c r="J9" s="310" t="n">
         <x:v>0.2803</x:v>
       </x:c>
-      <x:c r="K9" s="60" t="n">
+      <x:c r="K9" s="310" t="n">
         <x:v>0.0098</x:v>
       </x:c>
-      <x:c r="L9" s="60" t="n">
+      <x:c r="L9" s="310" t="n">
         <x:v>0.2803</x:v>
       </x:c>
-      <x:c r="M9" s="60" t="n">
+      <x:c r="M9" s="310" t="n">
         <x:v>0.14135</x:v>
       </x:c>
-      <x:c r="N9" s="60" t="n">
+      <x:c r="N9" s="310" t="n">
         <x:v>0.1275</x:v>
       </x:c>
-      <x:c r="O9" s="60" t="n">
+      <x:c r="O9" s="310" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="P9" s="57" t="str">
+      <x:c r="P9" s="303" t="str">
         <x:v>CH1+CH2; CSV 구간 0 V / 약 5 V / 약 10 V</x:v>
       </x:c>
-      <x:c r="Q9" s="25" t="str">
+      <x:c r="Q9" s="311" t="str">
         <x:f>IF(OR(H9="",I9="",J9=""),"INPUT",IF(I9="최대",IF(J9&lt;=H9,"PASS","FAIL"),IF(I9="최소",IF(J9&gt;=H9,"PASS","FAIL"),IF(I9="일치",IF(J9=H9,"PASS","FAIL"),"CHECK"))))</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R9" s="57" t="str">
+      <x:c r="R9" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S9" s="57" t="str">
+      <x:c r="S9" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T9" s="57" t="str">
+      <x:c r="T9" s="303" t="str">
         <x:v>50% 점 편차: I1 0.2803%, V1 0.0184%, I2 0.2569%, V2 0.0098%FS. 절대 게인은 현장 검증 이관.</x:v>
       </x:c>
-      <x:c r="U9" s="57" t="str">
+      <x:c r="U9" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_103337_769201.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="25" t="str">
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="308" t="str">
         <x:v>A-04</x:v>
       </x:c>
-      <x:c r="B10" s="58" t="n">
+      <x:c r="B10" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C10" s="57" t="str">
+      <x:c r="C10" s="303" t="str">
         <x:v>4b7b1d3</x:v>
       </x:c>
-      <x:c r="D10" s="25" t="str">
+      <x:c r="D10" s="301" t="str">
         <x:v>계측 정확도</x:v>
       </x:c>
-      <x:c r="E10" s="25" t="str">
+      <x:c r="E10" s="301" t="str">
         <x:v>CH1·CH2 입력 노이즈</x:v>
       </x:c>
-      <x:c r="F10" s="25" t="str">
+      <x:c r="F10" s="301" t="str">
         <x:v>RMS noise</x:v>
       </x:c>
-      <x:c r="G10" s="25" t="str">
+      <x:c r="G10" s="301" t="str">
         <x:v>mV/mA</x:v>
       </x:c>
-      <x:c r="H10" s="59" t="n">
+      <x:c r="H10" s="309" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I10" s="59" t="str">
+      <x:c r="I10" s="304" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J10" s="60" t="n">
+      <x:c r="J10" s="310" t="n">
         <x:v>18.206</x:v>
       </x:c>
-      <x:c r="K10" s="60" t="n">
+      <x:c r="K10" s="310" t="n">
         <x:v>0.209</x:v>
       </x:c>
-      <x:c r="L10" s="60" t="n">
+      <x:c r="L10" s="310" t="n">
         <x:v>18.206</x:v>
       </x:c>
-      <x:c r="M10" s="60" t="n">
+      <x:c r="M10" s="310" t="n">
         <x:v>7.988</x:v>
       </x:c>
-      <x:c r="N10" s="60" t="n">
+      <x:c r="N10" s="310" t="n">
         <x:v>7.492</x:v>
       </x:c>
-      <x:c r="O10" s="60" t="n">
+      <x:c r="O10" s="310" t="n">
         <x:v>3001</x:v>
       </x:c>
-      <x:c r="P10" s="57" t="str">
+      <x:c r="P10" s="303" t="str">
         <x:v>11 V / 5 A; CH1+CH2; final stable 5 min</x:v>
       </x:c>
-      <x:c r="Q10" s="25" t="str">
+      <x:c r="Q10" s="311" t="str">
         <x:f>IF(OR(H10="",I10="",J10=""),"INPUT",IF(I10="최대",IF(J10&lt;=H10,"PASS","FAIL"),IF(I10="최소",IF(J10&gt;=H10,"PASS","FAIL"),IF(I10="일치",IF(J10=H10,"PASS","FAIL"),"CHECK"))))</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R10" s="57" t="str">
+      <x:c r="R10" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S10" s="57" t="str">
+      <x:c r="S10" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T10" s="57" t="str">
+      <x:c r="T10" s="303" t="str">
         <x:v>RMS: I1 0.209 mA, V1 13.141 mV, I2 0.397 mA, V2 18.206 mV (최대값 판정).</x:v>
       </x:c>
-      <x:c r="U10" s="57" t="str">
+      <x:c r="U10" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="25" t="str">
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="308" t="str">
         <x:v>T-01</x:v>
       </x:c>
-      <x:c r="B11" s="58" t="n">
+      <x:c r="B11" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C11" s="57" t="str">
+      <x:c r="C11" s="303" t="str">
         <x:v>4b7b1d3</x:v>
       </x:c>
-      <x:c r="D11" s="25" t="str">
+      <x:c r="D11" s="301" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
-      <x:c r="E11" s="25" t="str">
+      <x:c r="E11" s="301" t="str">
         <x:v>ADC 수집률</x:v>
       </x:c>
-      <x:c r="F11" s="25" t="str">
+      <x:c r="F11" s="301" t="str">
         <x:v>실제 sample rate</x:v>
       </x:c>
-      <x:c r="G11" s="25" t="str">
+      <x:c r="G11" s="301" t="str">
         <x:v>Hz</x:v>
       </x:c>
-      <x:c r="H11" s="59" t="n">
+      <x:c r="H11" s="309" t="n">
         <x:v>1980</x:v>
       </x:c>
-      <x:c r="I11" s="59" t="str">
+      <x:c r="I11" s="304" t="str">
         <x:v>최소</x:v>
       </x:c>
-      <x:c r="J11" s="60" t="n">
+      <x:c r="J11" s="310" t="n">
         <x:v>1999.931</x:v>
       </x:c>
-      <x:c r="K11" s="60"/>
-      <x:c r="L11" s="60"/>
-      <x:c r="M11" s="60" t="n">
+      <x:c r="K11" s="310"/>
+      <x:c r="L11" s="310"/>
+      <x:c r="M11" s="310" t="n">
         <x:v>1999.931</x:v>
       </x:c>
-      <x:c r="N11" s="60"/>
-      <x:c r="O11" s="60" t="n">
+      <x:c r="N11" s="310"/>
+      <x:c r="O11" s="310" t="n">
         <x:v>16621</x:v>
       </x:c>
-      <x:c r="P11" s="57" t="str">
+      <x:c r="P11" s="303" t="str">
         <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
-      <x:c r="Q11" s="25" t="str">
+      <x:c r="Q11" s="311" t="str">
         <x:f>IF(J11&gt;=H11,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R11" s="57" t="str">
+      <x:c r="R11" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S11" s="57" t="str">
+      <x:c r="S11" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T11" s="57" t="str">
+      <x:c r="T11" s="303" t="str">
         <x:v>PC/보드 시간 1:1, ADC 1,999.931 Hz</x:v>
       </x:c>
-      <x:c r="U11" s="57" t="str">
+      <x:c r="U11" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="25" t="str">
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="308" t="str">
         <x:v>T-02</x:v>
       </x:c>
-      <x:c r="B12" s="58" t="n">
+      <x:c r="B12" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C12" s="57" t="str">
+      <x:c r="C12" s="303" t="str">
         <x:v>4b7b1d3</x:v>
       </x:c>
-      <x:c r="D12" s="25" t="str">
+      <x:c r="D12" s="301" t="str">
         <x:v>시간 성능</x:v>
       </x:c>
-      <x:c r="E12" s="25" t="str">
+      <x:c r="E12" s="301" t="str">
         <x:v>DMA/링버퍼</x:v>
       </x:c>
-      <x:c r="F12" s="25" t="str">
+      <x:c r="F12" s="301" t="str">
         <x:v>dropped frames</x:v>
       </x:c>
-      <x:c r="G12" s="25" t="str">
+      <x:c r="G12" s="301" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H12" s="59" t="n">
+      <x:c r="H12" s="309" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I12" s="59" t="str">
+      <x:c r="I12" s="304" t="str">
         <x:v>일치</x:v>
       </x:c>
-      <x:c r="J12" s="60" t="n">
+      <x:c r="J12" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K12" s="60" t="n">
+      <x:c r="K12" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L12" s="60" t="n">
+      <x:c r="L12" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M12" s="60" t="n">
+      <x:c r="M12" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N12" s="60" t="n">
+      <x:c r="N12" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O12" s="60" t="n">
+      <x:c r="O12" s="310" t="n">
         <x:v>16621</x:v>
       </x:c>
-      <x:c r="P12" s="57" t="str">
+      <x:c r="P12" s="303" t="str">
         <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
-      <x:c r="Q12" s="25" t="str">
+      <x:c r="Q12" s="311" t="str">
         <x:f>IF(J12=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R12" s="57" t="str">
+      <x:c r="R12" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S12" s="57" t="str">
+      <x:c r="S12" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T12" s="57" t="str">
+      <x:c r="T12" s="303" t="str">
         <x:v>27.7 min 동안 모든 드롭 원인 0</x:v>
       </x:c>
-      <x:c r="U12" s="57" t="str">
+      <x:c r="U12" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="25"/>
-      <x:c r="B13" s="58"/>
-      <x:c r="C13" s="57"/>
-      <x:c r="D13" s="25"/>
-      <x:c r="E13" s="25"/>
-      <x:c r="F13" s="25"/>
-      <x:c r="G13" s="25"/>
-      <x:c r="H13" s="59"/>
-      <x:c r="I13" s="59"/>
-      <x:c r="J13" s="60"/>
-      <x:c r="K13" s="60"/>
-      <x:c r="L13" s="60"/>
-      <x:c r="M13" s="60"/>
-      <x:c r="N13" s="60"/>
-      <x:c r="O13" s="60"/>
-      <x:c r="P13" s="57"/>
-      <x:c r="Q13" s="25"/>
-      <x:c r="R13" s="57"/>
-      <x:c r="S13" s="57"/>
-      <x:c r="T13" s="57"/>
-      <x:c r="U13" s="57"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="25" t="str">
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="308"/>
+      <x:c r="B13" s="302"/>
+      <x:c r="C13" s="303"/>
+      <x:c r="D13" s="301"/>
+      <x:c r="E13" s="301"/>
+      <x:c r="F13" s="301"/>
+      <x:c r="G13" s="301"/>
+      <x:c r="H13" s="309"/>
+      <x:c r="I13" s="304"/>
+      <x:c r="J13" s="310"/>
+      <x:c r="K13" s="310"/>
+      <x:c r="L13" s="310"/>
+      <x:c r="M13" s="310"/>
+      <x:c r="N13" s="310"/>
+      <x:c r="O13" s="310"/>
+      <x:c r="P13" s="303"/>
+      <x:c r="Q13" s="311"/>
+      <x:c r="R13" s="312"/>
+      <x:c r="S13" s="303"/>
+      <x:c r="T13" s="303"/>
+      <x:c r="U13" s="303"/>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="308" t="str">
         <x:v>N-01</x:v>
       </x:c>
-      <x:c r="B14" s="58" t="n">
+      <x:c r="B14" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C14" s="57" t="str">
+      <x:c r="C14" s="303" t="str">
         <x:v>4b7b1d3</x:v>
       </x:c>
-      <x:c r="D14" s="25" t="str">
+      <x:c r="D14" s="301" t="str">
         <x:v>통신</x:v>
       </x:c>
-      <x:c r="E14" s="25" t="str">
+      <x:c r="E14" s="301" t="str">
         <x:v>UDP 전송률</x:v>
       </x:c>
-      <x:c r="F14" s="25" t="str">
+      <x:c r="F14" s="301" t="str">
         <x:v>송신 주기</x:v>
       </x:c>
-      <x:c r="G14" s="25" t="str">
+      <x:c r="G14" s="301" t="str">
         <x:v>ms</x:v>
       </x:c>
-      <x:c r="H14" s="59" t="n">
+      <x:c r="H14" s="309" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="I14" s="59" t="str">
+      <x:c r="I14" s="304" t="str">
         <x:v>일치</x:v>
       </x:c>
-      <x:c r="J14" s="60" t="n">
+      <x:c r="J14" s="310" t="n">
         <x:v>99.999</x:v>
       </x:c>
-      <x:c r="K14" s="60" t="n">
+      <x:c r="K14" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L14" s="60" t="n">
+      <x:c r="L14" s="310" t="n">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="M14" s="60" t="n">
+      <x:c r="M14" s="310" t="n">
         <x:v>99.999</x:v>
       </x:c>
-      <x:c r="N14" s="60" t="n">
+      <x:c r="N14" s="310" t="n">
         <x:v>1.264</x:v>
       </x:c>
-      <x:c r="O14" s="60" t="n">
+      <x:c r="O14" s="310" t="n">
         <x:v>16620</x:v>
       </x:c>
-      <x:c r="P14" s="57" t="str">
+      <x:c r="P14" s="303" t="str">
         <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
-      <x:c r="Q14" s="25" t="str">
+      <x:c r="Q14" s="311" t="str">
         <x:f>IF(AND(J14&gt;=95,J14&lt;=105),"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R14" s="57" t="str">
+      <x:c r="R14" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S14" s="57" t="str">
+      <x:c r="S14" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T14" s="57" t="str">
+      <x:c r="T14" s="303" t="str">
         <x:v>평균 99.999 ms; PC 수신 타임스탬프 최대 gap 218 ms</x:v>
       </x:c>
-      <x:c r="U14" s="57" t="str">
+      <x:c r="U14" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="25" t="str">
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="308" t="str">
         <x:v>N-02</x:v>
       </x:c>
-      <x:c r="B15" s="58" t="n">
+      <x:c r="B15" s="302" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="C15" s="57" t="str">
+      <x:c r="C15" s="303" t="str">
         <x:v>4b7b1d3</x:v>
       </x:c>
-      <x:c r="D15" s="25" t="str">
+      <x:c r="D15" s="301" t="str">
         <x:v>통신</x:v>
       </x:c>
-      <x:c r="E15" s="25" t="str">
+      <x:c r="E15" s="301" t="str">
         <x:v>UDP 손실</x:v>
       </x:c>
-      <x:c r="F15" s="25" t="str">
+      <x:c r="F15" s="301" t="str">
         <x:v>sequence gap rate</x:v>
       </x:c>
-      <x:c r="G15" s="25" t="str">
+      <x:c r="G15" s="301" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="H15" s="59" t="n">
+      <x:c r="H15" s="309" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="I15" s="59" t="str">
+      <x:c r="I15" s="304" t="str">
         <x:v>최대</x:v>
       </x:c>
-      <x:c r="J15" s="60" t="n">
+      <x:c r="J15" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K15" s="60" t="n">
+      <x:c r="K15" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L15" s="60" t="n">
+      <x:c r="L15" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M15" s="60" t="n">
+      <x:c r="M15" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N15" s="60" t="n">
+      <x:c r="N15" s="310" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O15" s="60" t="n">
+      <x:c r="O15" s="310" t="n">
         <x:v>16620</x:v>
       </x:c>
-      <x:c r="P15" s="57" t="str">
+      <x:c r="P15" s="303" t="str">
         <x:v>11 V / 5 A; CH1+CH2; 27.7 min, pre-gain trim</x:v>
       </x:c>
-      <x:c r="Q15" s="25" t="str">
+      <x:c r="Q15" s="311" t="str">
         <x:f>IF(J15&lt;=H15,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="R15" s="57" t="str">
+      <x:c r="R15" s="312" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="S15" s="57" t="str">
+      <x:c r="S15" s="303" t="str">
         <x:v>지명환</x:v>
       </x:c>
-      <x:c r="T15" s="57" t="str">
+      <x:c r="T15" s="303" t="str">
         <x:v>ADC sequence 간격 최대 201 (정상 200)으로 UDP 손실 0%. PC 수신 gap 218 ms 1회는 호스트 지연으로 분리.</x:v>
       </x:c>
-      <x:c r="U15" s="57" t="str">
+      <x:c r="U15" s="303" t="str">
         <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="25"/>
-      <x:c r="B16" s="58"/>
-      <x:c r="C16" s="57"/>
-      <x:c r="D16" s="25"/>
-      <x:c r="E16" s="25"/>
-      <x:c r="F16" s="25"/>
-      <x:c r="G16" s="25"/>
-      <x:c r="H16" s="59"/>
-      <x:c r="I16" s="59"/>
-      <x:c r="J16" s="60"/>
-      <x:c r="K16" s="60"/>
-      <x:c r="L16" s="60"/>
-      <x:c r="M16" s="60"/>
-      <x:c r="N16" s="60"/>
-      <x:c r="O16" s="60"/>
-      <x:c r="P16" s="57"/>
-      <x:c r="Q16" s="25"/>
-      <x:c r="R16" s="57"/>
-      <x:c r="S16" s="57"/>
-      <x:c r="T16" s="57"/>
-      <x:c r="U16" s="57"/>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="308" t="str">
+        <x:v>L-01</x:v>
+      </x:c>
+      <x:c r="B16" s="302" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C16" s="303" t="str">
+        <x:v>4b7b1d3</x:v>
+      </x:c>
+      <x:c r="D16" s="301" t="str">
+        <x:v>장시간 안정성</x:v>
+      </x:c>
+      <x:c r="E16" s="301" t="str">
+        <x:v>양 채널 부하 안정성</x:v>
+      </x:c>
+      <x:c r="F16" s="301" t="str">
+        <x:v>연속 운전</x:v>
+      </x:c>
+      <x:c r="G16" s="301" t="str">
+        <x:v>min</x:v>
+      </x:c>
+      <x:c r="H16" s="309" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="I16" s="304" t="str">
+        <x:v>최소</x:v>
+      </x:c>
+      <x:c r="J16" s="310" t="n">
+        <x:v>27.7</x:v>
+      </x:c>
+      <x:c r="K16" s="310" t="n">
+        <x:v>27.7</x:v>
+      </x:c>
+      <x:c r="L16" s="310" t="n">
+        <x:v>27.7</x:v>
+      </x:c>
+      <x:c r="M16" s="310" t="n">
+        <x:v>27.7</x:v>
+      </x:c>
+      <x:c r="N16" s="310"/>
+      <x:c r="O16" s="310" t="n">
+        <x:v>16621</x:v>
+      </x:c>
+      <x:c r="P16" s="303" t="str">
+        <x:v>CH1+CH2 11 V / 5 A; 27.7 min; pre-gain trim</x:v>
+      </x:c>
+      <x:c r="Q16" s="311" t="str">
+        <x:f>IF(J16&gt;=H16,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="R16" s="312" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="S16" s="303" t="str">
+        <x:v>지명환</x:v>
+      </x:c>
+      <x:c r="T16" s="303" t="str">
+        <x:v>27.7분 동안 ADC 1,999.931 Hz, dropped/CRC/SPI/DAC 오류 0, UDP sequence loss 0%.</x:v>
+      </x:c>
+      <x:c r="U16" s="303" t="str">
+        <x:v>logs/cosmoke_capture_20260820_094031_980220.csv</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="25"/>
@@ -3131,6 +4024,10 @@
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="FAIL"/>
     <x:cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="INPUT"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="Q6:Q16">
+    <x:cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="PASS"/>
+    <x:cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="FIELD"/>
+  </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="R6:R20">
       <x:formula1>"미실행,진행 중,완료,보류"</x:formula1>
@@ -3147,259 +4044,279 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="43" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="270" t="str">
         <x:v>성능 튜닝 프로파일</x:v>
       </x:c>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="227"/>
+      <x:c r="B2" s="227"/>
+      <x:c r="C2" s="227"/>
+      <x:c r="D2" s="227"/>
+      <x:c r="E2" s="227"/>
+      <x:c r="F2" s="227"/>
+      <x:c r="G2" s="227"/>
+      <x:c r="H2" s="227"/>
+    </x:row>
     <x:row r="3">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="267" t="str">
         <x:v>설정 변경은 한 번에 하나씩 시험하고, 결과는 Test Log에 연결해 근거를 남기십시오. Current 값은 현재 펌웨어 설정 기준입니다.</x:v>
       </x:c>
-      <x:c r="B3" s="6"/>
-      <x:c r="C3" s="6"/>
-      <x:c r="D3" s="6"/>
-      <x:c r="E3" s="6"/>
-      <x:c r="F3" s="6"/>
-      <x:c r="G3" s="6"/>
-      <x:c r="H3" s="6"/>
+      <x:c r="B3" s="267"/>
+      <x:c r="C3" s="267"/>
+      <x:c r="D3" s="267"/>
+      <x:c r="E3" s="267"/>
+      <x:c r="F3" s="267"/>
+      <x:c r="G3" s="267"/>
+      <x:c r="H3" s="267"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="227"/>
+      <x:c r="B4" s="227"/>
+      <x:c r="C4" s="227"/>
+      <x:c r="D4" s="227"/>
+      <x:c r="E4" s="227"/>
+      <x:c r="F4" s="227"/>
+      <x:c r="G4" s="227"/>
+      <x:c r="H4" s="227"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="23" t="str">
+      <x:c r="A5" s="272" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B5" s="23" t="str">
+      <x:c r="B5" s="272" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C5" s="23" t="str">
+      <x:c r="C5" s="272" t="str">
         <x:v>Debug 제안</x:v>
       </x:c>
-      <x:c r="D5" s="23" t="str">
+      <x:c r="D5" s="272" t="str">
         <x:v>Bench 제안</x:v>
       </x:c>
-      <x:c r="E5" s="23" t="str">
+      <x:c r="E5" s="272" t="str">
         <x:v>Production 제안</x:v>
       </x:c>
-      <x:c r="F5" s="23" t="str">
+      <x:c r="F5" s="272" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="G5" s="23" t="str">
+      <x:c r="G5" s="272" t="str">
         <x:v>영향</x:v>
       </x:c>
-      <x:c r="H5" s="23" t="str">
+      <x:c r="H5" s="272" t="str">
         <x:v>검증 지표</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="55" t="str">
+    <x:row r="6" ht="32" customHeight="1">
+      <x:c r="A6" s="278" t="str">
         <x:v>APP_CHx_FILTER_ALPHA</x:v>
       </x:c>
-      <x:c r="B6" s="61" t="n">
+      <x:c r="B6" s="315" t="n">
         <x:v>0.05</x:v>
       </x:c>
-      <x:c r="C6" s="61" t="n">
+      <x:c r="C6" s="315" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="D6" s="61" t="n">
+      <x:c r="D6" s="315" t="n">
         <x:v>0.05</x:v>
       </x:c>
-      <x:c r="E6" s="61" t="n">
+      <x:c r="E6" s="315" t="n">
         <x:v>0.02</x:v>
       </x:c>
-      <x:c r="F6" s="55" t="str">
+      <x:c r="F6" s="275" t="str">
         <x:v>ratio</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="275" t="str">
         <x:v>값이 작을수록 노이즈 감소·응답 지연 증가</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="275" t="str">
         <x:v>RMS noise / DAC settling</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="55" t="str">
+    <x:row r="7" ht="32" customHeight="1">
+      <x:c r="A7" s="278" t="str">
         <x:v>APP_DAC_UPDATE_PERIOD_MS</x:v>
       </x:c>
-      <x:c r="B7" s="61" t="n">
+      <x:c r="B7" s="315" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C7" s="61" t="n">
+      <x:c r="C7" s="315" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D7" s="61" t="n">
+      <x:c r="D7" s="315" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E7" s="61" t="n">
+      <x:c r="E7" s="315" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F7" s="55" t="str">
+      <x:c r="F7" s="275" t="str">
         <x:v>ms</x:v>
       </x:c>
-      <x:c r="G7" s="55" t="str">
+      <x:c r="G7" s="275" t="str">
         <x:v>작을수록 DAC 응답 향상·SPI 부하 증가</x:v>
       </x:c>
-      <x:c r="H7" s="55" t="str">
+      <x:c r="H7" s="275" t="str">
         <x:v>dropped frames / response time</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="55" t="str">
+    <x:row r="8" ht="32" customHeight="1">
+      <x:c r="A8" s="278" t="str">
         <x:v>APP_TELEMETRY_PERIOD_MS</x:v>
       </x:c>
-      <x:c r="B8" s="61" t="n">
+      <x:c r="B8" s="315" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C8" s="61" t="n">
+      <x:c r="C8" s="315" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D8" s="61" t="n">
+      <x:c r="D8" s="315" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E8" s="61" t="n">
+      <x:c r="E8" s="315" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="F8" s="55" t="str">
+      <x:c r="F8" s="275" t="str">
         <x:v>ms</x:v>
       </x:c>
-      <x:c r="G8" s="55" t="str">
+      <x:c r="G8" s="275" t="str">
         <x:v>작을수록 관측성 향상·LAN/UART 부하 증가</x:v>
       </x:c>
-      <x:c r="H8" s="55" t="str">
+      <x:c r="H8" s="275" t="str">
         <x:v>UDP loss / jitter</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="55" t="str">
+    <x:row r="9" ht="32" customHeight="1">
+      <x:c r="A9" s="278" t="str">
         <x:v>APP_ADC_RING_CAPACITY</x:v>
       </x:c>
-      <x:c r="B9" s="61" t="n">
+      <x:c r="B9" s="315" t="n">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C9" s="61" t="n">
+      <x:c r="C9" s="315" t="n">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="D9" s="61" t="n">
+      <x:c r="D9" s="315" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="E9" s="61" t="n">
+      <x:c r="E9" s="315" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F9" s="55" t="str">
+      <x:c r="F9" s="275" t="str">
         <x:v>frames</x:v>
       </x:c>
-      <x:c r="G9" s="55" t="str">
+      <x:c r="G9" s="275" t="str">
         <x:v>증가 시 task 지연 흡수·RAM 사용 증가</x:v>
       </x:c>
-      <x:c r="H9" s="55" t="str">
+      <x:c r="H9" s="275" t="str">
         <x:v>dropped frames / RAM</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="55" t="str">
+    <x:row r="10" ht="32" customHeight="1">
+      <x:c r="A10" s="278" t="str">
         <x:v>APP_ADC_NO_PROGRESS_TIMEOUT_MS</x:v>
       </x:c>
-      <x:c r="B10" s="61" t="n">
+      <x:c r="B10" s="315" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="C10" s="61" t="n">
+      <x:c r="C10" s="315" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="D10" s="61" t="n">
+      <x:c r="D10" s="315" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="E10" s="61" t="n">
+      <x:c r="E10" s="315" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="F10" s="55" t="str">
+      <x:c r="F10" s="275" t="str">
         <x:v>ms</x:v>
       </x:c>
-      <x:c r="G10" s="55" t="str">
+      <x:c r="G10" s="275" t="str">
         <x:v>작을수록 빠른 fault 감지·false recovery 위험</x:v>
       </x:c>
-      <x:c r="H10" s="55" t="str">
+      <x:c r="H10" s="275" t="str">
         <x:v>fault transition time</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="55" t="str">
+    <x:row r="11" ht="32" customHeight="1">
+      <x:c r="A11" s="278" t="str">
         <x:v>APP_ADC_MAX_CONSECUTIVE_CRC_ERRORS</x:v>
       </x:c>
-      <x:c r="B11" s="61" t="n">
+      <x:c r="B11" s="315" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C11" s="61" t="n">
+      <x:c r="C11" s="315" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D11" s="61" t="n">
+      <x:c r="D11" s="315" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="E11" s="61" t="n">
+      <x:c r="E11" s="315" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F11" s="55" t="str">
+      <x:c r="F11" s="275" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="G11" s="55" t="str">
+      <x:c r="G11" s="275" t="str">
         <x:v>작을수록 빠른 CRC fault 감지</x:v>
       </x:c>
-      <x:c r="H11" s="55" t="str">
+      <x:c r="H11" s="275" t="str">
         <x:v>noise fault injection</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="55" t="str">
+    <x:row r="12" ht="32" customHeight="1">
+      <x:c r="A12" s="278" t="str">
         <x:v>APP_WARMUP_TIMEOUT_MS</x:v>
       </x:c>
-      <x:c r="B12" s="61" t="n">
+      <x:c r="B12" s="315" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="C12" s="61" t="n">
+      <x:c r="C12" s="315" t="n">
         <x:v>3000</x:v>
       </x:c>
-      <x:c r="D12" s="61" t="n">
+      <x:c r="D12" s="315" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="E12" s="61" t="n">
+      <x:c r="E12" s="315" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="F12" s="55" t="str">
+      <x:c r="F12" s="275" t="str">
         <x:v>ms</x:v>
       </x:c>
-      <x:c r="G12" s="55" t="str">
+      <x:c r="G12" s="275" t="str">
         <x:v>초기 안정화 여유와 startup time tradeoff</x:v>
       </x:c>
-      <x:c r="H12" s="55" t="str">
+      <x:c r="H12" s="275" t="str">
         <x:v>WARMUP→ACTIVE time</x:v>
       </x:c>
     </x:row>
@@ -3418,12 +4335,12 @@
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="53" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="31" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -3518,421 +4435,341 @@
       <x:c r="G9" s="55"/>
       <x:c r="H9" s="55"/>
     </x:row>
-    <x:row r="11" ht="32" customHeight="1">
-      <x:c r="A11" s="81" t="str">
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="258" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B11" s="81" t="str">
+      <x:c r="B11" s="258" t="str">
         <x:v>시험</x:v>
       </x:c>
-      <x:c r="C11" s="81" t="str">
+      <x:c r="C11" s="258" t="str">
         <x:v>사전 준비/장비</x:v>
       </x:c>
-      <x:c r="D11" s="81" t="str">
+      <x:c r="D11" s="258" t="str">
         <x:v>절차</x:v>
       </x:c>
-      <x:c r="E11" s="81" t="str">
+      <x:c r="E11" s="258" t="str">
         <x:v>기록값·CSV 확인</x:v>
       </x:c>
-      <x:c r="F11" s="81" t="str">
+      <x:c r="F11" s="258" t="str">
         <x:v>판정 기준</x:v>
       </x:c>
-      <x:c r="G11" s="81" t="str">
+      <x:c r="G11" s="258" t="str">
         <x:v>안전·주의</x:v>
       </x:c>
-      <x:c r="H11" s="81" t="str">
+      <x:c r="H11" s="258" t="str">
         <x:v>Test Log 작성</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="72" customHeight="1">
-      <x:c r="A12" s="85" t="str">
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="279" t="str">
         <x:v>F-01</x:v>
       </x:c>
-      <x:c r="B12" s="82" t="str">
+      <x:c r="B12" s="275" t="str">
         <x:v>부팅 상태 전이</x:v>
       </x:c>
-      <x:c r="C12" s="82" t="str">
+      <x:c r="C12" s="275" t="str">
         <x:v>UART/UDP 로그, 스톱워치</x:v>
       </x:c>
-      <x:c r="D12" s="82" t="str">
-        <x:v>전원을 3회 재인가합니다. 각 회차에서 WARMUP 표시부터 ACTIVE/OK까지 시간을 측정합니다.</x:v>
-      </x:c>
-      <x:c r="E12" s="82" t="str">
-        <x:v>CSV의 received_at·device_ms, WARMUP/MUTED 플래그, 첫 ACTIVE 프레임</x:v>
-      </x:c>
-      <x:c r="F12" s="87" t="str">
-        <x:v>2 s 이내</x:v>
-      </x:c>
-      <x:c r="G12" s="82" t="str">
+      <x:c r="D12" s="275" t="str">
+        <x:v>전원을 3회 재인가합니다. 매 회 WARMUP 표시부터 ACTIVE/OK까지 시간을 측정합니다.</x:v>
+      </x:c>
+      <x:c r="E12" s="275" t="str">
+        <x:v>CSV의 received_at·device_ms, 첫 ACTIVE 프레임</x:v>
+      </x:c>
+      <x:c r="F12" s="323" t="str">
+        <x:v>3 s 이내</x:v>
+      </x:c>
+      <x:c r="G12" s="275" t="str">
         <x:v>실부하 연결 전 수행</x:v>
       </x:c>
-      <x:c r="H12" s="82" t="str">
-        <x:v>측정값=최대 전이시간, 샘플 수=3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="72" customHeight="1">
-      <x:c r="A13" s="85" t="str">
+      <x:c r="H12" s="275" t="str">
+        <x:v>측정값=최대 전이 시간, 샘플 수=3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58" customHeight="1">
+      <x:c r="A13" s="279" t="str">
         <x:v>A-01</x:v>
       </x:c>
-      <x:c r="B13" s="82" t="str">
+      <x:c r="B13" s="275" t="str">
         <x:v>영점 오차</x:v>
       </x:c>
-      <x:c r="C13" s="82" t="str">
+      <x:c r="C13" s="275" t="str">
         <x:v>정밀 DMM, 입력 단락/0 기준</x:v>
       </x:c>
-      <x:c r="D13" s="82" t="str">
-        <x:v>채널별 0 입력을 10분 유지하고 안정화 후 100개 이상 프레임을 캡처합니다.</x:v>
-      </x:c>
-      <x:c r="E13" s="82" t="str">
-        <x:v>채널별 평균·최대 절대 오차, 필터 alpha, CSV 경로</x:v>
-      </x:c>
-      <x:c r="F13" s="87" t="str">
+      <x:c r="D13" s="275" t="str">
+        <x:v>채널별 0 입력을 5분 이상 유지하고 안정화 후 100프레임 이상을 분석합니다.</x:v>
+      </x:c>
+      <x:c r="E13" s="275" t="str">
+        <x:v>채널별 평균·최대 절대 오차, CSV 경로</x:v>
+      </x:c>
+      <x:c r="F13" s="323" t="str">
         <x:v>0.2 %FS 이하</x:v>
       </x:c>
-      <x:c r="G13" s="82" t="str">
-        <x:v>입력 단락 조건을 명확히 기록</x:v>
-      </x:c>
-      <x:c r="H13" s="82" t="str">
+      <x:c r="G13" s="275" t="str">
+        <x:v>입력 단락 조건과 필터 설정을 기록</x:v>
+      </x:c>
+      <x:c r="H13" s="275" t="str">
         <x:v>측정값=최대 절대 오차</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="72" customHeight="1">
-      <x:c r="A14" s="85" t="str">
+    <x:row r="14" ht="58" customHeight="1">
+      <x:c r="A14" s="279" t="str">
         <x:v>A-02</x:v>
       </x:c>
-      <x:c r="B14" s="82" t="str">
-        <x:v>Gain 오차</x:v>
-      </x:c>
-      <x:c r="C14" s="82" t="str">
+      <x:c r="B14" s="275" t="str">
+        <x:v>절대 gain 확인</x:v>
+      </x:c>
+      <x:c r="C14" s="275" t="str">
         <x:v>정밀 전압/전류원, DMM</x:v>
       </x:c>
-      <x:c r="D14" s="82" t="str">
+      <x:c r="D14" s="275" t="str">
         <x:v>0/50/100 %FS 기준점을 순서대로 인가하고 각 점에서 30초 이상 기록합니다.</x:v>
       </x:c>
-      <x:c r="E14" s="82" t="str">
+      <x:c r="E14" s="275" t="str">
         <x:v>기준값·표시 평균·오차(%FS), 보정 전/후 CSV</x:v>
       </x:c>
-      <x:c r="F14" s="87" t="str">
+      <x:c r="F14" s="323" t="str">
         <x:v>0.5 %FS 이하</x:v>
       </x:c>
-      <x:c r="G14" s="82" t="str">
-        <x:v>허용 입력 범위를 넘지 않음</x:v>
-      </x:c>
-      <x:c r="H14" s="82" t="str">
-        <x:v>측정값=100 %FS 오차</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="72" customHeight="1">
-      <x:c r="A15" s="85" t="str">
+      <x:c r="G14" s="275" t="str">
+        <x:v>현장 계측 환경에서 최종 검증</x:v>
+      </x:c>
+      <x:c r="H14" s="275" t="str">
+        <x:v>Result=FIELD로 이관 기록</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="279" t="str">
         <x:v>A-03</x:v>
       </x:c>
-      <x:c r="B15" s="82" t="str">
+      <x:c r="B15" s="275" t="str">
         <x:v>선형성</x:v>
       </x:c>
-      <x:c r="C15" s="82" t="str">
+      <x:c r="C15" s="275" t="str">
         <x:v>정밀 전압/전류원</x:v>
       </x:c>
-      <x:c r="D15" s="82" t="str">
-        <x:v>0/25/50/75/100 %FS를 상승·하강 방향으로 인가합니다.</x:v>
-      </x:c>
-      <x:c r="E15" s="82" t="str">
-        <x:v>각 점 평균과 직선 대비 최대 편차</x:v>
-      </x:c>
-      <x:c r="F15" s="87" t="str">
+      <x:c r="D15" s="275" t="str">
+        <x:v>0/50/100 %FS를 상승·하강 방향으로 인가합니다.</x:v>
+      </x:c>
+      <x:c r="E15" s="275" t="str">
+        <x:v>각 점 평균값과 직선 대비 최대 편차</x:v>
+      </x:c>
+      <x:c r="F15" s="323" t="str">
         <x:v>1.0 %FS 이하</x:v>
       </x:c>
-      <x:c r="G15" s="82" t="str">
+      <x:c r="G15" s="275" t="str">
         <x:v>히스테리시스는 비고에 별도 기록</x:v>
       </x:c>
-      <x:c r="H15" s="82" t="str">
+      <x:c r="H15" s="275" t="str">
         <x:v>측정값=최대 편차</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="72" customHeight="1">
-      <x:c r="A16" s="85" t="str">
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="279" t="str">
         <x:v>A-04</x:v>
       </x:c>
-      <x:c r="B16" s="82" t="str">
+      <x:c r="B16" s="275" t="str">
         <x:v>입력 노이즈</x:v>
       </x:c>
-      <x:c r="C16" s="82" t="str">
+      <x:c r="C16" s="275" t="str">
         <x:v>차폐 입력/고정 기준원, CSV</x:v>
       </x:c>
-      <x:c r="D16" s="82" t="str">
-        <x:v>고정 입력에서 최소 10분 캡처합니다. 필요 시 필터 alpha를 한 값씩만 변경해 비교합니다.</x:v>
-      </x:c>
-      <x:c r="E16" s="82" t="str">
-        <x:v>평균·표준편차·peak-to-peak, CSV sequence gap</x:v>
-      </x:c>
-      <x:c r="F16" s="87" t="str">
+      <x:c r="D16" s="275" t="str">
+        <x:v>고정 입력에서 5분 이상 캡처합니다. 필요 시 필터 alpha를 한 값씩만 변경해 비교합니다.</x:v>
+      </x:c>
+      <x:c r="E16" s="275" t="str">
+        <x:v>RMS·표준편차·peak-to-peak, CSV sequence gap</x:v>
+      </x:c>
+      <x:c r="F16" s="323" t="str">
         <x:v>50 mV/mA 이하</x:v>
       </x:c>
-      <x:c r="G16" s="82" t="str">
+      <x:c r="G16" s="275" t="str">
         <x:v>전원·접지·케이블 상태 기록</x:v>
       </x:c>
-      <x:c r="H16" s="82" t="str">
-        <x:v>측정값=RMS 또는 표준편차 기준값</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="72" customHeight="1">
-      <x:c r="A17" s="85" t="str">
+      <x:c r="H16" s="275" t="str">
+        <x:v>측정값=RMS 또는 표준편차</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="279" t="str">
         <x:v>T-01</x:v>
       </x:c>
-      <x:c r="B17" s="82" t="str">
+      <x:c r="B17" s="275" t="str">
         <x:v>ADC 수집률</x:v>
       </x:c>
-      <x:c r="C17" s="82" t="str">
-        <x:v>logic analyzer 또는 PC CSV</x:v>
-      </x:c>
-      <x:c r="D17" s="82" t="str">
-        <x:v>정상 입력에서 1분 이상 캡처하고 sequence/device_ms 변화로 실제 수집률을 계산합니다.</x:v>
-      </x:c>
-      <x:c r="E17" s="82" t="str">
-        <x:v>프레임 수 ÷ 경과시간, dropped, CRC/SPI 오류</x:v>
-      </x:c>
-      <x:c r="F17" s="87" t="str">
-        <x:v>1,980 Hz 이상 (명목 2 kSPS, ±1%)</x:v>
-      </x:c>
-      <x:c r="G17" s="82" t="str">
-        <x:v>텔레메트리는 100 ms이므로 ADC 원시율은 별도 계측 권장</x:v>
-      </x:c>
-      <x:c r="H17" s="82" t="str">
+      <x:c r="C17" s="275" t="str">
+        <x:v>PC CSV 또는 logic analyzer</x:v>
+      </x:c>
+      <x:c r="D17" s="275" t="str">
+        <x:v>정상 입력에서 1분 이상 캡처하고 sequence/device_ms로 실제 수집률을 계산합니다.</x:v>
+      </x:c>
+      <x:c r="E17" s="275" t="str">
+        <x:v>프레임 수·경과시간·dropped·CRC/SPI 오류</x:v>
+      </x:c>
+      <x:c r="F17" s="323" t="str">
+        <x:v>1,980 Hz 이상</x:v>
+      </x:c>
+      <x:c r="G17" s="275" t="str">
+        <x:v>텔레메트리는 100 ms이므로 ADC 윗값은 별도 계산</x:v>
+      </x:c>
+      <x:c r="H17" s="275" t="str">
         <x:v>측정값=실제 sample rate</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="72" customHeight="1">
-      <x:c r="A18" s="85" t="str">
+    <x:row r="18" ht="58" customHeight="1">
+      <x:c r="A18" s="279" t="str">
         <x:v>T-02</x:v>
       </x:c>
-      <x:c r="B18" s="82" t="str">
+      <x:c r="B18" s="275" t="str">
         <x:v>DMA/링버퍼</x:v>
       </x:c>
-      <x:c r="C18" s="82" t="str">
+      <x:c r="C18" s="275" t="str">
         <x:v>대시보드 CSV, 부하 조건</x:v>
       </x:c>
-      <x:c r="D18" s="82" t="str">
+      <x:c r="D18" s="275" t="str">
         <x:v>CPU·네트워크 부하를 단계적으로 올려 10분 이상 실행합니다.</x:v>
       </x:c>
-      <x:c r="E18" s="82" t="str">
+      <x:c r="E18" s="275" t="str">
         <x:v>dropped counter, sequence gap, CRC/SPI 오류</x:v>
       </x:c>
-      <x:c r="F18" s="87" t="str">
+      <x:c r="F18" s="323" t="str">
         <x:v>dropped=0</x:v>
       </x:c>
-      <x:c r="G18" s="82" t="str">
+      <x:c r="G18" s="275" t="str">
         <x:v>한 번에 하나의 부하만 변경</x:v>
       </x:c>
-      <x:c r="H18" s="82" t="str">
+      <x:c r="H18" s="275" t="str">
         <x:v>측정값=dropped frames</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="72" customHeight="1">
-      <x:c r="A19" s="85" t="str">
-        <x:v>T-03</x:v>
-      </x:c>
-      <x:c r="B19" s="82" t="str">
-        <x:v>DAC 응답</x:v>
-      </x:c>
-      <x:c r="C19" s="82" t="str">
-        <x:v>oscilloscope, 더미 부하</x:v>
-      </x:c>
-      <x:c r="D19" s="82" t="str">
-        <x:v>안전한 범위의 step 명령을 인가하고 입력 시점부터 출력 안정화까지 반복 측정합니다.</x:v>
-      </x:c>
-      <x:c r="E19" s="82" t="str">
-        <x:v>상승/하강 settling time, overshoot, CSV/파형 파일</x:v>
-      </x:c>
-      <x:c r="F19" s="87" t="str">
-        <x:v>30 ms 이하</x:v>
-      </x:c>
-      <x:c r="G19" s="82" t="str">
-        <x:v>실부하 전 더미 부하에서 확인</x:v>
-      </x:c>
-      <x:c r="H19" s="82" t="str">
-        <x:v>측정값=최악 settling time</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="72" customHeight="1">
-      <x:c r="A20" s="85" t="str">
+    <x:row r="19" ht="58" customHeight="1">
+      <x:c r="A19" s="279" t="str">
         <x:v>N-01</x:v>
       </x:c>
-      <x:c r="B20" s="82" t="str">
+      <x:c r="B19" s="275" t="str">
         <x:v>UDP 전송률</x:v>
       </x:c>
-      <x:c r="C20" s="82" t="str">
+      <x:c r="C19" s="275" t="str">
         <x:v>PC CSV 캡처</x:v>
       </x:c>
-      <x:c r="D20" s="82" t="str">
+      <x:c r="D19" s="275" t="str">
         <x:v>1분 이상 캡처한 뒤 received_at 인접 행 차이를 계산합니다.</x:v>
       </x:c>
-      <x:c r="E20" s="82" t="str">
+      <x:c r="E19" s="275" t="str">
         <x:v>평균 주기·최대 jitter·수신 frame 수</x:v>
       </x:c>
-      <x:c r="F20" s="87" t="str">
-        <x:v>평균 95–105 ms (명목 100 ms)</x:v>
-      </x:c>
-      <x:c r="G20" s="82" t="str">
-        <x:v>PC의 순간 부하는 비고에 기록</x:v>
-      </x:c>
-      <x:c r="H20" s="82" t="str">
+      <x:c r="F19" s="323" t="str">
+        <x:v>평균 95–105 ms</x:v>
+      </x:c>
+      <x:c r="G19" s="275" t="str">
+        <x:v>PC 순간 부하는 비고에 기록</x:v>
+      </x:c>
+      <x:c r="H19" s="275" t="str">
         <x:v>측정값=평균 송신 주기</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="72" customHeight="1">
-      <x:c r="A21" s="85" t="str">
+    <x:row r="20" ht="58" customHeight="1">
+      <x:c r="A20" s="279" t="str">
         <x:v>N-02</x:v>
       </x:c>
-      <x:c r="B21" s="82" t="str">
+      <x:c r="B20" s="275" t="str">
         <x:v>UDP 손실</x:v>
       </x:c>
-      <x:c r="C21" s="82" t="str">
+      <x:c r="C20" s="275" t="str">
         <x:v>PC CSV 캡처, 동일 LAN</x:v>
       </x:c>
-      <x:c r="D21" s="82" t="str">
+      <x:c r="D20" s="275" t="str">
         <x:v>10분 이상 캡처하고 sequence 누락과 모니터 종료 요약을 확인합니다.</x:v>
       </x:c>
-      <x:c r="E21" s="82" t="str">
+      <x:c r="E20" s="275" t="str">
         <x:v>estimated_udp_loss ÷ frames × 100, reset 구간</x:v>
       </x:c>
-      <x:c r="F21" s="87" t="str">
+      <x:c r="F20" s="323" t="str">
         <x:v>0.1 % 이하</x:v>
       </x:c>
-      <x:c r="G21" s="82" t="str">
+      <x:c r="G20" s="275" t="str">
         <x:v>Wi-Fi 대신 유선·동일 VLAN 권장</x:v>
       </x:c>
-      <x:c r="H21" s="82" t="str">
+      <x:c r="H20" s="275" t="str">
         <x:v>측정값=sequence gap rate</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="58" customHeight="1">
+      <x:c r="A21" s="279" t="str">
+        <x:v>L-01</x:v>
+      </x:c>
+      <x:c r="B21" s="275" t="str">
+        <x:v>양 채널 부하 안정성</x:v>
+      </x:c>
+      <x:c r="C21" s="275" t="str">
+        <x:v>PC CSV, Keysight E36233A</x:v>
+      </x:c>
+      <x:c r="D21" s="275" t="str">
+        <x:v>양 채널에 11 V / 5 A를 인가하고 25분 이상 연속 캡처합니다.</x:v>
+      </x:c>
+      <x:c r="E21" s="275" t="str">
+        <x:v>운전 시간·ADC rate·dropped·CRC/SPI/DAC·UDP loss</x:v>
+      </x:c>
+      <x:c r="F21" s="323" t="str">
+        <x:v>25 min 이상, 오류 0</x:v>
+      </x:c>
+      <x:c r="G21" s="275" t="str">
+        <x:v>다시간 soak·고의 fault 주입은 본 범위에서 제외</x:v>
+      </x:c>
+      <x:c r="H21" s="275" t="str">
+        <x:v>측정값=연속 운전 시간</x:v>
+      </x:c>
+    </x:row>
     <x:row r="22" ht="72" customHeight="1">
-      <x:c r="A22" s="85" t="str">
-        <x:v>R-01</x:v>
-      </x:c>
-      <x:c r="B22" s="82" t="str">
-        <x:v>ADC DRDY 정지</x:v>
-      </x:c>
-      <x:c r="C22" s="82" t="str">
-        <x:v>신호 차단 수단, 로그</x:v>
-      </x:c>
-      <x:c r="D22" s="82" t="str">
-        <x:v>DRDY 또는 ADC 프레임 흐름을 안전하게 중단하고 MUTED 전이와 안전 출력 상태를 확인합니다.</x:v>
-      </x:c>
-      <x:c r="E22" s="82" t="str">
-        <x:v>fault 발생→MUTED 시간, 플래그, 재복구 시간</x:v>
-      </x:c>
-      <x:c r="F22" s="87" t="str">
-        <x:v>500 ms 이하</x:v>
-      </x:c>
-      <x:c r="G22" s="82" t="str">
-        <x:v>실부하 비연결 상태에서 수행</x:v>
-      </x:c>
-      <x:c r="H22" s="82" t="str">
-        <x:v>측정값=MUTED 전이 시간</x:v>
-      </x:c>
+      <x:c r="A22" s="85"/>
+      <x:c r="B22" s="82"/>
+      <x:c r="C22" s="82"/>
+      <x:c r="D22" s="82"/>
+      <x:c r="E22" s="82"/>
+      <x:c r="F22" s="87"/>
+      <x:c r="G22" s="82"/>
+      <x:c r="H22" s="82"/>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">
-      <x:c r="A23" s="85" t="str">
-        <x:v>R-02</x:v>
-      </x:c>
-      <x:c r="B23" s="82" t="str">
-        <x:v>SPI 장애 복구</x:v>
-      </x:c>
-      <x:c r="C23" s="82" t="str">
-        <x:v>재현 가능한 fault injection</x:v>
-      </x:c>
-      <x:c r="D23" s="82" t="str">
-        <x:v>ADC/DAC 공유 SPI 동작 중 통신 오류를 유발하고 RECOVERING/WARMUP/ACTIVE 순서를 확인합니다.</x:v>
-      </x:c>
-      <x:c r="E23" s="82" t="str">
-        <x:v>SPI 오류·CRC·복구 시간·sequence reset·CSV</x:v>
-      </x:c>
-      <x:c r="F23" s="87" t="str">
-        <x:v>3 s 이하</x:v>
-      </x:c>
-      <x:c r="G23" s="82" t="str">
-        <x:v>DMA/CS 동작을 계측 가능하면 함께 확인</x:v>
-      </x:c>
-      <x:c r="H23" s="82" t="str">
-        <x:v>측정값=recovery 성공 시간</x:v>
-      </x:c>
+      <x:c r="A23" s="85"/>
+      <x:c r="B23" s="82"/>
+      <x:c r="C23" s="82"/>
+      <x:c r="D23" s="82"/>
+      <x:c r="E23" s="82"/>
+      <x:c r="F23" s="87"/>
+      <x:c r="G23" s="82"/>
+      <x:c r="H23" s="82"/>
     </x:row>
     <x:row r="24" ht="72" customHeight="1">
-      <x:c r="A24" s="85" t="str">
-        <x:v>R-03</x:v>
-      </x:c>
-      <x:c r="B24" s="82" t="str">
-        <x:v>DAC 통신 장애</x:v>
-      </x:c>
-      <x:c r="C24" s="82" t="str">
-        <x:v>DAC fault injection, oscilloscope</x:v>
-      </x:c>
-      <x:c r="D24" s="82" t="str">
-        <x:v>DAC 전송 오류를 2회 이상 유발하고 MUTED 전이 및 안전 출력 상태를 확인합니다.</x:v>
-      </x:c>
-      <x:c r="E24" s="82" t="str">
-        <x:v>DAC 오류·MUTED 시간·출력 파형·복구 결과</x:v>
-      </x:c>
-      <x:c r="F24" s="87" t="str">
-        <x:v>50 ms 이하</x:v>
-      </x:c>
-      <x:c r="G24" s="82" t="str">
-        <x:v>안전 출력 하드웨어 경로는 별도 확인</x:v>
-      </x:c>
-      <x:c r="H24" s="82" t="str">
-        <x:v>측정값=DAC fault 전이 시간</x:v>
-      </x:c>
+      <x:c r="A24" s="85"/>
+      <x:c r="B24" s="82"/>
+      <x:c r="C24" s="82"/>
+      <x:c r="D24" s="82"/>
+      <x:c r="E24" s="82"/>
+      <x:c r="F24" s="87"/>
+      <x:c r="G24" s="82"/>
+      <x:c r="H24" s="82"/>
     </x:row>
     <x:row r="25" ht="72" customHeight="1">
-      <x:c r="A25" s="85" t="str">
-        <x:v>R-04</x:v>
-      </x:c>
-      <x:c r="B25" s="82" t="str">
-        <x:v>LAN 미연결</x:v>
-      </x:c>
-      <x:c r="C25" s="82" t="str">
-        <x:v>Ethernet cable</x:v>
-      </x:c>
-      <x:c r="D25" s="82" t="str">
-        <x:v>정상 상태에서 LAN을 분리한 뒤 10분 관찰하고, 재연결 후 텔레메트리 복귀를 확인합니다.</x:v>
-      </x:c>
-      <x:c r="E25" s="82" t="str">
-        <x:v>재부팅 수, watchdog reset 징후, 재연결 시간</x:v>
-      </x:c>
-      <x:c r="F25" s="87" t="str">
-        <x:v>재부팅 0회</x:v>
-      </x:c>
-      <x:c r="G25" s="82" t="str">
-        <x:v>LAN 장애와 계측 task 장애를 구분</x:v>
-      </x:c>
-      <x:c r="H25" s="82" t="str">
-        <x:v>측정값=watchdog 재부팅 반복</x:v>
-      </x:c>
+      <x:c r="A25" s="85"/>
+      <x:c r="B25" s="82"/>
+      <x:c r="C25" s="82"/>
+      <x:c r="D25" s="82"/>
+      <x:c r="E25" s="82"/>
+      <x:c r="F25" s="87"/>
+      <x:c r="G25" s="82"/>
+      <x:c r="H25" s="82"/>
     </x:row>
     <x:row r="26" ht="72" customHeight="1">
-      <x:c r="A26" s="85" t="str">
-        <x:v>L-01</x:v>
-      </x:c>
-      <x:c r="B26" s="82" t="str">
-        <x:v>Soak test</x:v>
-      </x:c>
-      <x:c r="C26" s="82" t="str">
-        <x:v>전용 PC, CSV, 안정 전원</x:v>
-      </x:c>
-      <x:c r="D26" s="82" t="str">
-        <x:v>대표 부하·입력에서 최소 24시간 연속 캡처합니다. 중간에 파일·시스템 시간·전원 조건을 점검합니다.</x:v>
-      </x:c>
-      <x:c r="E26" s="82" t="str">
-        <x:v>frames·유실·reset·CRC/SPI/DAC 오류·온도·전압</x:v>
-      </x:c>
-      <x:c r="F26" s="87" t="str">
-        <x:v>24 h 이상</x:v>
-      </x:c>
-      <x:c r="G26" s="82" t="str">
-        <x:v>대용량 CSV 저장공간과 PC 절전 해제 확인</x:v>
-      </x:c>
-      <x:c r="H26" s="82" t="str">
-        <x:v>측정값=연속 동작 시간</x:v>
-      </x:c>
+      <x:c r="A26" s="85"/>
+      <x:c r="B26" s="82"/>
+      <x:c r="C26" s="82"/>
+      <x:c r="D26" s="82"/>
+      <x:c r="E26" s="82"/>
+      <x:c r="F26" s="87"/>
+      <x:c r="G26" s="82"/>
+      <x:c r="H26" s="82"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3971,92 +4808,92 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="200" t="str">
+      <x:c r="A1" s="216" t="str">
         <x:v>CSV 캡처 이력 및 분석 결과</x:v>
       </x:c>
-      <x:c r="B1" s="200"/>
-      <x:c r="C1" s="200"/>
-      <x:c r="D1" s="200"/>
-      <x:c r="E1" s="200"/>
-      <x:c r="F1" s="200"/>
-      <x:c r="G1" s="200"/>
-      <x:c r="H1" s="200"/>
-      <x:c r="I1" s="200"/>
-      <x:c r="J1" s="200"/>
-      <x:c r="K1" s="200"/>
-      <x:c r="L1" s="200"/>
-      <x:c r="M1" s="200"/>
-      <x:c r="N1" s="200"/>
-      <x:c r="O1" s="200"/>
-      <x:c r="P1" s="200"/>
+      <x:c r="B1" s="216"/>
+      <x:c r="C1" s="216"/>
+      <x:c r="D1" s="216"/>
+      <x:c r="E1" s="216"/>
+      <x:c r="F1" s="216"/>
+      <x:c r="G1" s="216"/>
+      <x:c r="H1" s="216"/>
+      <x:c r="I1" s="216"/>
+      <x:c r="J1" s="216"/>
+      <x:c r="K1" s="216"/>
+      <x:c r="L1" s="216"/>
+      <x:c r="M1" s="216"/>
+      <x:c r="N1" s="216"/>
+      <x:c r="O1" s="216"/>
+      <x:c r="P1" s="216"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="201" t="str">
+      <x:c r="A3" s="217" t="str">
         <x:v>모든 원본 CSV는 logs/에 보관합니다. PASS는 해당 캡처의 범위에서만 유효하며, 장시간·교정 시험은 별도 시험으로 확정합니다.</x:v>
       </x:c>
-      <x:c r="B3" s="201"/>
-      <x:c r="C3" s="201"/>
-      <x:c r="D3" s="201"/>
-      <x:c r="E3" s="201"/>
-      <x:c r="F3" s="201"/>
-      <x:c r="G3" s="201"/>
-      <x:c r="H3" s="201"/>
-      <x:c r="I3" s="201"/>
-      <x:c r="J3" s="201"/>
-      <x:c r="K3" s="201"/>
-      <x:c r="L3" s="201"/>
-      <x:c r="M3" s="201"/>
-      <x:c r="N3" s="201"/>
-      <x:c r="O3" s="201"/>
-      <x:c r="P3" s="201"/>
+      <x:c r="B3" s="217"/>
+      <x:c r="C3" s="217"/>
+      <x:c r="D3" s="217"/>
+      <x:c r="E3" s="217"/>
+      <x:c r="F3" s="217"/>
+      <x:c r="G3" s="217"/>
+      <x:c r="H3" s="217"/>
+      <x:c r="I3" s="217"/>
+      <x:c r="J3" s="217"/>
+      <x:c r="K3" s="217"/>
+      <x:c r="L3" s="217"/>
+      <x:c r="M3" s="217"/>
+      <x:c r="N3" s="217"/>
+      <x:c r="O3" s="217"/>
+      <x:c r="P3" s="217"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="202" t="str">
+      <x:c r="A5" s="218" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B5" s="202" t="str">
+      <x:c r="B5" s="218" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C5" s="202" t="str">
+      <x:c r="C5" s="218" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D5" s="202" t="str">
+      <x:c r="D5" s="218" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E5" s="202" t="str">
+      <x:c r="E5" s="218" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F5" s="202" t="str">
+      <x:c r="F5" s="218" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G5" s="202" t="str">
+      <x:c r="G5" s="218" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H5" s="202" t="str">
+      <x:c r="H5" s="218" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I5" s="202" t="str">
+      <x:c r="I5" s="218" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J5" s="202" t="str">
+      <x:c r="J5" s="218" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K5" s="202" t="str">
+      <x:c r="K5" s="218" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L5" s="202" t="str">
+      <x:c r="L5" s="218" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M5" s="202" t="str">
+      <x:c r="M5" s="218" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N5" s="202" t="str">
+      <x:c r="N5" s="218" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O5" s="202" t="str">
+      <x:c r="O5" s="218" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P5" s="202" t="str">
+      <x:c r="P5" s="218" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4103,7 +4940,7 @@
       <x:c r="N6" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O6" s="203" t="str">
+      <x:c r="O6" s="219" t="str">
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="P6" s="100" t="str">
@@ -4153,7 +4990,7 @@
       <x:c r="N7" s="100" t="str">
         <x:v>CH1, 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O7" s="204" t="str">
+      <x:c r="O7" s="220" t="str">
         <x:v>PASS (입력 응답)</x:v>
       </x:c>
       <x:c r="P7" s="100" t="str">
@@ -4199,7 +5036,7 @@
       <x:c r="N8" s="100" t="str">
         <x:v>Reset 반복</x:v>
       </x:c>
-      <x:c r="O8" s="205" t="str">
+      <x:c r="O8" s="221" t="str">
         <x:v>MIXED</x:v>
       </x:c>
       <x:c r="P8" s="100" t="str">
@@ -4249,7 +5086,7 @@
       <x:c r="N9" s="100" t="str">
         <x:v>11 V input; ST-LINK MCO; 2 kSPS / SPI 5.33 MHz / ring 256</x:v>
       </x:c>
-      <x:c r="O9" s="204" t="str">
+      <x:c r="O9" s="220" t="str">
         <x:v>PASS (예비)</x:v>
       </x:c>
       <x:c r="P9" s="100" t="str">
@@ -4299,7 +5136,7 @@
       <x:c r="N10" s="100" t="str">
         <x:v>0 V / 0 A; final 5 min = 3,001 frames</x:v>
       </x:c>
-      <x:c r="O10" s="204" t="str">
+      <x:c r="O10" s="220" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="P10" s="100" t="str">
@@ -4307,36 +5144,36 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="206" t="str">
+      <x:c r="A11" s="222" t="str">
         <x:v>현재 검증된 펌웨어 프로파일</x:v>
       </x:c>
-      <x:c r="B11" s="206"/>
-      <x:c r="C11" s="206"/>
-      <x:c r="D11" s="206"/>
-      <x:c r="E11" s="206"/>
-      <x:c r="F11" s="206"/>
-      <x:c r="G11" s="206"/>
-      <x:c r="H11" s="206"/>
-      <x:c r="I11" s="206"/>
-      <x:c r="J11" s="206"/>
-      <x:c r="K11" s="206"/>
-      <x:c r="L11" s="206"/>
-      <x:c r="M11" s="206"/>
-      <x:c r="N11" s="206"/>
-      <x:c r="O11" s="206"/>
-      <x:c r="P11" s="206"/>
+      <x:c r="B11" s="222"/>
+      <x:c r="C11" s="222"/>
+      <x:c r="D11" s="222"/>
+      <x:c r="E11" s="222"/>
+      <x:c r="F11" s="222"/>
+      <x:c r="G11" s="222"/>
+      <x:c r="H11" s="222"/>
+      <x:c r="I11" s="222"/>
+      <x:c r="J11" s="222"/>
+      <x:c r="K11" s="222"/>
+      <x:c r="L11" s="222"/>
+      <x:c r="M11" s="222"/>
+      <x:c r="N11" s="222"/>
+      <x:c r="O11" s="222"/>
+      <x:c r="P11" s="222"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="207" t="str">
+      <x:c r="A12" s="223" t="str">
         <x:v>설정</x:v>
       </x:c>
-      <x:c r="B12" s="207" t="str">
+      <x:c r="B12" s="223" t="str">
         <x:v>현재값</x:v>
       </x:c>
-      <x:c r="C12" s="207" t="str">
+      <x:c r="C12" s="223" t="str">
         <x:v>근거</x:v>
       </x:c>
-      <x:c r="D12" s="207" t="str">
+      <x:c r="D12" s="223" t="str">
         <x:v>상태</x:v>
       </x:c>
     </x:row>
@@ -4350,7 +5187,7 @@
       <x:c r="C13" s="110" t="str">
         <x:v>최종 CSV: 1,999.882 Hz</x:v>
       </x:c>
-      <x:c r="D13" s="208" t="str">
+      <x:c r="D13" s="224" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4364,7 +5201,7 @@
       <x:c r="C14" s="110" t="str">
         <x:v>ADC DMA 전송 여유 확보</x:v>
       </x:c>
-      <x:c r="D14" s="208" t="str">
+      <x:c r="D14" s="224" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
@@ -4378,47 +5215,47 @@
       <x:c r="C15" s="110" t="str">
         <x:v>PC/보드 시간 1:1</x:v>
       </x:c>
-      <x:c r="D15" s="208" t="str">
+      <x:c r="D15" s="224" t="str">
         <x:v>검증됨</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="206" t="str">
+      <x:c r="A17" s="222" t="str">
         <x:v>적용한 영점 보정값 (2026-08-20, 마지막 5분 평균)</x:v>
       </x:c>
-      <x:c r="B17" s="206"/>
-      <x:c r="C17" s="206"/>
-      <x:c r="D17" s="206"/>
-      <x:c r="E17" s="206"/>
-      <x:c r="F17" s="206"/>
-      <x:c r="G17" s="206"/>
-      <x:c r="H17" s="206"/>
-      <x:c r="I17" s="206"/>
-      <x:c r="J17" s="206"/>
-      <x:c r="K17" s="206"/>
-      <x:c r="L17" s="206"/>
-      <x:c r="M17" s="206"/>
-      <x:c r="N17" s="206"/>
-      <x:c r="O17" s="206"/>
-      <x:c r="P17" s="206"/>
+      <x:c r="B17" s="222"/>
+      <x:c r="C17" s="222"/>
+      <x:c r="D17" s="222"/>
+      <x:c r="E17" s="222"/>
+      <x:c r="F17" s="222"/>
+      <x:c r="G17" s="222"/>
+      <x:c r="H17" s="222"/>
+      <x:c r="I17" s="222"/>
+      <x:c r="J17" s="222"/>
+      <x:c r="K17" s="222"/>
+      <x:c r="L17" s="222"/>
+      <x:c r="M17" s="222"/>
+      <x:c r="N17" s="222"/>
+      <x:c r="O17" s="222"/>
+      <x:c r="P17" s="222"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="207" t="str">
+      <x:c r="A18" s="223" t="str">
         <x:v>채널</x:v>
       </x:c>
-      <x:c r="B18" s="207" t="str">
+      <x:c r="B18" s="223" t="str">
         <x:v>측정 평균</x:v>
       </x:c>
-      <x:c r="C18" s="207" t="str">
+      <x:c r="C18" s="223" t="str">
         <x:v>단위</x:v>
       </x:c>
-      <x:c r="D18" s="207" t="str">
+      <x:c r="D18" s="223" t="str">
         <x:v>펌웨어 매크로</x:v>
       </x:c>
-      <x:c r="E18" s="207" t="str">
+      <x:c r="E18" s="223" t="str">
         <x:v>적용 OFFSET_UNITS</x:v>
       </x:c>
-      <x:c r="F18" s="207" t="str">
+      <x:c r="F18" s="223" t="str">
         <x:v>CSV</x:v>
       </x:c>
     </x:row>
@@ -4503,72 +5340,72 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="206" t="str">
+      <x:c r="A24" s="222" t="str">
         <x:v>추가 캡처: 양 채널 11 V / 5 A 장시간 부하 시험</x:v>
       </x:c>
-      <x:c r="B24" s="206"/>
-      <x:c r="C24" s="206"/>
-      <x:c r="D24" s="206"/>
-      <x:c r="E24" s="206"/>
-      <x:c r="F24" s="206"/>
-      <x:c r="G24" s="206"/>
-      <x:c r="H24" s="206"/>
-      <x:c r="I24" s="206"/>
-      <x:c r="J24" s="206"/>
-      <x:c r="K24" s="206"/>
-      <x:c r="L24" s="206"/>
-      <x:c r="M24" s="206"/>
-      <x:c r="N24" s="206"/>
-      <x:c r="O24" s="206"/>
-      <x:c r="P24" s="206"/>
+      <x:c r="B24" s="222"/>
+      <x:c r="C24" s="222"/>
+      <x:c r="D24" s="222"/>
+      <x:c r="E24" s="222"/>
+      <x:c r="F24" s="222"/>
+      <x:c r="G24" s="222"/>
+      <x:c r="H24" s="222"/>
+      <x:c r="I24" s="222"/>
+      <x:c r="J24" s="222"/>
+      <x:c r="K24" s="222"/>
+      <x:c r="L24" s="222"/>
+      <x:c r="M24" s="222"/>
+      <x:c r="N24" s="222"/>
+      <x:c r="O24" s="222"/>
+      <x:c r="P24" s="222"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="202" t="str">
+      <x:c r="A25" s="218" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B25" s="202" t="str">
+      <x:c r="B25" s="218" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C25" s="202" t="str">
+      <x:c r="C25" s="218" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D25" s="202" t="str">
+      <x:c r="D25" s="218" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E25" s="202" t="str">
+      <x:c r="E25" s="218" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F25" s="202" t="str">
+      <x:c r="F25" s="218" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G25" s="202" t="str">
+      <x:c r="G25" s="218" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H25" s="202" t="str">
+      <x:c r="H25" s="218" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I25" s="202" t="str">
+      <x:c r="I25" s="218" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J25" s="202" t="str">
+      <x:c r="J25" s="218" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K25" s="202" t="str">
+      <x:c r="K25" s="218" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L25" s="202" t="str">
+      <x:c r="L25" s="218" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M25" s="202" t="str">
+      <x:c r="M25" s="218" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N25" s="202" t="str">
+      <x:c r="N25" s="218" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O25" s="202" t="str">
+      <x:c r="O25" s="218" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P25" s="202" t="str">
+      <x:c r="P25" s="218" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4615,7 +5452,7 @@
       <x:c r="N26" s="100" t="str">
         <x:v>CH1+CH2 11 V / 5 A</x:v>
       </x:c>
-      <x:c r="O26" s="204" t="str">
+      <x:c r="O26" s="220" t="str">
         <x:v>PASS (안정성)</x:v>
       </x:c>
       <x:c r="P26" s="100" t="str">
@@ -4623,72 +5460,72 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="206" t="str">
+      <x:c r="A28" s="222" t="str">
         <x:v>추가 캡처: 3점 상대 선형성 시험</x:v>
       </x:c>
-      <x:c r="B28" s="206"/>
-      <x:c r="C28" s="206"/>
-      <x:c r="D28" s="206"/>
-      <x:c r="E28" s="206"/>
-      <x:c r="F28" s="206"/>
-      <x:c r="G28" s="206"/>
-      <x:c r="H28" s="206"/>
-      <x:c r="I28" s="206"/>
-      <x:c r="J28" s="206"/>
-      <x:c r="K28" s="206"/>
-      <x:c r="L28" s="206"/>
-      <x:c r="M28" s="206"/>
-      <x:c r="N28" s="206"/>
-      <x:c r="O28" s="206"/>
-      <x:c r="P28" s="206"/>
+      <x:c r="B28" s="222"/>
+      <x:c r="C28" s="222"/>
+      <x:c r="D28" s="222"/>
+      <x:c r="E28" s="222"/>
+      <x:c r="F28" s="222"/>
+      <x:c r="G28" s="222"/>
+      <x:c r="H28" s="222"/>
+      <x:c r="I28" s="222"/>
+      <x:c r="J28" s="222"/>
+      <x:c r="K28" s="222"/>
+      <x:c r="L28" s="222"/>
+      <x:c r="M28" s="222"/>
+      <x:c r="N28" s="222"/>
+      <x:c r="O28" s="222"/>
+      <x:c r="P28" s="222"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="202" t="str">
+      <x:c r="A29" s="218" t="str">
         <x:v>CSV 파일</x:v>
       </x:c>
-      <x:c r="B29" s="202" t="str">
+      <x:c r="B29" s="218" t="str">
         <x:v>시험 목적</x:v>
       </x:c>
-      <x:c r="C29" s="202" t="str">
+      <x:c r="C29" s="218" t="str">
         <x:v>FW commit</x:v>
       </x:c>
-      <x:c r="D29" s="202" t="str">
+      <x:c r="D29" s="218" t="str">
         <x:v>부팅 구간</x:v>
       </x:c>
-      <x:c r="E29" s="202" t="str">
+      <x:c r="E29" s="218" t="str">
         <x:v>프레임</x:v>
       </x:c>
-      <x:c r="F29" s="202" t="str">
+      <x:c r="F29" s="218" t="str">
         <x:v>PC 시간 (s)</x:v>
       </x:c>
-      <x:c r="G29" s="202" t="str">
+      <x:c r="G29" s="218" t="str">
         <x:v>보드 시간 (s)</x:v>
       </x:c>
-      <x:c r="H29" s="202" t="str">
+      <x:c r="H29" s="218" t="str">
         <x:v>시간비</x:v>
       </x:c>
-      <x:c r="I29" s="202" t="str">
+      <x:c r="I29" s="218" t="str">
         <x:v>ADC rate (Hz)</x:v>
       </x:c>
-      <x:c r="J29" s="202" t="str">
+      <x:c r="J29" s="218" t="str">
         <x:v>UDP 평균 (ms)</x:v>
       </x:c>
-      <x:c r="K29" s="202" t="str">
+      <x:c r="K29" s="218" t="str">
         <x:v>UDP 범위 (ms)</x:v>
       </x:c>
-      <x:c r="L29" s="202" t="str">
+      <x:c r="L29" s="218" t="str">
         <x:v>드랍 최대</x:v>
       </x:c>
-      <x:c r="M29" s="202" t="str">
+      <x:c r="M29" s="218" t="str">
         <x:v>오류</x:v>
       </x:c>
-      <x:c r="N29" s="202" t="str">
+      <x:c r="N29" s="218" t="str">
         <x:v>입력/조건</x:v>
       </x:c>
-      <x:c r="O29" s="202" t="str">
+      <x:c r="O29" s="218" t="str">
         <x:v>판정</x:v>
       </x:c>
-      <x:c r="P29" s="202" t="str">
+      <x:c r="P29" s="218" t="str">
         <x:v>분석 메모</x:v>
       </x:c>
     </x:row>
@@ -4735,7 +5572,7 @@
       <x:c r="N30" s="100" t="str">
         <x:v>0 V / 약 5 V / 약 10 V</x:v>
       </x:c>
-      <x:c r="O30" s="204" t="str">
+      <x:c r="O30" s="220" t="str">
         <x:v>PASS (상대 선형성)</x:v>
       </x:c>
       <x:c r="P30" s="100" t="str">
@@ -4743,116 +5580,152 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="206" t="str">
+      <x:c r="A32" s="222" t="str">
         <x:v>열화상 참고 관찰: 양 채널 11 V / 5 A 부하 시험 말기</x:v>
       </x:c>
-      <x:c r="B32" s="206"/>
-      <x:c r="C32" s="206"/>
-      <x:c r="D32" s="206"/>
-      <x:c r="E32" s="206"/>
-      <x:c r="F32" s="206"/>
-      <x:c r="G32" s="206"/>
-      <x:c r="H32" s="206"/>
-      <x:c r="I32" s="206"/>
-      <x:c r="J32" s="206"/>
-      <x:c r="K32" s="206"/>
-      <x:c r="L32" s="206"/>
-      <x:c r="M32" s="206"/>
-      <x:c r="N32" s="206"/>
-      <x:c r="O32" s="206"/>
-      <x:c r="P32" s="206"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="213" t="str">
+      <x:c r="B32" s="222"/>
+      <x:c r="C32" s="222"/>
+      <x:c r="D32" s="222"/>
+      <x:c r="E32" s="222"/>
+      <x:c r="F32" s="222"/>
+      <x:c r="G32" s="222"/>
+      <x:c r="H32" s="222"/>
+      <x:c r="I32" s="222"/>
+      <x:c r="J32" s="222"/>
+      <x:c r="K32" s="222"/>
+      <x:c r="L32" s="222"/>
+      <x:c r="M32" s="222"/>
+      <x:c r="N32" s="222"/>
+      <x:c r="O32" s="222"/>
+      <x:c r="P32" s="222"/>
+    </x:row>
+    <x:row r="33" ht="32" customHeight="1">
+      <x:c r="A33" s="258" t="str">
         <x:v>증빙 이미지</x:v>
       </x:c>
-      <x:c r="B33" s="213" t="str">
+      <x:c r="B33" s="258" t="str">
         <x:v>시험 조건</x:v>
       </x:c>
-      <x:c r="C33" s="213" t="str">
+      <x:c r="C33" s="258" t="str">
         <x:v>표시 최대 (°C)</x:v>
       </x:c>
-      <x:c r="D33" s="213" t="str">
+      <x:c r="D33" s="258" t="str">
         <x:v>중앙 측정점 (°C)</x:v>
       </x:c>
-      <x:c r="E33" s="213" t="str">
+      <x:c r="E33" s="258" t="str">
         <x:v>표시 하한/주변 (°C)</x:v>
       </x:c>
-      <x:c r="F33" s="213" t="str">
+      <x:c r="F33" s="258" t="str">
         <x:v>카메라 설정</x:v>
       </x:c>
-      <x:c r="G33" s="213" t="str">
-        <x:v>판정/메모</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="48" customHeight="1">
-      <x:c r="A34" s="100" t="str">
+      <x:c r="G33" s="258" t="str">
+        <x:v>판정 / 해석</x:v>
+      </x:c>
+      <x:c r="H33" s="258"/>
+      <x:c r="I33" s="258"/>
+      <x:c r="J33" s="258"/>
+      <x:c r="K33" s="258"/>
+      <x:c r="L33" s="258"/>
+      <x:c r="M33" s="258"/>
+      <x:c r="N33" s="258"/>
+      <x:c r="O33" s="258"/>
+      <x:c r="P33" s="258"/>
+    </x:row>
+    <x:row r="34" ht="46" customHeight="1">
+      <x:c r="A34" s="278" t="str">
         <x:v>발열1.jpg</x:v>
       </x:c>
-      <x:c r="B34" s="100" t="str">
+      <x:c r="B34" s="275" t="str">
         <x:v>CH1+CH2 11 V / 5 A, 시험 말기</x:v>
       </x:c>
-      <x:c r="C34" s="215" t="n">
+      <x:c r="C34" s="337" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="D34" s="215" t="n">
+      <x:c r="D34" s="337" t="n">
         <x:v>33.5</x:v>
       </x:c>
-      <x:c r="E34" s="215" t="n">
+      <x:c r="E34" s="337" t="n">
         <x:v>26.9</x:v>
       </x:c>
-      <x:c r="F34" s="100" t="str">
+      <x:c r="F34" s="275" t="str">
         <x:v>Emissivity 0.95</x:v>
       </x:c>
-      <x:c r="G34" s="100" t="str">
+      <x:c r="G34" s="275" t="str">
         <x:v>국부 최고점 41.0°C 관찰; 부품 위치 미확정</x:v>
       </x:c>
-    </x:row>
-    <x:row r="35" ht="48" customHeight="1">
-      <x:c r="A35" s="100" t="str">
+      <x:c r="H34" s="275"/>
+      <x:c r="I34" s="275"/>
+      <x:c r="J34" s="275"/>
+      <x:c r="K34" s="275"/>
+      <x:c r="L34" s="275"/>
+      <x:c r="M34" s="275"/>
+      <x:c r="N34" s="275"/>
+      <x:c r="O34" s="275"/>
+      <x:c r="P34" s="275"/>
+    </x:row>
+    <x:row r="35" ht="46" customHeight="1">
+      <x:c r="A35" s="278" t="str">
         <x:v>발열2.jpg</x:v>
       </x:c>
-      <x:c r="B35" s="100" t="str">
+      <x:c r="B35" s="275" t="str">
         <x:v>CH1+CH2 11 V / 5 A, 시험 말기</x:v>
       </x:c>
-      <x:c r="C35" s="215" t="n">
+      <x:c r="C35" s="337" t="n">
         <x:v>42.9</x:v>
       </x:c>
-      <x:c r="D35" s="215" t="n">
+      <x:c r="D35" s="337" t="n">
         <x:v>37.6</x:v>
       </x:c>
-      <x:c r="E35" s="215" t="n">
+      <x:c r="E35" s="337" t="n">
         <x:v>28.6</x:v>
       </x:c>
-      <x:c r="F35" s="100" t="str">
+      <x:c r="F35" s="275" t="str">
         <x:v>Emissivity 0.95</x:v>
       </x:c>
-      <x:c r="G35" s="100" t="str">
+      <x:c r="G35" s="275" t="str">
         <x:v>국부 최고점 42.9°C 관찰; 과열 징후 없음</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36" ht="48" customHeight="1">
-      <x:c r="A36" s="100" t="str">
+      <x:c r="H35" s="275"/>
+      <x:c r="I35" s="275"/>
+      <x:c r="J35" s="275"/>
+      <x:c r="K35" s="275"/>
+      <x:c r="L35" s="275"/>
+      <x:c r="M35" s="275"/>
+      <x:c r="N35" s="275"/>
+      <x:c r="O35" s="275"/>
+      <x:c r="P35" s="275"/>
+    </x:row>
+    <x:row r="36" ht="46" customHeight="1">
+      <x:c r="A36" s="278" t="str">
         <x:v>발열3.jpg</x:v>
       </x:c>
-      <x:c r="B36" s="100" t="str">
+      <x:c r="B36" s="275" t="str">
         <x:v>CH1+CH2 11 V / 5 A, 시험 말기</x:v>
       </x:c>
-      <x:c r="C36" s="215" t="n">
+      <x:c r="C36" s="337" t="n">
         <x:v>42.9</x:v>
       </x:c>
-      <x:c r="D36" s="215" t="n">
+      <x:c r="D36" s="337" t="n">
         <x:v>34.2</x:v>
       </x:c>
-      <x:c r="E36" s="215" t="n">
+      <x:c r="E36" s="337" t="n">
         <x:v>27.6</x:v>
       </x:c>
-      <x:c r="F36" s="100" t="str">
+      <x:c r="F36" s="275" t="str">
         <x:v>Emissivity 0.95</x:v>
       </x:c>
-      <x:c r="G36" s="100" t="str">
+      <x:c r="G36" s="275" t="str">
         <x:v>국부 최고점 42.9°C 관찰; 정격 판정용이 아닌 참고 자료</x:v>
       </x:c>
+      <x:c r="H36" s="275"/>
+      <x:c r="I36" s="275"/>
+      <x:c r="J36" s="275"/>
+      <x:c r="K36" s="275"/>
+      <x:c r="L36" s="275"/>
+      <x:c r="M36" s="275"/>
+      <x:c r="N36" s="275"/>
+      <x:c r="O36" s="275"/>
+      <x:c r="P36" s="275"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4863,6 +5736,10 @@
     <x:mergeCell ref="A24:P24"/>
     <x:mergeCell ref="A28:P28"/>
     <x:mergeCell ref="A32:P32"/>
+    <x:mergeCell ref="G33:P33"/>
+    <x:mergeCell ref="G34:P34"/>
+    <x:mergeCell ref="G35:P35"/>
+    <x:mergeCell ref="G36:P36"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>